<commit_message>
feat: implement dashboard population logic
Add automatic population of the Dashboard sheet with project metadata and carry-forward balances. Update financial report test cases to reflect these values.
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_befuellt.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_befuellt.xlsx
@@ -5057,14 +5057,18 @@
       <c r="B5" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>158</v>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>PRJ-2025-042</t>
+        </is>
       </c>
       <c r="D5" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="E5" s="6" t="s">
-        <v>160</v>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
       </c>
       <c r="AA5" s="3" t="s">
         <v>6</v>
@@ -5074,8 +5078,10 @@
       <c r="B6" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="C6" s="5" t="s">
-        <v>158</v>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Aufbau Gemeindezentrum Beispielstadt</t>
+        </is>
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
@@ -5087,14 +5093,18 @@
       <c r="B7" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="C7" s="5" t="s">
-        <v>158</v>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Beispiel Hilfswerk e.V.</t>
+        </is>
       </c>
       <c r="D7" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="E7" s="5" t="s">
-        <v>158</v>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
       </c>
       <c r="AA7" s="3" t="s">
         <v>8</v>
@@ -5104,8 +5114,10 @@
       <c r="B8" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="C8" s="5" t="s">
-        <v>158</v>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>01.01.2025 - 31.12.2027</t>
+        </is>
       </c>
       <c r="D8" s="4" t="s">
         <v>165</v>
@@ -5121,14 +5133,18 @@
       <c r="B9" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="C9" s="9" t="s">
-        <v>158</v>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>PRJ-2022-017</t>
+        </is>
       </c>
       <c r="D9" s="8" t="s">
         <v>167</v>
       </c>
-      <c r="E9" s="9" t="s">
-        <v>158</v>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
       </c>
       <c r="AA9" s="3" t="s">
         <v>10</v>
@@ -5138,14 +5154,14 @@
       <c r="B10" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="C10" s="10" t="s">
-        <v>158</v>
+      <c r="C10" s="10">
+        <v>45657</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="E10" s="11" t="s">
-        <v>158</v>
+      <c r="E10" s="11">
+        <v>125</v>
       </c>
       <c r="AA10" s="3" t="s">
         <v>11</v>
@@ -5155,14 +5171,14 @@
       <c r="B11" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="C11" s="12" t="s">
-        <v>158</v>
+      <c r="C11" s="12">
+        <v>200000</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="E11" s="13" t="s">
-        <v>158</v>
+      <c r="E11" s="13">
+        <v>1600</v>
       </c>
       <c r="AA11" s="3" t="s">
         <v>12</v>
@@ -5172,14 +5188,14 @@
       <c r="B12" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="C12" s="10" t="s">
-        <v>158</v>
+      <c r="C12" s="10">
+        <v>45658</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="E12" s="11" t="s">
-        <v>158</v>
+      <c r="E12" s="11">
+        <v>125</v>
       </c>
       <c r="AA12" s="3" t="s">
         <v>13</v>
@@ -5189,14 +5205,14 @@
       <c r="B13" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="C13" s="12" t="s">
-        <v>158</v>
+      <c r="C13" s="12">
+        <v>200000</v>
       </c>
       <c r="D13" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="E13" s="13" t="s">
-        <v>158</v>
+      <c r="E13" s="13">
+        <v>1600</v>
       </c>
       <c r="AA13" s="3" t="s">
         <v>14</v>
@@ -5212,8 +5228,10 @@
         <v>175</v>
       </c>
       <c r="C15" s="14"/>
-      <c r="D15" s="15" t="s">
-        <v>176</v>
+      <c r="D15" s="15" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
       </c>
       <c r="E15" s="16" t="s">
         <v>177</v>
@@ -5225,8 +5243,10 @@
     <row r="16" ht="22" customHeight="true">
       <c r="B16" s="14"/>
       <c r="C16" s="14"/>
-      <c r="D16" s="15" t="s">
-        <v>176</v>
+      <c r="D16" s="15" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
       </c>
       <c r="E16" s="16" t="s">
         <v>178</v>
@@ -5238,8 +5258,10 @@
     <row r="17" ht="22" customHeight="true">
       <c r="B17" s="14"/>
       <c r="C17" s="14"/>
-      <c r="D17" s="15" t="s">
-        <v>176</v>
+      <c r="D17" s="15" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
       </c>
       <c r="E17" s="16" t="s">
         <v>179</v>
@@ -5251,8 +5273,10 @@
     <row r="18" ht="22" customHeight="true">
       <c r="B18" s="14"/>
       <c r="C18" s="14"/>
-      <c r="D18" s="15" t="s">
-        <v>176</v>
+      <c r="D18" s="15" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
       </c>
       <c r="E18" s="16" t="s">
         <v>180</v>
@@ -5264,8 +5288,10 @@
     <row r="19" ht="22" customHeight="true">
       <c r="B19" s="14"/>
       <c r="C19" s="14"/>
-      <c r="D19" s="15" t="s">
-        <v>176</v>
+      <c r="D19" s="15" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
       </c>
       <c r="E19" s="16" t="s">
         <v>181</v>
@@ -5277,8 +5303,10 @@
     <row r="20" ht="22" customHeight="true">
       <c r="B20" s="14"/>
       <c r="C20" s="14"/>
-      <c r="D20" s="15" t="s">
-        <v>176</v>
+      <c r="D20" s="15" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
       </c>
       <c r="E20" s="16" t="s">
         <v>182</v>
@@ -5290,8 +5318,10 @@
     <row r="21" ht="22" customHeight="true">
       <c r="B21" s="14"/>
       <c r="C21" s="14"/>
-      <c r="D21" s="15" t="s">
-        <v>176</v>
+      <c r="D21" s="15" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
       </c>
       <c r="E21" s="16" t="s">
         <v>183</v>
@@ -13525,7 +13555,7 @@
         <v>311</v>
       </c>
       <c r="C34" s="129">
-        <v>125000</v>
+        <v>325000</v>
       </c>
       <c r="D34" s="130" t="str">
         <f>=IF(C34=0, 0, IF(ROUND(SUM(C35:C36), 2)=0, ROUND(D31 - 0, 2), ROUND(C34 / ROUND(SUM(C34:C36), 2) * D31, 2)))</f>
@@ -13535,7 +13565,7 @@
         <v>311</v>
       </c>
       <c r="J34" s="129">
-        <v>175000</v>
+        <v>375000</v>
       </c>
       <c r="K34" s="130" t="str">
         <f>=IF(J34=0, 0, IF(ROUND(SUM(J35:J36), 2)=0, ROUND(K31 - 0, 2), ROUND(J34 / ROUND(SUM(J34:J36), 2) * K31, 2)))</f>

</xml_diff>

<commit_message>
fix: remove hardcoded donor names from table rows
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_befuellt.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_befuellt.xlsx
@@ -150,7 +150,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="404" uniqueCount="404">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="402">
   <si>
     <t xml:space="preserve">  DASHBOARD (v1.0)</t>
   </si>
@@ -1112,16 +1112,10 @@
     <t>Saldo des Vorprojekts</t>
   </si>
   <si>
-    <t>KMW</t>
-  </si>
-  <si>
     <t>Gesamteinnahmen in Periode</t>
   </si>
   <si>
     <t>Einnahmen (Durchschnittskurs)</t>
-  </si>
-  <si>
-    <t>Projektpartner</t>
   </si>
   <si>
     <t>Gesamt (Durchschnittskurs)</t>
@@ -7236,55 +7230,55 @@
   <sheetData>
     <row r="3">
       <c r="H3" s="176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="O3" s="176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="V3" s="176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="AC3" s="176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="AJ3" s="176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="AQ3" s="176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="AX3" s="176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="BE3" s="176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="BL3" s="176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="BS3" s="176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="BZ3" s="176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="CG3" s="176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="CN3" s="176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="CU3" s="176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="DB3" s="176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="DI3" s="176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="DP3" s="176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="4">
@@ -8424,7 +8418,7 @@
         <f>=ROUND(IF(Saldovortrag_EUR="",0,Saldovortrag_EUR),2)</f>
       </c>
       <c r="I11" s="143" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="J11" s="116" t="str">
         <f>=ROUND(FB_SaldoLC_1,2)</f>
@@ -8439,7 +8433,7 @@
         <f>=ROUND(FB_SaldoEUR_1,2)</f>
       </c>
       <c r="P11" s="143" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="Q11" s="116" t="str">
         <f>=ROUND(FB_SaldoLC_2,2)</f>
@@ -8454,7 +8448,7 @@
         <f>=ROUND(FB_SaldoEUR_2,2)</f>
       </c>
       <c r="W11" s="143" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="X11" s="116" t="str">
         <f>=ROUND(FB_SaldoLC_3,2)</f>
@@ -8469,7 +8463,7 @@
         <f>=ROUND(FB_SaldoEUR_3,2)</f>
       </c>
       <c r="AD11" s="143" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="AE11" s="116" t="str">
         <f>=ROUND(FB_SaldoLC_4,2)</f>
@@ -8484,7 +8478,7 @@
         <f>=ROUND(FB_SaldoEUR_4,2)</f>
       </c>
       <c r="AK11" s="143" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="AL11" s="116" t="str">
         <f>=ROUND(FB_SaldoLC_5,2)</f>
@@ -8499,7 +8493,7 @@
         <f>=ROUND(FB_SaldoEUR_5,2)</f>
       </c>
       <c r="AR11" s="143" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="AS11" s="116" t="str">
         <f>=ROUND(FB_SaldoLC_6,2)</f>
@@ -8514,7 +8508,7 @@
         <f>=ROUND(FB_SaldoEUR_6,2)</f>
       </c>
       <c r="AY11" s="143" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="AZ11" s="116" t="str">
         <f>=ROUND(FB_SaldoLC_7,2)</f>
@@ -8529,7 +8523,7 @@
         <f>=ROUND(FB_SaldoEUR_7,2)</f>
       </c>
       <c r="BF11" s="143" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="BG11" s="116" t="str">
         <f>=ROUND(FB_SaldoLC_8,2)</f>
@@ -8544,7 +8538,7 @@
         <f>=ROUND(FB_SaldoEUR_8,2)</f>
       </c>
       <c r="BM11" s="143" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="BN11" s="116" t="str">
         <f>=ROUND(FB_SaldoLC_9,2)</f>
@@ -8559,7 +8553,7 @@
         <f>=ROUND(FB_SaldoEUR_9,2)</f>
       </c>
       <c r="BT11" s="143" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="BU11" s="116" t="str">
         <f>=ROUND(FB_SaldoLC_10,2)</f>
@@ -8574,7 +8568,7 @@
         <f>=ROUND(FB_SaldoEUR_10,2)</f>
       </c>
       <c r="CA11" s="143" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="CB11" s="116" t="str">
         <f>=ROUND(FB_SaldoLC_11,2)</f>
@@ -8589,7 +8583,7 @@
         <f>=ROUND(FB_SaldoEUR_11,2)</f>
       </c>
       <c r="CH11" s="143" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="CI11" s="116" t="str">
         <f>=ROUND(FB_SaldoLC_12,2)</f>
@@ -8604,7 +8598,7 @@
         <f>=ROUND(FB_SaldoEUR_12,2)</f>
       </c>
       <c r="CO11" s="143" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="CP11" s="116" t="str">
         <f>=ROUND(FB_SaldoLC_13,2)</f>
@@ -8619,7 +8613,7 @@
         <f>=ROUND(FB_SaldoEUR_13,2)</f>
       </c>
       <c r="CV11" s="143" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="CW11" s="116" t="str">
         <f>=ROUND(FB_SaldoLC_14,2)</f>
@@ -8634,7 +8628,7 @@
         <f>=ROUND(FB_SaldoEUR_14,2)</f>
       </c>
       <c r="DC11" s="143" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="DD11" s="116" t="str">
         <f>=ROUND(FB_SaldoLC_15,2)</f>
@@ -8649,7 +8643,7 @@
         <f>=ROUND(FB_SaldoEUR_15,2)</f>
       </c>
       <c r="DJ11" s="143" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="DK11" s="116" t="str">
         <f>=ROUND(FB_SaldoLC_16,2)</f>
@@ -8664,7 +8658,7 @@
         <f>=ROUND(FB_SaldoEUR_16,2)</f>
       </c>
       <c r="DQ11" s="143" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="DR11" s="116" t="str">
         <f>=ROUND(FB_SaldoLC_17,2)</f>
@@ -14546,7 +14540,7 @@
         <f>=ROUND(IFERROR(D43/E43,0),6)</f>
       </c>
       <c r="I43" s="160" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="J43" s="161" t="s">
         <v>158</v>
@@ -14561,7 +14555,7 @@
         <f>=ROUND(IFERROR(K43/L43,0),6)</f>
       </c>
       <c r="P43" s="160" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="Q43" s="161" t="s">
         <v>158</v>
@@ -14576,7 +14570,7 @@
         <f>=ROUND(IFERROR(R43/S43,0),6)</f>
       </c>
       <c r="W43" s="160" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="X43" s="161" t="s">
         <v>158</v>
@@ -14591,7 +14585,7 @@
         <f>=ROUND(IFERROR(Y43/Z43,0),6)</f>
       </c>
       <c r="AD43" s="160" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="AE43" s="161" t="s">
         <v>158</v>
@@ -14606,7 +14600,7 @@
         <f>=ROUND(IFERROR(AF43/AG43,0),6)</f>
       </c>
       <c r="AK43" s="160" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="AL43" s="161" t="s">
         <v>158</v>
@@ -14621,7 +14615,7 @@
         <f>=ROUND(IFERROR(AM43/AN43,0),6)</f>
       </c>
       <c r="AR43" s="160" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="AS43" s="161" t="s">
         <v>158</v>
@@ -14636,7 +14630,7 @@
         <f>=ROUND(IFERROR(AT43/AU43,0),6)</f>
       </c>
       <c r="AY43" s="160" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="AZ43" s="161" t="s">
         <v>158</v>
@@ -14651,7 +14645,7 @@
         <f>=ROUND(IFERROR(BA43/BB43,0),6)</f>
       </c>
       <c r="BF43" s="160" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="BG43" s="161" t="s">
         <v>158</v>
@@ -14666,7 +14660,7 @@
         <f>=ROUND(IFERROR(BH43/BI43,0),6)</f>
       </c>
       <c r="BM43" s="160" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="BN43" s="161" t="s">
         <v>158</v>
@@ -14681,7 +14675,7 @@
         <f>=ROUND(IFERROR(BO43/BP43,0),6)</f>
       </c>
       <c r="BT43" s="160" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="BU43" s="161" t="s">
         <v>158</v>
@@ -14696,7 +14690,7 @@
         <f>=ROUND(IFERROR(BV43/BW43,0),6)</f>
       </c>
       <c r="CA43" s="160" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="CB43" s="161" t="s">
         <v>158</v>
@@ -14711,7 +14705,7 @@
         <f>=ROUND(IFERROR(CC43/CD43,0),6)</f>
       </c>
       <c r="CH43" s="160" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="CI43" s="161" t="s">
         <v>158</v>
@@ -14726,7 +14720,7 @@
         <f>=ROUND(IFERROR(CJ43/CK43,0),6)</f>
       </c>
       <c r="CO43" s="160" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="CP43" s="161" t="s">
         <v>158</v>
@@ -14741,7 +14735,7 @@
         <f>=ROUND(IFERROR(CQ43/CR43,0),6)</f>
       </c>
       <c r="CV43" s="160" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="CW43" s="161" t="s">
         <v>158</v>
@@ -14756,7 +14750,7 @@
         <f>=ROUND(IFERROR(CX43/CY43,0),6)</f>
       </c>
       <c r="DC43" s="160" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="DD43" s="161" t="s">
         <v>158</v>
@@ -14771,7 +14765,7 @@
         <f>=ROUND(IFERROR(DE43/DF43,0),6)</f>
       </c>
       <c r="DJ43" s="160" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="DK43" s="161" t="s">
         <v>158</v>
@@ -14786,7 +14780,7 @@
         <f>=ROUND(IFERROR(DL43/DM43,0),6)</f>
       </c>
       <c r="DQ43" s="160" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="DR43" s="161" t="s">
         <v>158</v>
@@ -14806,7 +14800,7 @@
         <v>199</v>
       </c>
       <c r="C44" s="166" t="s">
-        <v>320</v>
+        <v>158</v>
       </c>
       <c r="D44" s="167">
         <v>1250000</v>
@@ -14821,7 +14815,7 @@
         <v>199</v>
       </c>
       <c r="J44" s="166" t="s">
-        <v>320</v>
+        <v>158</v>
       </c>
       <c r="K44" s="167">
         <v>1000000</v>
@@ -14836,7 +14830,7 @@
         <v>199</v>
       </c>
       <c r="Q44" s="166" t="s">
-        <v>320</v>
+        <v>158</v>
       </c>
       <c r="R44" s="167"/>
       <c r="S44" s="168"/>
@@ -14847,7 +14841,7 @@
         <v>199</v>
       </c>
       <c r="X44" s="166" t="s">
-        <v>320</v>
+        <v>158</v>
       </c>
       <c r="Y44" s="167"/>
       <c r="Z44" s="168"/>
@@ -14858,7 +14852,7 @@
         <v>199</v>
       </c>
       <c r="AE44" s="166" t="s">
-        <v>320</v>
+        <v>158</v>
       </c>
       <c r="AF44" s="167"/>
       <c r="AG44" s="168"/>
@@ -14869,7 +14863,7 @@
         <v>199</v>
       </c>
       <c r="AL44" s="166" t="s">
-        <v>320</v>
+        <v>158</v>
       </c>
       <c r="AM44" s="167"/>
       <c r="AN44" s="168"/>
@@ -14880,7 +14874,7 @@
         <v>199</v>
       </c>
       <c r="AS44" s="166" t="s">
-        <v>320</v>
+        <v>158</v>
       </c>
       <c r="AT44" s="167"/>
       <c r="AU44" s="168"/>
@@ -14891,7 +14885,7 @@
         <v>199</v>
       </c>
       <c r="AZ44" s="166" t="s">
-        <v>320</v>
+        <v>158</v>
       </c>
       <c r="BA44" s="167"/>
       <c r="BB44" s="168"/>
@@ -14902,7 +14896,7 @@
         <v>199</v>
       </c>
       <c r="BG44" s="166" t="s">
-        <v>320</v>
+        <v>158</v>
       </c>
       <c r="BH44" s="167"/>
       <c r="BI44" s="168"/>
@@ -14913,7 +14907,7 @@
         <v>199</v>
       </c>
       <c r="BN44" s="166" t="s">
-        <v>320</v>
+        <v>158</v>
       </c>
       <c r="BO44" s="167"/>
       <c r="BP44" s="168"/>
@@ -14924,7 +14918,7 @@
         <v>199</v>
       </c>
       <c r="BU44" s="166" t="s">
-        <v>320</v>
+        <v>158</v>
       </c>
       <c r="BV44" s="167"/>
       <c r="BW44" s="168"/>
@@ -14935,7 +14929,7 @@
         <v>199</v>
       </c>
       <c r="CB44" s="166" t="s">
-        <v>320</v>
+        <v>158</v>
       </c>
       <c r="CC44" s="167"/>
       <c r="CD44" s="168"/>
@@ -14946,7 +14940,7 @@
         <v>199</v>
       </c>
       <c r="CI44" s="166" t="s">
-        <v>320</v>
+        <v>158</v>
       </c>
       <c r="CJ44" s="167"/>
       <c r="CK44" s="168"/>
@@ -14957,7 +14951,7 @@
         <v>199</v>
       </c>
       <c r="CP44" s="166" t="s">
-        <v>320</v>
+        <v>158</v>
       </c>
       <c r="CQ44" s="167"/>
       <c r="CR44" s="168"/>
@@ -14968,7 +14962,7 @@
         <v>199</v>
       </c>
       <c r="CW44" s="166" t="s">
-        <v>320</v>
+        <v>158</v>
       </c>
       <c r="CX44" s="167"/>
       <c r="CY44" s="168"/>
@@ -14979,7 +14973,7 @@
         <v>199</v>
       </c>
       <c r="DD44" s="166" t="s">
-        <v>320</v>
+        <v>158</v>
       </c>
       <c r="DE44" s="167"/>
       <c r="DF44" s="168"/>
@@ -14990,7 +14984,7 @@
         <v>199</v>
       </c>
       <c r="DK44" s="166" t="s">
-        <v>320</v>
+        <v>158</v>
       </c>
       <c r="DL44" s="167"/>
       <c r="DM44" s="168"/>
@@ -15001,7 +14995,7 @@
         <v>199</v>
       </c>
       <c r="DR44" s="166" t="s">
-        <v>320</v>
+        <v>158</v>
       </c>
       <c r="DS44" s="167"/>
       <c r="DT44" s="168"/>
@@ -15611,7 +15605,7 @@
     </row>
     <row r="48">
       <c r="B48" s="170" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C48" s="171" t="s">
         <v>292</v>
@@ -15626,7 +15620,7 @@
         <f>=ROUND(IFERROR(D48/E48,0),6)</f>
       </c>
       <c r="I48" s="170" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="J48" s="171" t="s">
         <v>292</v>
@@ -15641,7 +15635,7 @@
         <f>=ROUND(IFERROR(K48/L48,0),6)</f>
       </c>
       <c r="P48" s="170" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="Q48" s="171" t="s">
         <v>292</v>
@@ -15656,7 +15650,7 @@
         <f>=ROUND(IFERROR(R48/S48,0),6)</f>
       </c>
       <c r="W48" s="170" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="X48" s="171" t="s">
         <v>292</v>
@@ -15671,7 +15665,7 @@
         <f>=ROUND(IFERROR(Y48/Z48,0),6)</f>
       </c>
       <c r="AD48" s="170" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="AE48" s="171" t="s">
         <v>292</v>
@@ -15686,7 +15680,7 @@
         <f>=ROUND(IFERROR(AF48/AG48,0),6)</f>
       </c>
       <c r="AK48" s="170" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="AL48" s="171" t="s">
         <v>292</v>
@@ -15701,7 +15695,7 @@
         <f>=ROUND(IFERROR(AM48/AN48,0),6)</f>
       </c>
       <c r="AR48" s="170" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="AS48" s="171" t="s">
         <v>292</v>
@@ -15716,7 +15710,7 @@
         <f>=ROUND(IFERROR(AT48/AU48,0),6)</f>
       </c>
       <c r="AY48" s="170" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="AZ48" s="171" t="s">
         <v>292</v>
@@ -15731,7 +15725,7 @@
         <f>=ROUND(IFERROR(BA48/BB48,0),6)</f>
       </c>
       <c r="BF48" s="170" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="BG48" s="171" t="s">
         <v>292</v>
@@ -15746,7 +15740,7 @@
         <f>=ROUND(IFERROR(BH48/BI48,0),6)</f>
       </c>
       <c r="BM48" s="170" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="BN48" s="171" t="s">
         <v>292</v>
@@ -15761,7 +15755,7 @@
         <f>=ROUND(IFERROR(BO48/BP48,0),6)</f>
       </c>
       <c r="BT48" s="170" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="BU48" s="171" t="s">
         <v>292</v>
@@ -15776,7 +15770,7 @@
         <f>=ROUND(IFERROR(BV48/BW48,0),6)</f>
       </c>
       <c r="CA48" s="170" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="CB48" s="171" t="s">
         <v>292</v>
@@ -15791,7 +15785,7 @@
         <f>=ROUND(IFERROR(CC48/CD48,0),6)</f>
       </c>
       <c r="CH48" s="170" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="CI48" s="171" t="s">
         <v>292</v>
@@ -15806,7 +15800,7 @@
         <f>=ROUND(IFERROR(CJ48/CK48,0),6)</f>
       </c>
       <c r="CO48" s="170" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="CP48" s="171" t="s">
         <v>292</v>
@@ -15821,7 +15815,7 @@
         <f>=ROUND(IFERROR(CQ48/CR48,0),6)</f>
       </c>
       <c r="CV48" s="170" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="CW48" s="171" t="s">
         <v>292</v>
@@ -15836,7 +15830,7 @@
         <f>=ROUND(IFERROR(CX48/CY48,0),6)</f>
       </c>
       <c r="DC48" s="170" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="DD48" s="171" t="s">
         <v>292</v>
@@ -15851,7 +15845,7 @@
         <f>=ROUND(IFERROR(DE48/DF48,0),6)</f>
       </c>
       <c r="DJ48" s="170" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="DK48" s="171" t="s">
         <v>292</v>
@@ -15866,7 +15860,7 @@
         <f>=ROUND(IFERROR(DL48/DM48,0),6)</f>
       </c>
       <c r="DQ48" s="170" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="DR48" s="171" t="s">
         <v>292</v>
@@ -15883,58 +15877,58 @@
     </row>
     <row r="50">
       <c r="B50" s="105" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="I50" s="105" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="P50" s="105" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="W50" s="105" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="AD50" s="105" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="AK50" s="105" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="AR50" s="105" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="AY50" s="105" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="BF50" s="105" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="BM50" s="105" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="BT50" s="105" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="CA50" s="105" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="CH50" s="105" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="CO50" s="105" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="CV50" s="105" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="DC50" s="105" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="DJ50" s="105" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="DQ50" s="105" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="51">
@@ -16214,7 +16208,7 @@
         <v>194</v>
       </c>
       <c r="C52" s="166" t="s">
-        <v>323</v>
+        <v>158</v>
       </c>
       <c r="D52" s="167">
         <v>250000</v>
@@ -16229,7 +16223,7 @@
         <v>194</v>
       </c>
       <c r="J52" s="166" t="s">
-        <v>323</v>
+        <v>158</v>
       </c>
       <c r="K52" s="167">
         <v>200000</v>
@@ -16244,7 +16238,7 @@
         <v>194</v>
       </c>
       <c r="Q52" s="166" t="s">
-        <v>323</v>
+        <v>158</v>
       </c>
       <c r="R52" s="167"/>
       <c r="S52" s="175" t="str">
@@ -16257,7 +16251,7 @@
         <v>194</v>
       </c>
       <c r="X52" s="166" t="s">
-        <v>323</v>
+        <v>158</v>
       </c>
       <c r="Y52" s="167"/>
       <c r="Z52" s="175" t="str">
@@ -16270,7 +16264,7 @@
         <v>194</v>
       </c>
       <c r="AE52" s="166" t="s">
-        <v>323</v>
+        <v>158</v>
       </c>
       <c r="AF52" s="167"/>
       <c r="AG52" s="175" t="str">
@@ -16283,7 +16277,7 @@
         <v>194</v>
       </c>
       <c r="AL52" s="166" t="s">
-        <v>323</v>
+        <v>158</v>
       </c>
       <c r="AM52" s="167"/>
       <c r="AN52" s="175" t="str">
@@ -16296,7 +16290,7 @@
         <v>194</v>
       </c>
       <c r="AS52" s="166" t="s">
-        <v>323</v>
+        <v>158</v>
       </c>
       <c r="AT52" s="167"/>
       <c r="AU52" s="175" t="str">
@@ -16309,7 +16303,7 @@
         <v>194</v>
       </c>
       <c r="AZ52" s="166" t="s">
-        <v>323</v>
+        <v>158</v>
       </c>
       <c r="BA52" s="167"/>
       <c r="BB52" s="175" t="str">
@@ -16322,7 +16316,7 @@
         <v>194</v>
       </c>
       <c r="BG52" s="166" t="s">
-        <v>323</v>
+        <v>158</v>
       </c>
       <c r="BH52" s="167"/>
       <c r="BI52" s="175" t="str">
@@ -16335,7 +16329,7 @@
         <v>194</v>
       </c>
       <c r="BN52" s="166" t="s">
-        <v>323</v>
+        <v>158</v>
       </c>
       <c r="BO52" s="167"/>
       <c r="BP52" s="175" t="str">
@@ -16348,7 +16342,7 @@
         <v>194</v>
       </c>
       <c r="BU52" s="166" t="s">
-        <v>323</v>
+        <v>158</v>
       </c>
       <c r="BV52" s="167"/>
       <c r="BW52" s="175" t="str">
@@ -16361,7 +16355,7 @@
         <v>194</v>
       </c>
       <c r="CB52" s="166" t="s">
-        <v>323</v>
+        <v>158</v>
       </c>
       <c r="CC52" s="167"/>
       <c r="CD52" s="175" t="str">
@@ -16374,7 +16368,7 @@
         <v>194</v>
       </c>
       <c r="CI52" s="166" t="s">
-        <v>323</v>
+        <v>158</v>
       </c>
       <c r="CJ52" s="167"/>
       <c r="CK52" s="175" t="str">
@@ -16387,7 +16381,7 @@
         <v>194</v>
       </c>
       <c r="CP52" s="166" t="s">
-        <v>323</v>
+        <v>158</v>
       </c>
       <c r="CQ52" s="167"/>
       <c r="CR52" s="175" t="str">
@@ -16400,7 +16394,7 @@
         <v>194</v>
       </c>
       <c r="CW52" s="166" t="s">
-        <v>323</v>
+        <v>158</v>
       </c>
       <c r="CX52" s="167"/>
       <c r="CY52" s="175" t="str">
@@ -16413,7 +16407,7 @@
         <v>194</v>
       </c>
       <c r="DD52" s="166" t="s">
-        <v>323</v>
+        <v>158</v>
       </c>
       <c r="DE52" s="167"/>
       <c r="DF52" s="175" t="str">
@@ -16426,7 +16420,7 @@
         <v>194</v>
       </c>
       <c r="DK52" s="166" t="s">
-        <v>323</v>
+        <v>158</v>
       </c>
       <c r="DL52" s="167"/>
       <c r="DM52" s="175" t="str">
@@ -16439,7 +16433,7 @@
         <v>194</v>
       </c>
       <c r="DR52" s="166" t="s">
-        <v>323</v>
+        <v>158</v>
       </c>
       <c r="DS52" s="167"/>
       <c r="DT52" s="175" t="str">
@@ -16694,7 +16688,7 @@
         <v>301</v>
       </c>
       <c r="C54" s="166" t="s">
-        <v>311</v>
+        <v>158</v>
       </c>
       <c r="D54" s="167"/>
       <c r="E54" s="175" t="str">
@@ -16707,7 +16701,7 @@
         <v>301</v>
       </c>
       <c r="J54" s="166" t="s">
-        <v>311</v>
+        <v>158</v>
       </c>
       <c r="K54" s="167"/>
       <c r="L54" s="175" t="str">
@@ -16720,7 +16714,7 @@
         <v>301</v>
       </c>
       <c r="Q54" s="166" t="s">
-        <v>311</v>
+        <v>158</v>
       </c>
       <c r="R54" s="167"/>
       <c r="S54" s="175" t="str">
@@ -16733,7 +16727,7 @@
         <v>301</v>
       </c>
       <c r="X54" s="166" t="s">
-        <v>311</v>
+        <v>158</v>
       </c>
       <c r="Y54" s="167"/>
       <c r="Z54" s="175" t="str">
@@ -16746,7 +16740,7 @@
         <v>301</v>
       </c>
       <c r="AE54" s="166" t="s">
-        <v>311</v>
+        <v>158</v>
       </c>
       <c r="AF54" s="167"/>
       <c r="AG54" s="175" t="str">
@@ -16759,7 +16753,7 @@
         <v>301</v>
       </c>
       <c r="AL54" s="166" t="s">
-        <v>311</v>
+        <v>158</v>
       </c>
       <c r="AM54" s="167"/>
       <c r="AN54" s="175" t="str">
@@ -16772,7 +16766,7 @@
         <v>301</v>
       </c>
       <c r="AS54" s="166" t="s">
-        <v>311</v>
+        <v>158</v>
       </c>
       <c r="AT54" s="167"/>
       <c r="AU54" s="175" t="str">
@@ -16785,7 +16779,7 @@
         <v>301</v>
       </c>
       <c r="AZ54" s="166" t="s">
-        <v>311</v>
+        <v>158</v>
       </c>
       <c r="BA54" s="167"/>
       <c r="BB54" s="175" t="str">
@@ -16798,7 +16792,7 @@
         <v>301</v>
       </c>
       <c r="BG54" s="166" t="s">
-        <v>311</v>
+        <v>158</v>
       </c>
       <c r="BH54" s="167"/>
       <c r="BI54" s="175" t="str">
@@ -16811,7 +16805,7 @@
         <v>301</v>
       </c>
       <c r="BN54" s="166" t="s">
-        <v>311</v>
+        <v>158</v>
       </c>
       <c r="BO54" s="167"/>
       <c r="BP54" s="175" t="str">
@@ -16824,7 +16818,7 @@
         <v>301</v>
       </c>
       <c r="BU54" s="166" t="s">
-        <v>311</v>
+        <v>158</v>
       </c>
       <c r="BV54" s="167"/>
       <c r="BW54" s="175" t="str">
@@ -16837,7 +16831,7 @@
         <v>301</v>
       </c>
       <c r="CB54" s="166" t="s">
-        <v>311</v>
+        <v>158</v>
       </c>
       <c r="CC54" s="167"/>
       <c r="CD54" s="175" t="str">
@@ -16850,7 +16844,7 @@
         <v>301</v>
       </c>
       <c r="CI54" s="166" t="s">
-        <v>311</v>
+        <v>158</v>
       </c>
       <c r="CJ54" s="167"/>
       <c r="CK54" s="175" t="str">
@@ -16863,7 +16857,7 @@
         <v>301</v>
       </c>
       <c r="CP54" s="166" t="s">
-        <v>311</v>
+        <v>158</v>
       </c>
       <c r="CQ54" s="167"/>
       <c r="CR54" s="175" t="str">
@@ -16876,7 +16870,7 @@
         <v>301</v>
       </c>
       <c r="CW54" s="166" t="s">
-        <v>311</v>
+        <v>158</v>
       </c>
       <c r="CX54" s="167"/>
       <c r="CY54" s="175" t="str">
@@ -16889,7 +16883,7 @@
         <v>301</v>
       </c>
       <c r="DD54" s="166" t="s">
-        <v>311</v>
+        <v>158</v>
       </c>
       <c r="DE54" s="167"/>
       <c r="DF54" s="175" t="str">
@@ -16902,7 +16896,7 @@
         <v>301</v>
       </c>
       <c r="DK54" s="166" t="s">
-        <v>311</v>
+        <v>158</v>
       </c>
       <c r="DL54" s="167"/>
       <c r="DM54" s="175" t="str">
@@ -16915,7 +16909,7 @@
         <v>301</v>
       </c>
       <c r="DR54" s="166" t="s">
-        <v>311</v>
+        <v>158</v>
       </c>
       <c r="DS54" s="167"/>
       <c r="DT54" s="175" t="str">
@@ -17635,7 +17629,7 @@
     </row>
     <row r="58">
       <c r="B58" s="170" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C58" s="171" t="s">
         <v>292</v>
@@ -17650,7 +17644,7 @@
         <f>=ROUND(IFERROR(D58/E58,0),6)</f>
       </c>
       <c r="I58" s="170" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="J58" s="171" t="s">
         <v>292</v>
@@ -17665,7 +17659,7 @@
         <f>=ROUND(IFERROR(K58/L58,0),6)</f>
       </c>
       <c r="P58" s="170" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="Q58" s="171" t="s">
         <v>292</v>
@@ -17680,7 +17674,7 @@
         <f>=ROUND(IFERROR(R58/S58,0),6)</f>
       </c>
       <c r="W58" s="170" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="X58" s="171" t="s">
         <v>292</v>
@@ -17695,7 +17689,7 @@
         <f>=ROUND(IFERROR(Y58/Z58,0),6)</f>
       </c>
       <c r="AD58" s="170" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="AE58" s="171" t="s">
         <v>292</v>
@@ -17710,7 +17704,7 @@
         <f>=ROUND(IFERROR(AF58/AG58,0),6)</f>
       </c>
       <c r="AK58" s="170" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="AL58" s="171" t="s">
         <v>292</v>
@@ -17725,7 +17719,7 @@
         <f>=ROUND(IFERROR(AM58/AN58,0),6)</f>
       </c>
       <c r="AR58" s="170" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="AS58" s="171" t="s">
         <v>292</v>
@@ -17740,7 +17734,7 @@
         <f>=ROUND(IFERROR(AT58/AU58,0),6)</f>
       </c>
       <c r="AY58" s="170" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="AZ58" s="171" t="s">
         <v>292</v>
@@ -17755,7 +17749,7 @@
         <f>=ROUND(IFERROR(BA58/BB58,0),6)</f>
       </c>
       <c r="BF58" s="170" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="BG58" s="171" t="s">
         <v>292</v>
@@ -17770,7 +17764,7 @@
         <f>=ROUND(IFERROR(BH58/BI58,0),6)</f>
       </c>
       <c r="BM58" s="170" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="BN58" s="171" t="s">
         <v>292</v>
@@ -17785,7 +17779,7 @@
         <f>=ROUND(IFERROR(BO58/BP58,0),6)</f>
       </c>
       <c r="BT58" s="170" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="BU58" s="171" t="s">
         <v>292</v>
@@ -17800,7 +17794,7 @@
         <f>=ROUND(IFERROR(BV58/BW58,0),6)</f>
       </c>
       <c r="CA58" s="170" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="CB58" s="171" t="s">
         <v>292</v>
@@ -17815,7 +17809,7 @@
         <f>=ROUND(IFERROR(CC58/CD58,0),6)</f>
       </c>
       <c r="CH58" s="170" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="CI58" s="171" t="s">
         <v>292</v>
@@ -17830,7 +17824,7 @@
         <f>=ROUND(IFERROR(CJ58/CK58,0),6)</f>
       </c>
       <c r="CO58" s="170" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="CP58" s="171" t="s">
         <v>292</v>
@@ -17845,7 +17839,7 @@
         <f>=ROUND(IFERROR(CQ58/CR58,0),6)</f>
       </c>
       <c r="CV58" s="170" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="CW58" s="171" t="s">
         <v>292</v>
@@ -17860,7 +17854,7 @@
         <f>=ROUND(IFERROR(CX58/CY58,0),6)</f>
       </c>
       <c r="DC58" s="170" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="DD58" s="171" t="s">
         <v>292</v>
@@ -17875,7 +17869,7 @@
         <f>=ROUND(IFERROR(DE58/DF58,0),6)</f>
       </c>
       <c r="DJ58" s="170" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="DK58" s="171" t="s">
         <v>292</v>
@@ -17890,7 +17884,7 @@
         <f>=ROUND(IFERROR(DL58/DM58,0),6)</f>
       </c>
       <c r="DQ58" s="170" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="DR58" s="171" t="s">
         <v>292</v>
@@ -18521,55 +18515,55 @@
   <sheetData>
     <row r="3">
       <c r="E3" s="176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="I3" s="176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="M3" s="176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="Q3" s="176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="U3" s="176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="Y3" s="176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="AC3" s="176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="AG3" s="176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="AK3" s="176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="AO3" s="176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="AS3" s="176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="AW3" s="176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="BA3" s="176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="BE3" s="176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="BI3" s="176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="BM3" s="176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="BQ3" s="176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="4">
@@ -19022,96 +19016,96 @@
     </row>
     <row r="8">
       <c r="B8" s="105" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="C8" s="179">
         <v>125</v>
       </c>
       <c r="D8" s="179"/>
       <c r="F8" s="105" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="G8" s="179">
         <v>125</v>
       </c>
       <c r="H8" s="179"/>
       <c r="J8" s="105" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="K8" s="179"/>
       <c r="L8" s="179"/>
       <c r="N8" s="105" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="O8" s="179"/>
       <c r="P8" s="179"/>
       <c r="R8" s="105" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="S8" s="179"/>
       <c r="T8" s="179"/>
       <c r="V8" s="105" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="W8" s="179"/>
       <c r="X8" s="179"/>
       <c r="Z8" s="105" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="AA8" s="179"/>
       <c r="AB8" s="179"/>
       <c r="AD8" s="105" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="AE8" s="179"/>
       <c r="AF8" s="179"/>
       <c r="AH8" s="105" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="AI8" s="179"/>
       <c r="AJ8" s="179"/>
       <c r="AL8" s="105" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="AM8" s="179"/>
       <c r="AN8" s="179"/>
       <c r="AP8" s="105" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="AQ8" s="179"/>
       <c r="AR8" s="179"/>
       <c r="AT8" s="105" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="AU8" s="179"/>
       <c r="AV8" s="179"/>
       <c r="AX8" s="105" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="AY8" s="179"/>
       <c r="AZ8" s="179"/>
       <c r="BB8" s="105" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="BC8" s="179"/>
       <c r="BD8" s="179"/>
       <c r="BF8" s="105" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="BG8" s="179"/>
       <c r="BH8" s="179"/>
       <c r="BJ8" s="105" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="BK8" s="179"/>
       <c r="BL8" s="179"/>
       <c r="BN8" s="105" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="BO8" s="179"/>
       <c r="BP8" s="179"/>
       <c r="BR8" s="105" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="BS8" s="179"/>
       <c r="BT8" s="179"/>
@@ -19121,163 +19115,163 @@
         <v>202</v>
       </c>
       <c r="C9" s="180" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="D9" s="180" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="F9" s="180" t="s">
         <v>202</v>
       </c>
       <c r="G9" s="180" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="H9" s="180" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="J9" s="180" t="s">
         <v>202</v>
       </c>
       <c r="K9" s="180" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="L9" s="180" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="N9" s="180" t="s">
         <v>202</v>
       </c>
       <c r="O9" s="180" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="P9" s="180" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="R9" s="180" t="s">
         <v>202</v>
       </c>
       <c r="S9" s="180" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="T9" s="180" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="V9" s="180" t="s">
         <v>202</v>
       </c>
       <c r="W9" s="180" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="X9" s="180" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="Z9" s="180" t="s">
         <v>202</v>
       </c>
       <c r="AA9" s="180" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="AB9" s="180" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="AD9" s="180" t="s">
         <v>202</v>
       </c>
       <c r="AE9" s="180" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="AF9" s="180" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="AH9" s="180" t="s">
         <v>202</v>
       </c>
       <c r="AI9" s="180" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="AJ9" s="180" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="AL9" s="180" t="s">
         <v>202</v>
       </c>
       <c r="AM9" s="180" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="AN9" s="180" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="AP9" s="180" t="s">
         <v>202</v>
       </c>
       <c r="AQ9" s="180" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="AR9" s="180" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="AT9" s="180" t="s">
         <v>202</v>
       </c>
       <c r="AU9" s="180" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="AV9" s="180" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="AX9" s="180" t="s">
         <v>202</v>
       </c>
       <c r="AY9" s="180" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="AZ9" s="180" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="BB9" s="180" t="s">
         <v>202</v>
       </c>
       <c r="BC9" s="180" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="BD9" s="180" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="BF9" s="180" t="s">
         <v>202</v>
       </c>
       <c r="BG9" s="180" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="BH9" s="180" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="BJ9" s="180" t="s">
         <v>202</v>
       </c>
       <c r="BK9" s="180" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="BL9" s="180" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="BN9" s="180" t="s">
         <v>202</v>
       </c>
       <c r="BO9" s="180" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="BP9" s="180" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="BR9" s="180" t="s">
         <v>202</v>
       </c>
       <c r="BS9" s="180" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="BT9" s="180" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="10">
@@ -20328,7 +20322,7 @@
     </row>
     <row r="18">
       <c r="B18" s="183" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="C18" s="184" t="str">
         <f>=ROUND(SUBTOTAL(109,MA_1[Angefordert (LC)]),2)</f>
@@ -20337,7 +20331,7 @@
         <f>=ROUND(SUBTOTAL(109,MA_1[Angefordert (EUR)]),2)</f>
       </c>
       <c r="F18" s="183" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="G18" s="184" t="str">
         <f>=ROUND(SUBTOTAL(109,MA_2[Angefordert (LC)]),2)</f>
@@ -20346,7 +20340,7 @@
         <f>=ROUND(SUBTOTAL(109,MA_2[Angefordert (EUR)]),2)</f>
       </c>
       <c r="J18" s="183" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="K18" s="184" t="str">
         <f>=ROUND(SUBTOTAL(109,MA_3[Angefordert (LC)]),2)</f>
@@ -20355,7 +20349,7 @@
         <f>=ROUND(SUBTOTAL(109,MA_3[Angefordert (EUR)]),2)</f>
       </c>
       <c r="N18" s="183" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="O18" s="184" t="str">
         <f>=ROUND(SUBTOTAL(109,MA_4[Angefordert (LC)]),2)</f>
@@ -20364,7 +20358,7 @@
         <f>=ROUND(SUBTOTAL(109,MA_4[Angefordert (EUR)]),2)</f>
       </c>
       <c r="R18" s="183" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="S18" s="184" t="str">
         <f>=ROUND(SUBTOTAL(109,MA_5[Angefordert (LC)]),2)</f>
@@ -20373,7 +20367,7 @@
         <f>=ROUND(SUBTOTAL(109,MA_5[Angefordert (EUR)]),2)</f>
       </c>
       <c r="V18" s="183" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="W18" s="184" t="str">
         <f>=ROUND(SUBTOTAL(109,MA_6[Angefordert (LC)]),2)</f>
@@ -20382,7 +20376,7 @@
         <f>=ROUND(SUBTOTAL(109,MA_6[Angefordert (EUR)]),2)</f>
       </c>
       <c r="Z18" s="183" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="AA18" s="184" t="str">
         <f>=ROUND(SUBTOTAL(109,MA_7[Angefordert (LC)]),2)</f>
@@ -20391,7 +20385,7 @@
         <f>=ROUND(SUBTOTAL(109,MA_7[Angefordert (EUR)]),2)</f>
       </c>
       <c r="AD18" s="183" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="AE18" s="184" t="str">
         <f>=ROUND(SUBTOTAL(109,MA_8[Angefordert (LC)]),2)</f>
@@ -20400,7 +20394,7 @@
         <f>=ROUND(SUBTOTAL(109,MA_8[Angefordert (EUR)]),2)</f>
       </c>
       <c r="AH18" s="183" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="AI18" s="184" t="str">
         <f>=ROUND(SUBTOTAL(109,MA_9[Angefordert (LC)]),2)</f>
@@ -20409,7 +20403,7 @@
         <f>=ROUND(SUBTOTAL(109,MA_9[Angefordert (EUR)]),2)</f>
       </c>
       <c r="AL18" s="183" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="AM18" s="184" t="str">
         <f>=ROUND(SUBTOTAL(109,MA_10[Angefordert (LC)]),2)</f>
@@ -20418,7 +20412,7 @@
         <f>=ROUND(SUBTOTAL(109,MA_10[Angefordert (EUR)]),2)</f>
       </c>
       <c r="AP18" s="183" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="AQ18" s="184" t="str">
         <f>=ROUND(SUBTOTAL(109,MA_11[Angefordert (LC)]),2)</f>
@@ -20427,7 +20421,7 @@
         <f>=ROUND(SUBTOTAL(109,MA_11[Angefordert (EUR)]),2)</f>
       </c>
       <c r="AT18" s="183" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="AU18" s="184" t="str">
         <f>=ROUND(SUBTOTAL(109,MA_12[Angefordert (LC)]),2)</f>
@@ -20436,7 +20430,7 @@
         <f>=ROUND(SUBTOTAL(109,MA_12[Angefordert (EUR)]),2)</f>
       </c>
       <c r="AX18" s="183" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="AY18" s="184" t="str">
         <f>=ROUND(SUBTOTAL(109,MA_13[Angefordert (LC)]),2)</f>
@@ -20445,7 +20439,7 @@
         <f>=ROUND(SUBTOTAL(109,MA_13[Angefordert (EUR)]),2)</f>
       </c>
       <c r="BB18" s="183" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="BC18" s="184" t="str">
         <f>=ROUND(SUBTOTAL(109,MA_14[Angefordert (LC)]),2)</f>
@@ -20454,7 +20448,7 @@
         <f>=ROUND(SUBTOTAL(109,MA_14[Angefordert (EUR)]),2)</f>
       </c>
       <c r="BF18" s="183" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="BG18" s="184" t="str">
         <f>=ROUND(SUBTOTAL(109,MA_15[Angefordert (LC)]),2)</f>
@@ -20463,7 +20457,7 @@
         <f>=ROUND(SUBTOTAL(109,MA_15[Angefordert (EUR)]),2)</f>
       </c>
       <c r="BJ18" s="183" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="BK18" s="184" t="str">
         <f>=ROUND(SUBTOTAL(109,MA_16[Angefordert (LC)]),2)</f>
@@ -20472,7 +20466,7 @@
         <f>=ROUND(SUBTOTAL(109,MA_16[Angefordert (EUR)]),2)</f>
       </c>
       <c r="BN18" s="183" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="BO18" s="184" t="str">
         <f>=ROUND(SUBTOTAL(109,MA_17[Angefordert (LC)]),2)</f>
@@ -20481,7 +20475,7 @@
         <f>=ROUND(SUBTOTAL(109,MA_17[Angefordert (EUR)]),2)</f>
       </c>
       <c r="BR18" s="183" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="BS18" s="184" t="str">
         <f>=ROUND(SUBTOTAL(109,MA_18[Angefordert (LC)]),2)</f>
@@ -20492,7 +20486,7 @@
     </row>
     <row r="20">
       <c r="B20" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="C20" s="186" t="str">
         <f>=ROUND($C$18,2)</f>
@@ -20501,7 +20495,7 @@
         <f>=ROUND($D$18,2)</f>
       </c>
       <c r="F20" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="G20" s="186" t="str">
         <f>=ROUND($G$18,2)</f>
@@ -20510,7 +20504,7 @@
         <f>=ROUND($H$18,2)</f>
       </c>
       <c r="J20" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="K20" s="186" t="str">
         <f>=ROUND($K$18,2)</f>
@@ -20519,7 +20513,7 @@
         <f>=ROUND($L$18,2)</f>
       </c>
       <c r="N20" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="O20" s="186" t="str">
         <f>=ROUND($O$18,2)</f>
@@ -20528,7 +20522,7 @@
         <f>=ROUND($P$18,2)</f>
       </c>
       <c r="R20" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="S20" s="186" t="str">
         <f>=ROUND($S$18,2)</f>
@@ -20537,7 +20531,7 @@
         <f>=ROUND($T$18,2)</f>
       </c>
       <c r="V20" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="W20" s="186" t="str">
         <f>=ROUND($W$18,2)</f>
@@ -20546,7 +20540,7 @@
         <f>=ROUND($X$18,2)</f>
       </c>
       <c r="Z20" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="AA20" s="186" t="str">
         <f>=ROUND($AA$18,2)</f>
@@ -20555,7 +20549,7 @@
         <f>=ROUND($AB$18,2)</f>
       </c>
       <c r="AD20" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="AE20" s="186" t="str">
         <f>=ROUND($AE$18,2)</f>
@@ -20564,7 +20558,7 @@
         <f>=ROUND($AF$18,2)</f>
       </c>
       <c r="AH20" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="AI20" s="186" t="str">
         <f>=ROUND($AI$18,2)</f>
@@ -20573,7 +20567,7 @@
         <f>=ROUND($AJ$18,2)</f>
       </c>
       <c r="AL20" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="AM20" s="186" t="str">
         <f>=ROUND($AM$18,2)</f>
@@ -20582,7 +20576,7 @@
         <f>=ROUND($AN$18,2)</f>
       </c>
       <c r="AP20" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="AQ20" s="186" t="str">
         <f>=ROUND($AQ$18,2)</f>
@@ -20591,7 +20585,7 @@
         <f>=ROUND($AR$18,2)</f>
       </c>
       <c r="AT20" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="AU20" s="186" t="str">
         <f>=ROUND($AU$18,2)</f>
@@ -20600,7 +20594,7 @@
         <f>=ROUND($AV$18,2)</f>
       </c>
       <c r="AX20" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="AY20" s="186" t="str">
         <f>=ROUND($AY$18,2)</f>
@@ -20609,7 +20603,7 @@
         <f>=ROUND($AZ$18,2)</f>
       </c>
       <c r="BB20" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BC20" s="186" t="str">
         <f>=ROUND($BC$18,2)</f>
@@ -20618,7 +20612,7 @@
         <f>=ROUND($BD$18,2)</f>
       </c>
       <c r="BF20" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BG20" s="186" t="str">
         <f>=ROUND($BG$18,2)</f>
@@ -20627,7 +20621,7 @@
         <f>=ROUND($BH$18,2)</f>
       </c>
       <c r="BJ20" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BK20" s="186" t="str">
         <f>=ROUND($BK$18,2)</f>
@@ -20636,7 +20630,7 @@
         <f>=ROUND($BL$18,2)</f>
       </c>
       <c r="BN20" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BO20" s="186" t="str">
         <f>=ROUND($BO$18,2)</f>
@@ -20645,7 +20639,7 @@
         <f>=ROUND($BP$18,2)</f>
       </c>
       <c r="BR20" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="BS20" s="186" t="str">
         <f>=ROUND($BS$18,2)</f>
@@ -20656,7 +20650,7 @@
     </row>
     <row r="21">
       <c r="B21" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="C21" s="24">
         <v>250000</v>
@@ -20665,7 +20659,7 @@
         <f>=IFERROR(ROUND($C$21/$C$8,2),0)</f>
       </c>
       <c r="F21" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="G21" s="24">
         <v>200000</v>
@@ -20674,112 +20668,112 @@
         <f>=IFERROR(ROUND($G$21/$G$8,2),0)</f>
       </c>
       <c r="J21" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="K21" s="24"/>
       <c r="L21" s="182" t="str">
         <f>=IFERROR(ROUND($K$21/$K$8,2),0)</f>
       </c>
       <c r="N21" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="O21" s="24"/>
       <c r="P21" s="182" t="str">
         <f>=IFERROR(ROUND($O$21/$O$8,2),0)</f>
       </c>
       <c r="R21" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="S21" s="24"/>
       <c r="T21" s="182" t="str">
         <f>=IFERROR(ROUND($S$21/$S$8,2),0)</f>
       </c>
       <c r="V21" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="W21" s="24"/>
       <c r="X21" s="182" t="str">
         <f>=IFERROR(ROUND($W$21/$W$8,2),0)</f>
       </c>
       <c r="Z21" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="AA21" s="24"/>
       <c r="AB21" s="182" t="str">
         <f>=IFERROR(ROUND($AA$21/$AA$8,2),0)</f>
       </c>
       <c r="AD21" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="AE21" s="24"/>
       <c r="AF21" s="182" t="str">
         <f>=IFERROR(ROUND($AE$21/$AE$8,2),0)</f>
       </c>
       <c r="AH21" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="AI21" s="24"/>
       <c r="AJ21" s="182" t="str">
         <f>=IFERROR(ROUND($AI$21/$AI$8,2),0)</f>
       </c>
       <c r="AL21" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="AM21" s="24"/>
       <c r="AN21" s="182" t="str">
         <f>=IFERROR(ROUND($AM$21/$AM$8,2),0)</f>
       </c>
       <c r="AP21" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="AQ21" s="24"/>
       <c r="AR21" s="182" t="str">
         <f>=IFERROR(ROUND($AQ$21/$AQ$8,2),0)</f>
       </c>
       <c r="AT21" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="AU21" s="24"/>
       <c r="AV21" s="182" t="str">
         <f>=IFERROR(ROUND($AU$21/$AU$8,2),0)</f>
       </c>
       <c r="AX21" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="AY21" s="24"/>
       <c r="AZ21" s="182" t="str">
         <f>=IFERROR(ROUND($AY$21/$AY$8,2),0)</f>
       </c>
       <c r="BB21" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="BC21" s="24"/>
       <c r="BD21" s="182" t="str">
         <f>=IFERROR(ROUND($BC$21/$BC$8,2),0)</f>
       </c>
       <c r="BF21" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="BG21" s="24"/>
       <c r="BH21" s="182" t="str">
         <f>=IFERROR(ROUND($BG$21/$BG$8,2),0)</f>
       </c>
       <c r="BJ21" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="BK21" s="24"/>
       <c r="BL21" s="182" t="str">
         <f>=IFERROR(ROUND($BK$21/$BK$8,2),0)</f>
       </c>
       <c r="BN21" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="BO21" s="24"/>
       <c r="BP21" s="182" t="str">
         <f>=IFERROR(ROUND($BO$21/$BO$8,2),0)</f>
       </c>
       <c r="BR21" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="BS21" s="24"/>
       <c r="BT21" s="182" t="str">
@@ -20788,7 +20782,7 @@
     </row>
     <row r="22">
       <c r="B22" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="C22" s="24">
         <v>125000</v>
@@ -20797,7 +20791,7 @@
         <f>=IFERROR(ROUND($C$22/$C$8,2),0)</f>
       </c>
       <c r="F22" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="G22" s="24">
         <v>100000</v>
@@ -20806,112 +20800,112 @@
         <f>=IFERROR(ROUND($G$22/$G$8,2),0)</f>
       </c>
       <c r="J22" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="K22" s="24"/>
       <c r="L22" s="182" t="str">
         <f>=IFERROR(ROUND($K$22/$K$8,2),0)</f>
       </c>
       <c r="N22" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="O22" s="24"/>
       <c r="P22" s="182" t="str">
         <f>=IFERROR(ROUND($O$22/$O$8,2),0)</f>
       </c>
       <c r="R22" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="S22" s="24"/>
       <c r="T22" s="182" t="str">
         <f>=IFERROR(ROUND($S$22/$S$8,2),0)</f>
       </c>
       <c r="V22" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="W22" s="24"/>
       <c r="X22" s="182" t="str">
         <f>=IFERROR(ROUND($W$22/$W$8,2),0)</f>
       </c>
       <c r="Z22" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="AA22" s="24"/>
       <c r="AB22" s="182" t="str">
         <f>=IFERROR(ROUND($AA$22/$AA$8,2),0)</f>
       </c>
       <c r="AD22" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="AE22" s="24"/>
       <c r="AF22" s="182" t="str">
         <f>=IFERROR(ROUND($AE$22/$AE$8,2),0)</f>
       </c>
       <c r="AH22" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="AI22" s="24"/>
       <c r="AJ22" s="182" t="str">
         <f>=IFERROR(ROUND($AI$22/$AI$8,2),0)</f>
       </c>
       <c r="AL22" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="AM22" s="24"/>
       <c r="AN22" s="182" t="str">
         <f>=IFERROR(ROUND($AM$22/$AM$8,2),0)</f>
       </c>
       <c r="AP22" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="AQ22" s="24"/>
       <c r="AR22" s="182" t="str">
         <f>=IFERROR(ROUND($AQ$22/$AQ$8,2),0)</f>
       </c>
       <c r="AT22" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="AU22" s="24"/>
       <c r="AV22" s="182" t="str">
         <f>=IFERROR(ROUND($AU$22/$AU$8,2),0)</f>
       </c>
       <c r="AX22" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="AY22" s="24"/>
       <c r="AZ22" s="182" t="str">
         <f>=IFERROR(ROUND($AY$22/$AY$8,2),0)</f>
       </c>
       <c r="BB22" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="BC22" s="24"/>
       <c r="BD22" s="182" t="str">
         <f>=IFERROR(ROUND($BC$22/$BC$8,2),0)</f>
       </c>
       <c r="BF22" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="BG22" s="24"/>
       <c r="BH22" s="182" t="str">
         <f>=IFERROR(ROUND($BG$22/$BG$8,2),0)</f>
       </c>
       <c r="BJ22" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="BK22" s="24"/>
       <c r="BL22" s="182" t="str">
         <f>=IFERROR(ROUND($BK$22/$BK$8,2),0)</f>
       </c>
       <c r="BN22" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="BO22" s="24"/>
       <c r="BP22" s="182" t="str">
         <f>=IFERROR(ROUND($BO$22/$BO$8,2),0)</f>
       </c>
       <c r="BR22" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="BS22" s="24"/>
       <c r="BT22" s="182" t="str">
@@ -20920,7 +20914,7 @@
     </row>
     <row r="23">
       <c r="B23" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="C23" s="188" t="str">
         <f>=ROUND(IF(Saldovortrag_LW="",0,Saldovortrag_LW),2)</f>
@@ -20929,7 +20923,7 @@
         <f>=IFERROR(ROUND($C$23/$C$8,2),0)</f>
       </c>
       <c r="F23" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="G23" s="188" t="str">
         <f>=ROUND(IFERROR(FB_SaldoLC_1,0),2)</f>
@@ -20938,7 +20932,7 @@
         <f>=IFERROR(ROUND($G$23/$G$8,2),0)</f>
       </c>
       <c r="J23" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="K23" s="188" t="str">
         <f>=ROUND(IFERROR(FB_SaldoLC_2,0),2)</f>
@@ -20947,7 +20941,7 @@
         <f>=IFERROR(ROUND($K$23/$K$8,2),0)</f>
       </c>
       <c r="N23" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="O23" s="188" t="str">
         <f>=ROUND(IFERROR(FB_SaldoLC_3,0),2)</f>
@@ -20956,7 +20950,7 @@
         <f>=IFERROR(ROUND($O$23/$O$8,2),0)</f>
       </c>
       <c r="R23" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="S23" s="188" t="str">
         <f>=ROUND(IFERROR(FB_SaldoLC_4,0),2)</f>
@@ -20965,7 +20959,7 @@
         <f>=IFERROR(ROUND($S$23/$S$8,2),0)</f>
       </c>
       <c r="V23" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="W23" s="188" t="str">
         <f>=ROUND(IFERROR(FB_SaldoLC_5,0),2)</f>
@@ -20974,7 +20968,7 @@
         <f>=IFERROR(ROUND($W$23/$W$8,2),0)</f>
       </c>
       <c r="Z23" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="AA23" s="188" t="str">
         <f>=ROUND(IFERROR(FB_SaldoLC_6,0),2)</f>
@@ -20983,7 +20977,7 @@
         <f>=IFERROR(ROUND($AA$23/$AA$8,2),0)</f>
       </c>
       <c r="AD23" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="AE23" s="188" t="str">
         <f>=ROUND(IFERROR(FB_SaldoLC_7,0),2)</f>
@@ -20992,7 +20986,7 @@
         <f>=IFERROR(ROUND($AE$23/$AE$8,2),0)</f>
       </c>
       <c r="AH23" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="AI23" s="188" t="str">
         <f>=ROUND(IFERROR(FB_SaldoLC_8,0),2)</f>
@@ -21001,7 +20995,7 @@
         <f>=IFERROR(ROUND($AI$23/$AI$8,2),0)</f>
       </c>
       <c r="AL23" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="AM23" s="188" t="str">
         <f>=ROUND(IFERROR(FB_SaldoLC_9,0),2)</f>
@@ -21010,7 +21004,7 @@
         <f>=IFERROR(ROUND($AM$23/$AM$8,2),0)</f>
       </c>
       <c r="AP23" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="AQ23" s="188" t="str">
         <f>=ROUND(IFERROR(FB_SaldoLC_10,0),2)</f>
@@ -21019,7 +21013,7 @@
         <f>=IFERROR(ROUND($AQ$23/$AQ$8,2),0)</f>
       </c>
       <c r="AT23" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="AU23" s="188" t="str">
         <f>=ROUND(IFERROR(FB_SaldoLC_11,0),2)</f>
@@ -21028,7 +21022,7 @@
         <f>=IFERROR(ROUND($AU$23/$AU$8,2),0)</f>
       </c>
       <c r="AX23" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="AY23" s="188" t="str">
         <f>=ROUND(IFERROR(FB_SaldoLC_12,0),2)</f>
@@ -21037,7 +21031,7 @@
         <f>=IFERROR(ROUND($AY$23/$AY$8,2),0)</f>
       </c>
       <c r="BB23" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="BC23" s="188" t="str">
         <f>=ROUND(IFERROR(FB_SaldoLC_13,0),2)</f>
@@ -21046,7 +21040,7 @@
         <f>=IFERROR(ROUND($BC$23/$BC$8,2),0)</f>
       </c>
       <c r="BF23" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="BG23" s="188" t="str">
         <f>=ROUND(IFERROR(FB_SaldoLC_14,0),2)</f>
@@ -21055,7 +21049,7 @@
         <f>=IFERROR(ROUND($BG$23/$BG$8,2),0)</f>
       </c>
       <c r="BJ23" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="BK23" s="188" t="str">
         <f>=ROUND(IFERROR(FB_SaldoLC_15,0),2)</f>
@@ -21064,7 +21058,7 @@
         <f>=IFERROR(ROUND($BK$23/$BK$8,2),0)</f>
       </c>
       <c r="BN23" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="BO23" s="188" t="str">
         <f>=ROUND(IFERROR(FB_SaldoLC_16,0),2)</f>
@@ -21073,7 +21067,7 @@
         <f>=IFERROR(ROUND($BO$23/$BO$8,2),0)</f>
       </c>
       <c r="BR23" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="BS23" s="188" t="str">
         <f>=ROUND(IFERROR(FB_SaldoLC_17,0),2)</f>
@@ -21084,7 +21078,7 @@
     </row>
     <row r="25">
       <c r="B25" s="189" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="C25" s="190" t="str">
         <f>=IFERROR(ROUND($C$18-$C$21-$C$22-$C$23,2),0)</f>
@@ -21093,7 +21087,7 @@
         <f>=IFERROR(ROUND($D$18-$D$21-$D$22-$D$23,2),0)</f>
       </c>
       <c r="F25" s="189" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="G25" s="190" t="str">
         <f>=IFERROR(ROUND($G$18-$G$21-$G$22-$G$23,2),0)</f>
@@ -21102,7 +21096,7 @@
         <f>=IFERROR(ROUND($H$18-$H$21-$H$22-$H$23,2),0)</f>
       </c>
       <c r="J25" s="189" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="K25" s="190" t="str">
         <f>=IFERROR(ROUND($K$18-$K$21-$K$22-$K$23,2),0)</f>
@@ -21111,7 +21105,7 @@
         <f>=IFERROR(ROUND($L$18-$L$21-$L$22-$L$23,2),0)</f>
       </c>
       <c r="N25" s="189" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="O25" s="190" t="str">
         <f>=IFERROR(ROUND($O$18-$O$21-$O$22-$O$23,2),0)</f>
@@ -21120,7 +21114,7 @@
         <f>=IFERROR(ROUND($P$18-$P$21-$P$22-$P$23,2),0)</f>
       </c>
       <c r="R25" s="189" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="S25" s="190" t="str">
         <f>=IFERROR(ROUND($S$18-$S$21-$S$22-$S$23,2),0)</f>
@@ -21129,7 +21123,7 @@
         <f>=IFERROR(ROUND($T$18-$T$21-$T$22-$T$23,2),0)</f>
       </c>
       <c r="V25" s="189" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="W25" s="190" t="str">
         <f>=IFERROR(ROUND($W$18-$W$21-$W$22-$W$23,2),0)</f>
@@ -21138,7 +21132,7 @@
         <f>=IFERROR(ROUND($X$18-$X$21-$X$22-$X$23,2),0)</f>
       </c>
       <c r="Z25" s="189" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="AA25" s="190" t="str">
         <f>=IFERROR(ROUND($AA$18-$AA$21-$AA$22-$AA$23,2),0)</f>
@@ -21147,7 +21141,7 @@
         <f>=IFERROR(ROUND($AB$18-$AB$21-$AB$22-$AB$23,2),0)</f>
       </c>
       <c r="AD25" s="189" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="AE25" s="190" t="str">
         <f>=IFERROR(ROUND($AE$18-$AE$21-$AE$22-$AE$23,2),0)</f>
@@ -21156,7 +21150,7 @@
         <f>=IFERROR(ROUND($AF$18-$AF$21-$AF$22-$AF$23,2),0)</f>
       </c>
       <c r="AH25" s="189" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="AI25" s="190" t="str">
         <f>=IFERROR(ROUND($AI$18-$AI$21-$AI$22-$AI$23,2),0)</f>
@@ -21165,7 +21159,7 @@
         <f>=IFERROR(ROUND($AJ$18-$AJ$21-$AJ$22-$AJ$23,2),0)</f>
       </c>
       <c r="AL25" s="189" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="AM25" s="190" t="str">
         <f>=IFERROR(ROUND($AM$18-$AM$21-$AM$22-$AM$23,2),0)</f>
@@ -21174,7 +21168,7 @@
         <f>=IFERROR(ROUND($AN$18-$AN$21-$AN$22-$AN$23,2),0)</f>
       </c>
       <c r="AP25" s="189" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="AQ25" s="190" t="str">
         <f>=IFERROR(ROUND($AQ$18-$AQ$21-$AQ$22-$AQ$23,2),0)</f>
@@ -21183,7 +21177,7 @@
         <f>=IFERROR(ROUND($AR$18-$AR$21-$AR$22-$AR$23,2),0)</f>
       </c>
       <c r="AT25" s="189" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="AU25" s="190" t="str">
         <f>=IFERROR(ROUND($AU$18-$AU$21-$AU$22-$AU$23,2),0)</f>
@@ -21192,7 +21186,7 @@
         <f>=IFERROR(ROUND($AV$18-$AV$21-$AV$22-$AV$23,2),0)</f>
       </c>
       <c r="AX25" s="189" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="AY25" s="190" t="str">
         <f>=IFERROR(ROUND($AY$18-$AY$21-$AY$22-$AY$23,2),0)</f>
@@ -21201,7 +21195,7 @@
         <f>=IFERROR(ROUND($AZ$18-$AZ$21-$AZ$22-$AZ$23,2),0)</f>
       </c>
       <c r="BB25" s="189" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="BC25" s="190" t="str">
         <f>=IFERROR(ROUND($BC$18-$BC$21-$BC$22-$BC$23,2),0)</f>
@@ -21210,7 +21204,7 @@
         <f>=IFERROR(ROUND($BD$18-$BD$21-$BD$22-$BD$23,2),0)</f>
       </c>
       <c r="BF25" s="189" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="BG25" s="190" t="str">
         <f>=IFERROR(ROUND($BG$18-$BG$21-$BG$22-$BG$23,2),0)</f>
@@ -21219,7 +21213,7 @@
         <f>=IFERROR(ROUND($BH$18-$BH$21-$BH$22-$BH$23,2),0)</f>
       </c>
       <c r="BJ25" s="189" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="BK25" s="190" t="str">
         <f>=IFERROR(ROUND($BK$18-$BK$21-$BK$22-$BK$23,2),0)</f>
@@ -21228,7 +21222,7 @@
         <f>=IFERROR(ROUND($BL$18-$BL$21-$BL$22-$BL$23,2),0)</f>
       </c>
       <c r="BN25" s="189" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="BO25" s="190" t="str">
         <f>=IFERROR(ROUND($BO$18-$BO$21-$BO$22-$BO$23,2),0)</f>
@@ -21237,7 +21231,7 @@
         <f>=IFERROR(ROUND($BP$18-$BP$21-$BP$22-$BP$23,2),0)</f>
       </c>
       <c r="BR25" s="189" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="BS25" s="190" t="str">
         <f>=IFERROR(ROUND($BS$18-$BS$21-$BS$22-$BS$23,2),0)</f>
@@ -21437,7 +21431,7 @@
   <sheetData>
     <row r="2" ht="30" customHeight="true">
       <c r="B2" s="192" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C2" s="192"/>
       <c r="D2" s="192"/>
@@ -21450,7 +21444,7 @@
     </row>
     <row r="3" ht="18" customHeight="true">
       <c r="B3" s="193" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="C3" s="193"/>
       <c r="D3" s="193"/>
@@ -21463,7 +21457,7 @@
     </row>
     <row r="5" ht="22" customHeight="true">
       <c r="B5" s="194" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="C5" s="194"/>
       <c r="D5" s="194"/>
@@ -21484,7 +21478,7 @@
     </row>
     <row r="6">
       <c r="B6" s="195" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="C6" s="195"/>
       <c r="D6" s="195"/>
@@ -21513,7 +21507,7 @@
     </row>
     <row r="8" ht="22" customHeight="true">
       <c r="C8" s="202" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="D8" s="203"/>
       <c r="E8" s="203"/>
@@ -21529,11 +21523,11 @@
     </row>
     <row r="9">
       <c r="C9" s="205" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="D9" s="197"/>
       <c r="E9" s="63" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="F9" s="63"/>
       <c r="G9" s="206"/>
@@ -21547,7 +21541,7 @@
     </row>
     <row r="10">
       <c r="C10" s="205" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="D10" s="197"/>
       <c r="E10" s="198" t="str">
@@ -21557,7 +21551,7 @@
       <c r="F10" s="198"/>
       <c r="G10" s="207"/>
       <c r="L10" s="315" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="M10" s="310" t="str">
         <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$C$8,'IV. MA'!$G$8,'IV. MA'!$K$8,'IV. MA'!$O$8,'IV. MA'!$S$8,'IV. MA'!$W$8,'IV. MA'!$AA$8,'IV. MA'!$AE$8,'IV. MA'!$AI$8,'IV. MA'!$AM$8,'IV. MA'!$AQ$8,'IV. MA'!$AU$8,'IV. MA'!$AY$8,'IV. MA'!$BC$8,'IV. MA'!$BG$8,'IV. MA'!$BK$8,'IV. MA'!$BO$8,'IV. MA'!$BS$8),"")</f>
@@ -21566,7 +21560,7 @@
     </row>
     <row r="11">
       <c r="C11" s="205" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="D11" s="197"/>
       <c r="E11" s="198" t="str">
@@ -21579,7 +21573,7 @@
     </row>
     <row r="12">
       <c r="C12" s="209" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="D12" s="199"/>
       <c r="E12" s="199"/>
@@ -21589,10 +21583,10 @@
         <v>202</v>
       </c>
       <c r="M12" s="180" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="N12" s="321" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="13">
@@ -21740,7 +21734,7 @@
     </row>
     <row r="20" ht="22" customHeight="true">
       <c r="B20" s="18" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="C20" s="18"/>
       <c r="D20" s="18"/>
@@ -21762,7 +21756,7 @@
     </row>
     <row r="21">
       <c r="L21" s="322" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="M21" s="243" t="str">
         <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$C$18,'IV. MA'!$G$18,'IV. MA'!$K$18,'IV. MA'!$O$18,'IV. MA'!$S$18,'IV. MA'!$W$18,'IV. MA'!$AA$18,'IV. MA'!$AE$18,'IV. MA'!$AI$18,'IV. MA'!$AM$18,'IV. MA'!$AQ$18,'IV. MA'!$AU$18,'IV. MA'!$AY$18,'IV. MA'!$BC$18,'IV. MA'!$BG$18,'IV. MA'!$BK$18,'IV. MA'!$BO$18,'IV. MA'!$BS$18),"")</f>
@@ -21773,14 +21767,14 @@
     </row>
     <row r="22">
       <c r="B22" s="223" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="C22" s="224"/>
       <c r="D22" s="225" t="str">
         <f>=IFERROR(ROUND(KMW_Mittel_EUR,2),0)</f>
       </c>
       <c r="F22" s="230" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="G22" s="231"/>
       <c r="H22" s="231"/>
@@ -21790,24 +21784,24 @@
     </row>
     <row r="23">
       <c r="B23" s="205" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="C23" s="197"/>
       <c r="D23" s="226" t="str">
         <f>=IFERROR(ROUND(Kosten_Reserve_EUR,2),0)</f>
       </c>
       <c r="F23" s="233" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="G23" s="197" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="H23" s="197"/>
       <c r="I23" s="234" t="str">
         <f>=IFERROR(ROUND(Saldovortrag_EUR,2),0)</f>
       </c>
       <c r="L23" s="143" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="M23" s="116" t="str">
         <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$C$20,'IV. MA'!$G$20,'IV. MA'!$K$20,'IV. MA'!$O$20,'IV. MA'!$S$20,'IV. MA'!$W$20,'IV. MA'!$AA$20,'IV. MA'!$AE$20,'IV. MA'!$AI$20,'IV. MA'!$AM$20,'IV. MA'!$AQ$20,'IV. MA'!$AU$20,'IV. MA'!$AY$20,'IV. MA'!$BC$20,'IV. MA'!$BG$20,'IV. MA'!$BK$20,'IV. MA'!$BO$20,'IV. MA'!$BS$20),"")</f>
@@ -21825,10 +21819,10 @@
         <f>=IF(Reserve_Freigabe="Ja",ROUND($D$22,2),ROUND($D$22-$D$23,2))</f>
       </c>
       <c r="F24" s="233" t="s">
+        <v>352</v>
+      </c>
+      <c r="G24" s="197" t="s">
         <v>354</v>
-      </c>
-      <c r="G24" s="197" t="s">
-        <v>356</v>
       </c>
       <c r="H24" s="197"/>
       <c r="I24" s="234" t="str">
@@ -21836,7 +21830,7 @@
         <v>0</v>
       </c>
       <c r="L24" s="143" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="M24" s="116" t="str">
         <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$C$21,'IV. MA'!$G$21,'IV. MA'!$K$21,'IV. MA'!$O$21,'IV. MA'!$S$21,'IV. MA'!$W$21,'IV. MA'!$AA$21,'IV. MA'!$AE$21,'IV. MA'!$AI$21,'IV. MA'!$AM$21,'IV. MA'!$AQ$21,'IV. MA'!$AU$21,'IV. MA'!$AY$21,'IV. MA'!$BC$21,'IV. MA'!$BG$21,'IV. MA'!$BK$21,'IV. MA'!$BO$21,'IV. MA'!$BS$21),"")</f>
@@ -21847,17 +21841,17 @@
     </row>
     <row r="25">
       <c r="B25" s="205" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="C25" s="197"/>
       <c r="D25" s="226" t="str">
         <f>=IFERROR(ROUND(SUBTOTAL(109,TblKMWMittel[Betrag]),2),0)</f>
       </c>
       <c r="F25" s="233" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="G25" s="197" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="H25" s="197"/>
       <c r="I25" s="234" t="str">
@@ -21865,7 +21859,7 @@
         <v>0</v>
       </c>
       <c r="L25" s="143" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="M25" s="116" t="str">
         <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$C$22,'IV. MA'!$G$22,'IV. MA'!$K$22,'IV. MA'!$O$22,'IV. MA'!$S$22,'IV. MA'!$W$22,'IV. MA'!$AA$22,'IV. MA'!$AE$22,'IV. MA'!$AI$22,'IV. MA'!$AM$22,'IV. MA'!$AQ$22,'IV. MA'!$AU$22,'IV. MA'!$AY$22,'IV. MA'!$BC$22,'IV. MA'!$BG$22,'IV. MA'!$BK$22,'IV. MA'!$BO$22,'IV. MA'!$BS$22),"")</f>
@@ -21876,7 +21870,7 @@
     </row>
     <row r="26">
       <c r="B26" s="227" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="C26" s="228"/>
       <c r="D26" s="229" t="str">
@@ -21884,7 +21878,7 @@
       </c>
       <c r="F26" s="47"/>
       <c r="G26" s="218" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="H26" s="218"/>
       <c r="I26" s="235" t="str">
@@ -21903,7 +21897,7 @@
     <row r="27">
       <c r="F27" s="236"/>
       <c r="G27" s="228" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="H27" s="228"/>
       <c r="I27" s="229" t="str">
@@ -21914,7 +21908,7 @@
     </row>
     <row r="28">
       <c r="L28" s="323" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="M28" s="324" t="str">
         <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$C$25,'IV. MA'!$G$25,'IV. MA'!$K$25,'IV. MA'!$O$25,'IV. MA'!$S$25,'IV. MA'!$W$25,'IV. MA'!$AA$25,'IV. MA'!$AE$25,'IV. MA'!$AI$25,'IV. MA'!$AM$25,'IV. MA'!$AQ$25,'IV. MA'!$AU$25,'IV. MA'!$AY$25,'IV. MA'!$BC$25,'IV. MA'!$BG$25,'IV. MA'!$BK$25,'IV. MA'!$BO$25,'IV. MA'!$BS$25),"")</f>
@@ -21925,14 +21919,14 @@
     </row>
     <row r="29">
       <c r="B29" s="223" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="C29" s="224"/>
       <c r="D29" s="225" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"KMW-Mittel",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,E11),2),0)</f>
       </c>
       <c r="F29" s="223" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="G29" s="224"/>
       <c r="H29" s="224"/>
@@ -21942,14 +21936,14 @@
     </row>
     <row r="30">
       <c r="B30" s="227" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="C30" s="228"/>
       <c r="D30" s="229" t="str">
         <f>=ROUND($D$26-MAX(0,$D$29),2)</f>
       </c>
       <c r="F30" s="227" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="G30" s="228"/>
       <c r="H30" s="228"/>
@@ -21959,12 +21953,12 @@
     </row>
     <row r="32">
       <c r="B32" s="223" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="C32" s="224"/>
       <c r="D32" s="237"/>
       <c r="F32" s="223" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="G32" s="224"/>
       <c r="H32" s="224"/>
@@ -21972,14 +21966,14 @@
     </row>
     <row r="33">
       <c r="B33" s="227" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="C33" s="228"/>
       <c r="D33" s="229" t="str">
         <f>=ROUND($D$26-MAX(0,$D$29)-MAX(0,$D$32),2)</f>
       </c>
       <c r="F33" s="227" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="G33" s="228"/>
       <c r="H33" s="228"/>
@@ -21989,7 +21983,7 @@
     </row>
     <row r="36" ht="22" customHeight="true">
       <c r="B36" s="18" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="C36" s="18"/>
       <c r="D36" s="18"/>
@@ -22005,18 +21999,18 @@
         <v>158</v>
       </c>
       <c r="C38" s="247" t="s">
+        <v>363</v>
+      </c>
+      <c r="D38" s="247" t="s">
+        <v>364</v>
+      </c>
+      <c r="E38" s="248" t="s">
         <v>365</v>
-      </c>
-      <c r="D38" s="247" t="s">
-        <v>366</v>
-      </c>
-      <c r="E38" s="248" t="s">
-        <v>367</v>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="205" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="C39" s="239" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BF$1:$BF$18,'Daten'!$BB$1:$BB$18,E10,'Daten'!$BD$1:$BD$18,"&lt;="&amp;E11,'Daten'!$BD$1:$BD$18,"&gt;=1"),2),0)</f>
@@ -22028,7 +22022,7 @@
     </row>
     <row r="40">
       <c r="B40" s="205" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C40" s="239" t="str">
         <f>=IFERROR(ROUND(SUBTOTAL(109,TblBudgetAusgaben[Jahr 1]),2),0)</f>
@@ -22042,7 +22036,7 @@
     </row>
     <row r="41">
       <c r="B41" s="205" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="C41" s="239" t="str">
         <f>=IFERROR(ROUND(SUBTOTAL(109,TblBudgetAusgaben[Jahr 2]),2),0)</f>
@@ -22056,7 +22050,7 @@
     </row>
     <row r="42">
       <c r="B42" s="205" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="C42" s="239" t="str">
         <f>=IFERROR(ROUND(SUBTOTAL(109,TblBudgetAusgaben[Jahr 3]),2),0)</f>
@@ -22070,7 +22064,7 @@
     </row>
     <row r="43">
       <c r="B43" s="205" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="C43" s="242" t="str">
         <f>=$D$40+$D$41+$D$42</f>
@@ -22080,7 +22074,7 @@
     </row>
     <row r="44">
       <c r="B44" s="205" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="C44" s="242" t="str">
         <f>=IFERROR(CHOOSE(IFERROR(SUMPRODUCT('Daten'!$BA$1:$BA$18,('Daten'!$BB$1:$BB$18=E10)*('Daten'!$BD$1:$BD$18=E11)),0),'IV. MA'!$C$7,'IV. MA'!$G$7,'IV. MA'!$K$7,'IV. MA'!$O$7,'IV. MA'!$S$7,'IV. MA'!$W$7,'IV. MA'!$AA$7,'IV. MA'!$AE$7,'IV. MA'!$AI$7,'IV. MA'!$AM$7,'IV. MA'!$AQ$7,'IV. MA'!$AU$7,'IV. MA'!$AY$7,'IV. MA'!$BC$7,'IV. MA'!$BG$7,'IV. MA'!$BK$7,'IV. MA'!$BO$7,'IV. MA'!$BS$7),0)</f>
@@ -22090,7 +22084,7 @@
     </row>
     <row r="45">
       <c r="B45" s="251" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="C45" s="243" t="str">
         <f>=IFERROR(ROUND($C$40*$D$40/12+$C$41*$D$41/12+$C$42*$D$42/12,2),0)</f>
@@ -22102,7 +22096,7 @@
     </row>
     <row r="46">
       <c r="B46" s="251" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="C46" s="244" t="str">
         <f>=IF($C$39&lt;=$C$45,"OK","ÜBERSCHRITTEN")</f>
@@ -22114,7 +22108,7 @@
     </row>
     <row r="47">
       <c r="B47" s="205" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C47" s="239" t="str">
         <f>=ROUND(MAX(0,$C$39-$C$45),2)</f>
@@ -22126,7 +22120,7 @@
     </row>
     <row r="48">
       <c r="B48" s="253" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="C48" s="254" t="str">
         <f>=IFERROR($C$39/$C$45,0)</f>
@@ -22138,7 +22132,7 @@
     </row>
     <row r="50" ht="22" customHeight="true">
       <c r="B50" s="18" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="C50" s="18"/>
       <c r="D50" s="18"/>
@@ -22151,31 +22145,31 @@
     </row>
     <row r="52" ht="28" customHeight="true">
       <c r="B52" s="263" t="s">
+        <v>377</v>
+      </c>
+      <c r="C52" s="264" t="s">
+        <v>378</v>
+      </c>
+      <c r="D52" s="264" t="s">
         <v>379</v>
       </c>
-      <c r="C52" s="264" t="s">
+      <c r="E52" s="264" t="s">
         <v>380</v>
       </c>
-      <c r="D52" s="264" t="s">
+      <c r="F52" s="264" t="s">
         <v>381</v>
       </c>
-      <c r="E52" s="264" t="s">
+      <c r="G52" s="264" t="s">
         <v>382</v>
       </c>
-      <c r="F52" s="264" t="s">
+      <c r="H52" s="264" t="s">
         <v>383</v>
       </c>
-      <c r="G52" s="264" t="s">
+      <c r="I52" s="264" t="s">
         <v>384</v>
       </c>
-      <c r="H52" s="264" t="s">
+      <c r="J52" s="265" t="s">
         <v>385</v>
-      </c>
-      <c r="I52" s="264" t="s">
-        <v>386</v>
-      </c>
-      <c r="J52" s="265" t="s">
-        <v>387</v>
       </c>
     </row>
     <row r="53">
@@ -22325,7 +22319,7 @@
     </row>
     <row r="59" ht="22" customHeight="true">
       <c r="B59" s="18" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="C59" s="18"/>
       <c r="D59" s="18"/>
@@ -22338,31 +22332,31 @@
     </row>
     <row r="61" ht="28" customHeight="true">
       <c r="B61" s="263" t="s">
+        <v>377</v>
+      </c>
+      <c r="C61" s="264" t="s">
+        <v>378</v>
+      </c>
+      <c r="D61" s="264" t="s">
         <v>379</v>
       </c>
-      <c r="C61" s="264" t="s">
+      <c r="E61" s="264" t="s">
         <v>380</v>
       </c>
-      <c r="D61" s="264" t="s">
+      <c r="F61" s="264" t="s">
         <v>381</v>
       </c>
-      <c r="E61" s="264" t="s">
+      <c r="G61" s="264" t="s">
         <v>382</v>
       </c>
-      <c r="F61" s="264" t="s">
+      <c r="H61" s="264" t="s">
         <v>383</v>
       </c>
-      <c r="G61" s="264" t="s">
+      <c r="I61" s="264" t="s">
         <v>384</v>
       </c>
-      <c r="H61" s="264" t="s">
+      <c r="J61" s="265" t="s">
         <v>385</v>
-      </c>
-      <c r="I61" s="264" t="s">
-        <v>386</v>
-      </c>
-      <c r="J61" s="265" t="s">
-        <v>387</v>
       </c>
     </row>
     <row r="62">
@@ -22628,7 +22622,7 @@
     </row>
     <row r="76" ht="22" customHeight="true">
       <c r="B76" s="194" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="C76" s="194"/>
       <c r="D76" s="194"/>
@@ -22648,7 +22642,7 @@
     </row>
     <row r="77">
       <c r="B77" s="195" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="C77" s="195"/>
       <c r="D77" s="195"/>
@@ -22681,7 +22675,7 @@
     </row>
     <row r="79" ht="22" customHeight="true">
       <c r="C79" s="202" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="D79" s="203"/>
       <c r="E79" s="203"/>
@@ -22699,11 +22693,11 @@
     </row>
     <row r="80">
       <c r="C80" s="205" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="D80" s="197"/>
       <c r="E80" s="63" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="F80" s="63"/>
       <c r="G80" s="206"/>
@@ -22719,7 +22713,7 @@
     </row>
     <row r="81">
       <c r="C81" s="253" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="D81" s="286"/>
       <c r="E81" s="287" t="str">
@@ -22743,7 +22737,7 @@
     </row>
     <row r="83" ht="22" customHeight="true">
       <c r="B83" s="18" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="C83" s="18"/>
       <c r="D83" s="18"/>
@@ -22780,14 +22774,14 @@
     </row>
     <row r="85">
       <c r="B85" s="223" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="C85" s="224"/>
       <c r="D85" s="225" t="str">
         <f>=IFERROR(ROUND(KMW_Mittel_EUR,2),0)</f>
       </c>
       <c r="F85" s="230" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="G85" s="231"/>
       <c r="H85" s="231"/>
@@ -22810,17 +22804,17 @@
     </row>
     <row r="86">
       <c r="B86" s="205" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="C86" s="197"/>
       <c r="D86" s="226" t="str">
         <f>=IFERROR(ROUND(Kosten_Reserve_EUR,2),0)</f>
       </c>
       <c r="F86" s="233" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="G86" s="197" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="H86" s="197"/>
       <c r="I86" s="234" t="str">
@@ -22851,10 +22845,10 @@
         <f>=IF(Reserve_Freigabe="Ja",ROUND($D$85,2),ROUND($D$85-$D$86,2))</f>
       </c>
       <c r="F87" s="233" t="s">
+        <v>352</v>
+      </c>
+      <c r="G87" s="197" t="s">
         <v>354</v>
-      </c>
-      <c r="G87" s="197" t="s">
-        <v>356</v>
       </c>
       <c r="H87" s="197"/>
       <c r="I87" s="234" t="str">
@@ -22879,7 +22873,7 @@
     </row>
     <row r="88">
       <c r="B88" s="205" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="C88" s="197"/>
       <c r="D88" s="226" t="str">
@@ -22887,7 +22881,7 @@
       </c>
       <c r="F88" s="47"/>
       <c r="G88" s="218" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="H88" s="218"/>
       <c r="I88" s="235" t="str">
@@ -22911,7 +22905,7 @@
     </row>
     <row r="89">
       <c r="B89" s="227" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="C89" s="228"/>
       <c r="D89" s="229" t="str">
@@ -22919,7 +22913,7 @@
       </c>
       <c r="F89" s="236"/>
       <c r="G89" s="228" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="H89" s="228"/>
       <c r="I89" s="229" t="str">
@@ -22986,7 +22980,7 @@
     </row>
     <row r="93" ht="22" customHeight="true">
       <c r="B93" s="18" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="C93" s="18"/>
       <c r="D93" s="18"/>
@@ -23031,31 +23025,31 @@
     </row>
     <row r="95" ht="28" customHeight="true">
       <c r="B95" s="263" t="s">
+        <v>377</v>
+      </c>
+      <c r="C95" s="264" t="s">
+        <v>393</v>
+      </c>
+      <c r="D95" s="264" t="s">
         <v>379</v>
       </c>
-      <c r="C95" s="264" t="s">
-        <v>395</v>
-      </c>
-      <c r="D95" s="264" t="s">
+      <c r="E95" s="264" t="s">
+        <v>380</v>
+      </c>
+      <c r="F95" s="264" t="s">
         <v>381</v>
       </c>
-      <c r="E95" s="264" t="s">
-        <v>382</v>
-      </c>
-      <c r="F95" s="264" t="s">
+      <c r="G95" s="264" t="s">
+        <v>394</v>
+      </c>
+      <c r="H95" s="264" t="s">
         <v>383</v>
       </c>
-      <c r="G95" s="264" t="s">
-        <v>396</v>
-      </c>
-      <c r="H95" s="264" t="s">
+      <c r="I95" s="264" t="s">
+        <v>384</v>
+      </c>
+      <c r="J95" s="265" t="s">
         <v>385</v>
-      </c>
-      <c r="I95" s="264" t="s">
-        <v>386</v>
-      </c>
-      <c r="J95" s="265" t="s">
-        <v>387</v>
       </c>
       <c r="L95" s="143" t="str">
         <f>=IFERROR(CHOOSE(E81,'III. Finanzberichte'!$B$21,'III. Finanzberichte'!$I$21,'III. Finanzberichte'!$P$21,'III. Finanzberichte'!$W$21,'III. Finanzberichte'!$AD$21,'III. Finanzberichte'!$AK$21,'III. Finanzberichte'!$AR$21,'III. Finanzberichte'!$AY$21,'III. Finanzberichte'!$BF$21,'III. Finanzberichte'!$BM$21,'III. Finanzberichte'!$BT$21,'III. Finanzberichte'!$CA$21,'III. Finanzberichte'!$CH$21,'III. Finanzberichte'!$CO$21,'III. Finanzberichte'!$CV$21,'III. Finanzberichte'!$DC$21,'III. Finanzberichte'!$DJ$21,'III. Finanzberichte'!$DQ$21),"")</f>
@@ -23312,7 +23306,7 @@
     </row>
     <row r="102" ht="22" customHeight="true">
       <c r="B102" s="18" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="C102" s="18"/>
       <c r="D102" s="18"/>
@@ -23357,31 +23351,31 @@
     </row>
     <row r="104" ht="28" customHeight="true">
       <c r="B104" s="263" t="s">
+        <v>377</v>
+      </c>
+      <c r="C104" s="264" t="s">
+        <v>393</v>
+      </c>
+      <c r="D104" s="264" t="s">
         <v>379</v>
       </c>
-      <c r="C104" s="264" t="s">
-        <v>395</v>
-      </c>
-      <c r="D104" s="264" t="s">
+      <c r="E104" s="264" t="s">
+        <v>380</v>
+      </c>
+      <c r="F104" s="264" t="s">
         <v>381</v>
       </c>
-      <c r="E104" s="264" t="s">
-        <v>382</v>
-      </c>
-      <c r="F104" s="264" t="s">
+      <c r="G104" s="264" t="s">
+        <v>394</v>
+      </c>
+      <c r="H104" s="264" t="s">
         <v>383</v>
       </c>
-      <c r="G104" s="264" t="s">
-        <v>396</v>
-      </c>
-      <c r="H104" s="264" t="s">
+      <c r="I104" s="264" t="s">
+        <v>384</v>
+      </c>
+      <c r="J104" s="265" t="s">
         <v>385</v>
-      </c>
-      <c r="I104" s="264" t="s">
-        <v>386</v>
-      </c>
-      <c r="J104" s="265" t="s">
-        <v>387</v>
       </c>
       <c r="L104" s="47"/>
       <c r="P104" s="48"/>
@@ -24004,16 +23998,16 @@
         <v>247</v>
       </c>
       <c r="C1" s="351" t="s">
+        <v>398</v>
+      </c>
+      <c r="I1" s="351" t="s">
+        <v>399</v>
+      </c>
+      <c r="O1" s="351" t="s">
         <v>400</v>
       </c>
-      <c r="I1" s="351" t="s">
+      <c r="U1" s="351" t="s">
         <v>401</v>
-      </c>
-      <c r="O1" s="351" t="s">
-        <v>402</v>
-      </c>
-      <c r="U1" s="351" t="s">
-        <v>403</v>
       </c>
       <c r="BA1">
         <v>1</v>

</xml_diff>

<commit_message>
feat: add conditional formatting for active budget areas
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_befuellt.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_befuellt.xlsx
@@ -3306,7 +3306,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="18">
+  <dxfs count="17">
     <dxf>
       <font>
         <name val="Segoe UI"/>
@@ -3354,35 +3354,6 @@
           <color rgb="FF808080"/>
         </top>
         <bottom style="medium">
-          <color rgb="FF808080"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Segoe UI"/>
-        <family val="2"/>
-        <b val="1"/>
-        <color rgb="FFFFFFFF"/>
-        <sz val="9"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FF3C3C3C"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center"/>
-      <border>
-        <left style="thin">
-          <color rgb="FF808080"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF808080"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF808080"/>
-        </top>
-        <bottom style="thin">
           <color rgb="FF808080"/>
         </bottom>
       </border>
@@ -6760,63 +6731,58 @@
       <formula>$K$5="Ja"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K8">
+  <conditionalFormatting sqref="K9:M12">
     <cfRule type="expression" dxfId="3" priority="2">
       <formula>$K$5="Ja"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K9:M12">
+  <conditionalFormatting sqref="E32">
     <cfRule type="expression" dxfId="4" priority="3">
-      <formula>$K$5="Ja"</formula>
+      <formula>$E$32="OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E32">
     <cfRule type="expression" dxfId="5" priority="4">
-      <formula>$E$32="OK"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E32">
-    <cfRule type="expression" dxfId="6" priority="5">
       <formula>$E$32&lt;&gt;"OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E33">
-    <cfRule type="expression" dxfId="5" priority="6">
+    <cfRule type="expression" dxfId="4" priority="5">
       <formula>$E$33="OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E33">
-    <cfRule type="expression" dxfId="6" priority="7">
+    <cfRule type="expression" dxfId="5" priority="6">
       <formula>$E$33&lt;&gt;"OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E34">
-    <cfRule type="expression" dxfId="5" priority="8">
+    <cfRule type="expression" dxfId="4" priority="7">
       <formula>$E$34="OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E34">
-    <cfRule type="expression" dxfId="6" priority="9">
+    <cfRule type="expression" dxfId="5" priority="8">
       <formula>$E$34&lt;&gt;"OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E35">
-    <cfRule type="expression" dxfId="5" priority="10">
+    <cfRule type="expression" dxfId="4" priority="9">
       <formula>$E$35="OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E35">
-    <cfRule type="expression" dxfId="6" priority="11">
+    <cfRule type="expression" dxfId="5" priority="10">
       <formula>$E$35&lt;&gt;"OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E36">
-    <cfRule type="expression" dxfId="7" priority="12">
+    <cfRule type="expression" dxfId="6" priority="11">
       <formula>$E$36="OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E36">
-    <cfRule type="expression" dxfId="8" priority="13">
+    <cfRule type="expression" dxfId="7" priority="12">
       <formula>$E$36&lt;&gt;"OK"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -23749,202 +23715,202 @@
     <mergeCell ref="L91:P91"/>
   </mergeCells>
   <conditionalFormatting sqref="C13:D13">
-    <cfRule type="expression" dxfId="9" priority="1">
+    <cfRule type="expression" dxfId="8" priority="1">
       <formula>$C$13&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E13:F13">
-    <cfRule type="expression" dxfId="10" priority="2">
+    <cfRule type="expression" dxfId="9" priority="2">
       <formula>$C$13&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G13:G13">
-    <cfRule type="expression" dxfId="11" priority="3">
+    <cfRule type="expression" dxfId="10" priority="3">
       <formula>$C$13&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C14:D14">
-    <cfRule type="expression" dxfId="9" priority="4">
+    <cfRule type="expression" dxfId="8" priority="4">
       <formula>$C$14&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E14:F14">
-    <cfRule type="expression" dxfId="10" priority="5">
+    <cfRule type="expression" dxfId="9" priority="5">
       <formula>$C$14&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G14:G14">
-    <cfRule type="expression" dxfId="11" priority="6">
+    <cfRule type="expression" dxfId="10" priority="6">
       <formula>$C$14&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C15:D15">
-    <cfRule type="expression" dxfId="9" priority="7">
+    <cfRule type="expression" dxfId="8" priority="7">
       <formula>$C$15&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E15:F15">
-    <cfRule type="expression" dxfId="10" priority="8">
+    <cfRule type="expression" dxfId="9" priority="8">
       <formula>$C$15&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G15:G15">
-    <cfRule type="expression" dxfId="11" priority="9">
+    <cfRule type="expression" dxfId="10" priority="9">
       <formula>$C$15&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C16:D16">
-    <cfRule type="expression" dxfId="9" priority="10">
+    <cfRule type="expression" dxfId="8" priority="10">
       <formula>$C$16&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E16:F16">
-    <cfRule type="expression" dxfId="10" priority="11">
+    <cfRule type="expression" dxfId="9" priority="11">
       <formula>$C$16&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G16:G16">
-    <cfRule type="expression" dxfId="11" priority="12">
+    <cfRule type="expression" dxfId="10" priority="12">
       <formula>$C$16&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C17:D17">
-    <cfRule type="expression" dxfId="9" priority="13">
+    <cfRule type="expression" dxfId="8" priority="13">
       <formula>$C$17&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E17:F17">
-    <cfRule type="expression" dxfId="10" priority="14">
+    <cfRule type="expression" dxfId="9" priority="14">
       <formula>$C$17&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G17:G17">
-    <cfRule type="expression" dxfId="11" priority="15">
+    <cfRule type="expression" dxfId="10" priority="15">
       <formula>$C$17&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C18:D18">
-    <cfRule type="expression" dxfId="9" priority="16">
+    <cfRule type="expression" dxfId="8" priority="16">
       <formula>$C$18&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E18:F18">
-    <cfRule type="expression" dxfId="10" priority="17">
+    <cfRule type="expression" dxfId="9" priority="17">
       <formula>$C$18&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G18:G18">
-    <cfRule type="expression" dxfId="11" priority="18">
+    <cfRule type="expression" dxfId="10" priority="18">
       <formula>$C$18&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C46">
-    <cfRule type="expression" dxfId="12" priority="19">
+    <cfRule type="expression" dxfId="11" priority="19">
       <formula>$C$46="OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C46">
-    <cfRule type="expression" dxfId="13" priority="20">
+    <cfRule type="expression" dxfId="12" priority="20">
       <formula>$C$46&lt;&gt;"OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E46">
-    <cfRule type="expression" dxfId="12" priority="21">
+    <cfRule type="expression" dxfId="11" priority="21">
       <formula>$E$46="OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E46">
-    <cfRule type="expression" dxfId="13" priority="22">
+    <cfRule type="expression" dxfId="12" priority="22">
       <formula>$E$46&lt;&gt;"OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C47">
-    <cfRule type="expression" dxfId="14" priority="23">
+    <cfRule type="expression" dxfId="13" priority="23">
       <formula>$C$47&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E47">
-    <cfRule type="expression" dxfId="15" priority="24">
+    <cfRule type="expression" dxfId="14" priority="24">
       <formula>$E$47&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F53:F56">
-    <cfRule type="expression" dxfId="16" priority="25">
+    <cfRule type="expression" dxfId="15" priority="25">
       <formula>F53&gt;=0.2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F53:F56">
-    <cfRule type="expression" dxfId="17" priority="26">
+    <cfRule type="expression" dxfId="16" priority="26">
       <formula>AND(F53&gt;=0.1,F53&lt;0.2)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J53:J56">
-    <cfRule type="expression" dxfId="16" priority="27">
+    <cfRule type="expression" dxfId="15" priority="27">
       <formula>J53&gt;=0.2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J53:J56">
-    <cfRule type="expression" dxfId="17" priority="28">
+    <cfRule type="expression" dxfId="16" priority="28">
       <formula>AND(J53&gt;=0.1,J53&lt;0.2)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F62:F69">
-    <cfRule type="expression" dxfId="16" priority="29">
+    <cfRule type="expression" dxfId="15" priority="29">
       <formula>F62&gt;=0.2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F62:F69">
-    <cfRule type="expression" dxfId="17" priority="30">
+    <cfRule type="expression" dxfId="16" priority="30">
       <formula>AND(F62&gt;=0.1,F62&lt;0.2)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J62:J69">
-    <cfRule type="expression" dxfId="16" priority="31">
+    <cfRule type="expression" dxfId="15" priority="31">
       <formula>J62&gt;=0.2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J62:J69">
-    <cfRule type="expression" dxfId="17" priority="32">
+    <cfRule type="expression" dxfId="16" priority="32">
       <formula>AND(J62&gt;=0.1,J62&lt;0.2)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F96:F99">
-    <cfRule type="expression" dxfId="16" priority="33">
+    <cfRule type="expression" dxfId="15" priority="33">
       <formula>F96&gt;=0.2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F96:F99">
-    <cfRule type="expression" dxfId="17" priority="34">
+    <cfRule type="expression" dxfId="16" priority="34">
       <formula>AND(F96&gt;=0.1,F96&lt;0.2)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J96:J99">
-    <cfRule type="expression" dxfId="16" priority="35">
+    <cfRule type="expression" dxfId="15" priority="35">
       <formula>J96&gt;=0.2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J96:J99">
-    <cfRule type="expression" dxfId="17" priority="36">
+    <cfRule type="expression" dxfId="16" priority="36">
       <formula>AND(J96&gt;=0.1,J96&lt;0.2)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F105:F112">
-    <cfRule type="expression" dxfId="16" priority="37">
+    <cfRule type="expression" dxfId="15" priority="37">
       <formula>F105&gt;=0.2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F105:F112">
-    <cfRule type="expression" dxfId="17" priority="38">
+    <cfRule type="expression" dxfId="16" priority="38">
       <formula>AND(F105&gt;=0.1,F105&lt;0.2)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J105:J112">
-    <cfRule type="expression" dxfId="16" priority="39">
+    <cfRule type="expression" dxfId="15" priority="39">
       <formula>J105&gt;=0.2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J105:J112">
-    <cfRule type="expression" dxfId="17" priority="40">
+    <cfRule type="expression" dxfId="16" priority="40">
       <formula>AND(J105&gt;=0.1,J105&lt;0.2)</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
chore: update pre-check output files
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_befuellt.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_befuellt.xlsx
@@ -1374,7 +1374,7 @@
     <numFmt numFmtId="172" formatCode="0"/>
     <numFmt numFmtId="173" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="27">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1478,13 +1478,6 @@
       <family val="2"/>
       <b val="1"/>
       <color rgb="FF595959"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF7F7F7F"/>
       <sz val="9"/>
     </font>
     <font>
@@ -2456,13 +2449,13 @@
     <xf numFmtId="0" fontId="15" fillId="8" borderId="37" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="7" borderId="38" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
@@ -2474,16 +2467,16 @@
     <xf numFmtId="0" fontId="13" fillId="7" borderId="40" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="8" borderId="18" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="8" borderId="21" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
@@ -2639,13 +2632,13 @@
     <xf numFmtId="167" fontId="3" fillId="9" borderId="44" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
+    <xf numFmtId="166" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
+    <xf numFmtId="167" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
@@ -2711,13 +2704,13 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="48" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="18" fillId="0" borderId="8" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="166" fontId="17" fillId="0" borderId="8" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="18" fillId="0" borderId="8" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="167" fontId="17" fillId="0" borderId="8" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="true" applyAlignment="false">
@@ -2774,7 +2767,7 @@
     <xf numFmtId="167" fontId="3" fillId="9" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="44" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
@@ -2813,43 +2806,127 @@
     <xf numFmtId="166" fontId="8" fillId="0" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="50" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="50" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="20" fillId="10" borderId="49" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="166" fontId="19" fillId="10" borderId="49" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="20" fillId="10" borderId="49" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="167" fontId="19" fillId="10" borderId="49" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="21" fillId="11" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="12" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="51" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="7" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="52" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="18" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="12" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="12" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="17" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="18" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="20" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="21" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="11" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="12" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="38" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="12" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="39" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="167" fontId="3" fillId="8" borderId="40" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="8" borderId="21" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="11" borderId="51" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
@@ -2861,90 +2938,6 @@
     <xf numFmtId="0" fontId="23" fillId="11" borderId="52" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="18" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="172" fontId="12" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="172" fontId="12" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="17" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="18" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="20" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="21" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="12" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="11" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="12" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="38" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="39" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="8" borderId="40" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="12" fillId="8" borderId="21" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="11" borderId="51" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="11" borderId="7" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="11" borderId="52" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="17" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3017,31 +3010,31 @@
     <xf numFmtId="173" fontId="3" fillId="8" borderId="21" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center" wrapText="true"/>
     </xf>
     <xf numFmtId="173" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="11" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="26" fillId="11" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="166" fontId="25" fillId="11" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="26" fillId="11" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="173" fontId="25" fillId="11" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="26" fillId="11" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="167" fontId="25" fillId="11" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="51" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="51" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="7" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="7" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="52" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="52" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
@@ -3059,19 +3052,19 @@
     <xf numFmtId="173" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="11" borderId="32" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="32" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="26" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="166" fontId="25" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="26" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="173" fontId="25" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="26" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="167" fontId="25" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="26" fillId="11" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="173" fontId="25" fillId="11" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="173" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
@@ -3098,10 +3091,10 @@
     <xf numFmtId="173" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="26" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="173" fontId="25" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="26" fillId="11" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="173" fontId="25" fillId="11" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
@@ -3128,10 +3121,10 @@
     <xf numFmtId="173" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="26" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="173" fontId="25" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="26" fillId="11" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="173" fontId="25" fillId="11" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="173" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
@@ -3158,10 +3151,10 @@
     <xf numFmtId="173" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="26" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="173" fontId="25" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="26" fillId="11" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="173" fontId="25" fillId="11" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">

</xml_diff>

<commit_message>
feat: add manual amount deduction to KMW evaluation
Implement manual amount input field for each period and deduct the
corresponding value in the evaluation report.
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_befuellt.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_befuellt.xlsx
@@ -103,23 +103,41 @@
     <definedName name="FB_SaldoLC_18">'III. Finanzberichte'!$DR$31</definedName>
     <definedName name="FB_SaldoEUR_18">'III. Finanzberichte'!$DS$31</definedName>
     <definedName name="MA_Kurs_1">'IV. MA'!$C$8</definedName>
+    <definedName name="MA_ManBetrag_1">'IV. MA'!$D$24</definedName>
     <definedName name="MA_Kurs_2">'IV. MA'!$G$8</definedName>
+    <definedName name="MA_ManBetrag_2">'IV. MA'!$H$24</definedName>
     <definedName name="MA_Kurs_3">'IV. MA'!$K$8</definedName>
+    <definedName name="MA_ManBetrag_3">'IV. MA'!$L$24</definedName>
     <definedName name="MA_Kurs_4">'IV. MA'!$O$8</definedName>
+    <definedName name="MA_ManBetrag_4">'IV. MA'!$P$24</definedName>
     <definedName name="MA_Kurs_5">'IV. MA'!$S$8</definedName>
+    <definedName name="MA_ManBetrag_5">'IV. MA'!$T$24</definedName>
     <definedName name="MA_Kurs_6">'IV. MA'!$W$8</definedName>
+    <definedName name="MA_ManBetrag_6">'IV. MA'!$X$24</definedName>
     <definedName name="MA_Kurs_7">'IV. MA'!$AA$8</definedName>
+    <definedName name="MA_ManBetrag_7">'IV. MA'!$AB$24</definedName>
     <definedName name="MA_Kurs_8">'IV. MA'!$AE$8</definedName>
+    <definedName name="MA_ManBetrag_8">'IV. MA'!$AF$24</definedName>
     <definedName name="MA_Kurs_9">'IV. MA'!$AI$8</definedName>
+    <definedName name="MA_ManBetrag_9">'IV. MA'!$AJ$24</definedName>
     <definedName name="MA_Kurs_10">'IV. MA'!$AM$8</definedName>
+    <definedName name="MA_ManBetrag_10">'IV. MA'!$AN$24</definedName>
     <definedName name="MA_Kurs_11">'IV. MA'!$AQ$8</definedName>
+    <definedName name="MA_ManBetrag_11">'IV. MA'!$AR$24</definedName>
     <definedName name="MA_Kurs_12">'IV. MA'!$AU$8</definedName>
+    <definedName name="MA_ManBetrag_12">'IV. MA'!$AV$24</definedName>
     <definedName name="MA_Kurs_13">'IV. MA'!$AY$8</definedName>
+    <definedName name="MA_ManBetrag_13">'IV. MA'!$AZ$24</definedName>
     <definedName name="MA_Kurs_14">'IV. MA'!$BC$8</definedName>
+    <definedName name="MA_ManBetrag_14">'IV. MA'!$BD$24</definedName>
     <definedName name="MA_Kurs_15">'IV. MA'!$BG$8</definedName>
+    <definedName name="MA_ManBetrag_15">'IV. MA'!$BH$24</definedName>
     <definedName name="MA_Kurs_16">'IV. MA'!$BK$8</definedName>
+    <definedName name="MA_ManBetrag_16">'IV. MA'!$BL$24</definedName>
     <definedName name="MA_Kurs_17">'IV. MA'!$BO$8</definedName>
+    <definedName name="MA_ManBetrag_17">'IV. MA'!$BP$24</definedName>
     <definedName name="MA_Kurs_18">'IV. MA'!$BS$8</definedName>
+    <definedName name="MA_ManBetrag_18">'IV. MA'!$BT$24</definedName>
     <definedName name="FB_Auswahl_Liste">OFFSET('Daten'!$BP$1,0,0,COUNTA('Daten'!$BP:$BP),1)</definedName>
     <definedName name="MA_Auswahl_Liste">OFFSET('Daten'!$BN$1,0,0,COUNTA('Daten'!$BN:$BN),1)</definedName>
   </definedNames>
@@ -150,7 +168,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="402">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="403">
   <si>
     <t xml:space="preserve">  DASHBOARD (v1.0)</t>
   </si>
@@ -1152,6 +1170,9 @@
   </si>
   <si>
     <t>abzueglich Saldo Vorprojekt:</t>
+  </si>
+  <si>
+    <t>Manueller Betrag:</t>
   </si>
   <si>
     <t>KMW-Mittel Anforderung:</t>
@@ -2806,6 +2827,9 @@
     <xf numFmtId="166" fontId="8" fillId="0" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="50" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -2950,7 +2974,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="true" applyAlignment="false">
       <alignment/>
     </xf>
-    <xf numFmtId="167" fontId="3" fillId="5" borderId="40" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="167" fontId="3" fillId="12" borderId="40" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="7" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
@@ -2958,9 +2982,6 @@
     </xf>
     <xf numFmtId="166" fontId="3" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment/>
     </xf>
     <xf numFmtId="172" fontId="3" fillId="5" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
@@ -20882,7 +20903,7 @@
         <f>=IFERROR(ROUND($C$23/$C$8,2),0)</f>
       </c>
       <c r="F23" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G23" s="188" t="str">
         <f>=ROUND(IFERROR(FB_SaldoLC_1,0),2)</f>
@@ -20891,7 +20912,7 @@
         <f>=IFERROR(ROUND($G$23/$G$8,2),0)</f>
       </c>
       <c r="J23" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="K23" s="188" t="str">
         <f>=ROUND(IFERROR(FB_SaldoLC_2,0),2)</f>
@@ -20900,7 +20921,7 @@
         <f>=IFERROR(ROUND($K$23/$K$8,2),0)</f>
       </c>
       <c r="N23" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="O23" s="188" t="str">
         <f>=ROUND(IFERROR(FB_SaldoLC_3,0),2)</f>
@@ -20909,7 +20930,7 @@
         <f>=IFERROR(ROUND($O$23/$O$8,2),0)</f>
       </c>
       <c r="R23" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="S23" s="188" t="str">
         <f>=ROUND(IFERROR(FB_SaldoLC_4,0),2)</f>
@@ -20918,7 +20939,7 @@
         <f>=IFERROR(ROUND($S$23/$S$8,2),0)</f>
       </c>
       <c r="V23" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="W23" s="188" t="str">
         <f>=ROUND(IFERROR(FB_SaldoLC_5,0),2)</f>
@@ -20927,7 +20948,7 @@
         <f>=IFERROR(ROUND($W$23/$W$8,2),0)</f>
       </c>
       <c r="Z23" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="AA23" s="188" t="str">
         <f>=ROUND(IFERROR(FB_SaldoLC_6,0),2)</f>
@@ -20936,7 +20957,7 @@
         <f>=IFERROR(ROUND($AA$23/$AA$8,2),0)</f>
       </c>
       <c r="AD23" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="AE23" s="188" t="str">
         <f>=ROUND(IFERROR(FB_SaldoLC_7,0),2)</f>
@@ -20945,7 +20966,7 @@
         <f>=IFERROR(ROUND($AE$23/$AE$8,2),0)</f>
       </c>
       <c r="AH23" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="AI23" s="188" t="str">
         <f>=ROUND(IFERROR(FB_SaldoLC_8,0),2)</f>
@@ -20954,7 +20975,7 @@
         <f>=IFERROR(ROUND($AI$23/$AI$8,2),0)</f>
       </c>
       <c r="AL23" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="AM23" s="188" t="str">
         <f>=ROUND(IFERROR(FB_SaldoLC_9,0),2)</f>
@@ -20963,7 +20984,7 @@
         <f>=IFERROR(ROUND($AM$23/$AM$8,2),0)</f>
       </c>
       <c r="AP23" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="AQ23" s="188" t="str">
         <f>=ROUND(IFERROR(FB_SaldoLC_10,0),2)</f>
@@ -20972,7 +20993,7 @@
         <f>=IFERROR(ROUND($AQ$23/$AQ$8,2),0)</f>
       </c>
       <c r="AT23" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="AU23" s="188" t="str">
         <f>=ROUND(IFERROR(FB_SaldoLC_11,0),2)</f>
@@ -20981,7 +21002,7 @@
         <f>=IFERROR(ROUND($AU$23/$AU$8,2),0)</f>
       </c>
       <c r="AX23" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="AY23" s="188" t="str">
         <f>=ROUND(IFERROR(FB_SaldoLC_12,0),2)</f>
@@ -20990,7 +21011,7 @@
         <f>=IFERROR(ROUND($AY$23/$AY$8,2),0)</f>
       </c>
       <c r="BB23" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="BC23" s="188" t="str">
         <f>=ROUND(IFERROR(FB_SaldoLC_13,0),2)</f>
@@ -20999,7 +21020,7 @@
         <f>=IFERROR(ROUND($BC$23/$BC$8,2),0)</f>
       </c>
       <c r="BF23" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="BG23" s="188" t="str">
         <f>=ROUND(IFERROR(FB_SaldoLC_14,0),2)</f>
@@ -21008,7 +21029,7 @@
         <f>=IFERROR(ROUND($BG$23/$BG$8,2),0)</f>
       </c>
       <c r="BJ23" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="BK23" s="188" t="str">
         <f>=ROUND(IFERROR(FB_SaldoLC_15,0),2)</f>
@@ -21017,7 +21038,7 @@
         <f>=IFERROR(ROUND($BK$23/$BK$8,2),0)</f>
       </c>
       <c r="BN23" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="BO23" s="188" t="str">
         <f>=ROUND(IFERROR(FB_SaldoLC_16,0),2)</f>
@@ -21026,7 +21047,7 @@
         <f>=IFERROR(ROUND($BO$23/$BO$8,2),0)</f>
       </c>
       <c r="BR23" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="BS23" s="188" t="str">
         <f>=ROUND(IFERROR(FB_SaldoLC_17,0),2)</f>
@@ -21035,167 +21056,259 @@
         <f>=IFERROR(ROUND($BS$23/$BS$8,2),0)</f>
       </c>
     </row>
+    <row r="24">
+      <c r="B24" t="s">
+        <v>334</v>
+      </c>
+      <c r="C24" s="189"/>
+      <c r="D24" s="25"/>
+      <c r="F24" t="s">
+        <v>334</v>
+      </c>
+      <c r="G24" s="189"/>
+      <c r="H24" s="25"/>
+      <c r="J24" t="s">
+        <v>334</v>
+      </c>
+      <c r="K24" s="189"/>
+      <c r="L24" s="25"/>
+      <c r="N24" t="s">
+        <v>334</v>
+      </c>
+      <c r="O24" s="189"/>
+      <c r="P24" s="25"/>
+      <c r="R24" t="s">
+        <v>334</v>
+      </c>
+      <c r="S24" s="189"/>
+      <c r="T24" s="25"/>
+      <c r="V24" t="s">
+        <v>334</v>
+      </c>
+      <c r="W24" s="189"/>
+      <c r="X24" s="25"/>
+      <c r="Z24" t="s">
+        <v>334</v>
+      </c>
+      <c r="AA24" s="189"/>
+      <c r="AB24" s="25"/>
+      <c r="AD24" t="s">
+        <v>334</v>
+      </c>
+      <c r="AE24" s="189"/>
+      <c r="AF24" s="25"/>
+      <c r="AH24" t="s">
+        <v>334</v>
+      </c>
+      <c r="AI24" s="189"/>
+      <c r="AJ24" s="25"/>
+      <c r="AL24" t="s">
+        <v>334</v>
+      </c>
+      <c r="AM24" s="189"/>
+      <c r="AN24" s="25"/>
+      <c r="AP24" t="s">
+        <v>334</v>
+      </c>
+      <c r="AQ24" s="189"/>
+      <c r="AR24" s="25"/>
+      <c r="AT24" t="s">
+        <v>334</v>
+      </c>
+      <c r="AU24" s="189"/>
+      <c r="AV24" s="25"/>
+      <c r="AX24" t="s">
+        <v>334</v>
+      </c>
+      <c r="AY24" s="189"/>
+      <c r="AZ24" s="25"/>
+      <c r="BB24" t="s">
+        <v>334</v>
+      </c>
+      <c r="BC24" s="189"/>
+      <c r="BD24" s="25"/>
+      <c r="BF24" t="s">
+        <v>334</v>
+      </c>
+      <c r="BG24" s="189"/>
+      <c r="BH24" s="25"/>
+      <c r="BJ24" t="s">
+        <v>334</v>
+      </c>
+      <c r="BK24" s="189"/>
+      <c r="BL24" s="25"/>
+      <c r="BN24" t="s">
+        <v>334</v>
+      </c>
+      <c r="BO24" s="189"/>
+      <c r="BP24" s="25"/>
+      <c r="BR24" t="s">
+        <v>334</v>
+      </c>
+      <c r="BS24" s="189"/>
+      <c r="BT24" s="25"/>
+    </row>
     <row r="25">
-      <c r="B25" s="189" t="s">
-        <v>334</v>
-      </c>
-      <c r="C25" s="190" t="str">
+      <c r="B25" s="190" t="s">
+        <v>335</v>
+      </c>
+      <c r="C25" s="191" t="str">
         <f>=IFERROR(ROUND($C$18-$C$21-$C$22-$C$23,2),0)</f>
       </c>
-      <c r="D25" s="191" t="str">
+      <c r="D25" s="192" t="str">
         <f>=IFERROR(ROUND($D$18-$D$21-$D$22-$D$23,2),0)</f>
       </c>
-      <c r="F25" s="189" t="s">
-        <v>334</v>
-      </c>
-      <c r="G25" s="190" t="str">
+      <c r="F25" s="190" t="s">
+        <v>335</v>
+      </c>
+      <c r="G25" s="191" t="str">
         <f>=IFERROR(ROUND($G$18-$G$21-$G$22-$G$23,2),0)</f>
       </c>
-      <c r="H25" s="191" t="str">
+      <c r="H25" s="192" t="str">
         <f>=IFERROR(ROUND($H$18-$H$21-$H$22-$H$23,2),0)</f>
       </c>
-      <c r="J25" s="189" t="s">
-        <v>334</v>
-      </c>
-      <c r="K25" s="190" t="str">
+      <c r="J25" s="190" t="s">
+        <v>335</v>
+      </c>
+      <c r="K25" s="191" t="str">
         <f>=IFERROR(ROUND($K$18-$K$21-$K$22-$K$23,2),0)</f>
       </c>
-      <c r="L25" s="191" t="str">
+      <c r="L25" s="192" t="str">
         <f>=IFERROR(ROUND($L$18-$L$21-$L$22-$L$23,2),0)</f>
       </c>
-      <c r="N25" s="189" t="s">
-        <v>334</v>
-      </c>
-      <c r="O25" s="190" t="str">
+      <c r="N25" s="190" t="s">
+        <v>335</v>
+      </c>
+      <c r="O25" s="191" t="str">
         <f>=IFERROR(ROUND($O$18-$O$21-$O$22-$O$23,2),0)</f>
       </c>
-      <c r="P25" s="191" t="str">
+      <c r="P25" s="192" t="str">
         <f>=IFERROR(ROUND($P$18-$P$21-$P$22-$P$23,2),0)</f>
       </c>
-      <c r="R25" s="189" t="s">
-        <v>334</v>
-      </c>
-      <c r="S25" s="190" t="str">
+      <c r="R25" s="190" t="s">
+        <v>335</v>
+      </c>
+      <c r="S25" s="191" t="str">
         <f>=IFERROR(ROUND($S$18-$S$21-$S$22-$S$23,2),0)</f>
       </c>
-      <c r="T25" s="191" t="str">
+      <c r="T25" s="192" t="str">
         <f>=IFERROR(ROUND($T$18-$T$21-$T$22-$T$23,2),0)</f>
       </c>
-      <c r="V25" s="189" t="s">
-        <v>334</v>
-      </c>
-      <c r="W25" s="190" t="str">
+      <c r="V25" s="190" t="s">
+        <v>335</v>
+      </c>
+      <c r="W25" s="191" t="str">
         <f>=IFERROR(ROUND($W$18-$W$21-$W$22-$W$23,2),0)</f>
       </c>
-      <c r="X25" s="191" t="str">
+      <c r="X25" s="192" t="str">
         <f>=IFERROR(ROUND($X$18-$X$21-$X$22-$X$23,2),0)</f>
       </c>
-      <c r="Z25" s="189" t="s">
-        <v>334</v>
-      </c>
-      <c r="AA25" s="190" t="str">
+      <c r="Z25" s="190" t="s">
+        <v>335</v>
+      </c>
+      <c r="AA25" s="191" t="str">
         <f>=IFERROR(ROUND($AA$18-$AA$21-$AA$22-$AA$23,2),0)</f>
       </c>
-      <c r="AB25" s="191" t="str">
+      <c r="AB25" s="192" t="str">
         <f>=IFERROR(ROUND($AB$18-$AB$21-$AB$22-$AB$23,2),0)</f>
       </c>
-      <c r="AD25" s="189" t="s">
-        <v>334</v>
-      </c>
-      <c r="AE25" s="190" t="str">
+      <c r="AD25" s="190" t="s">
+        <v>335</v>
+      </c>
+      <c r="AE25" s="191" t="str">
         <f>=IFERROR(ROUND($AE$18-$AE$21-$AE$22-$AE$23,2),0)</f>
       </c>
-      <c r="AF25" s="191" t="str">
+      <c r="AF25" s="192" t="str">
         <f>=IFERROR(ROUND($AF$18-$AF$21-$AF$22-$AF$23,2),0)</f>
       </c>
-      <c r="AH25" s="189" t="s">
-        <v>334</v>
-      </c>
-      <c r="AI25" s="190" t="str">
+      <c r="AH25" s="190" t="s">
+        <v>335</v>
+      </c>
+      <c r="AI25" s="191" t="str">
         <f>=IFERROR(ROUND($AI$18-$AI$21-$AI$22-$AI$23,2),0)</f>
       </c>
-      <c r="AJ25" s="191" t="str">
+      <c r="AJ25" s="192" t="str">
         <f>=IFERROR(ROUND($AJ$18-$AJ$21-$AJ$22-$AJ$23,2),0)</f>
       </c>
-      <c r="AL25" s="189" t="s">
-        <v>334</v>
-      </c>
-      <c r="AM25" s="190" t="str">
+      <c r="AL25" s="190" t="s">
+        <v>335</v>
+      </c>
+      <c r="AM25" s="191" t="str">
         <f>=IFERROR(ROUND($AM$18-$AM$21-$AM$22-$AM$23,2),0)</f>
       </c>
-      <c r="AN25" s="191" t="str">
+      <c r="AN25" s="192" t="str">
         <f>=IFERROR(ROUND($AN$18-$AN$21-$AN$22-$AN$23,2),0)</f>
       </c>
-      <c r="AP25" s="189" t="s">
-        <v>334</v>
-      </c>
-      <c r="AQ25" s="190" t="str">
+      <c r="AP25" s="190" t="s">
+        <v>335</v>
+      </c>
+      <c r="AQ25" s="191" t="str">
         <f>=IFERROR(ROUND($AQ$18-$AQ$21-$AQ$22-$AQ$23,2),0)</f>
       </c>
-      <c r="AR25" s="191" t="str">
+      <c r="AR25" s="192" t="str">
         <f>=IFERROR(ROUND($AR$18-$AR$21-$AR$22-$AR$23,2),0)</f>
       </c>
-      <c r="AT25" s="189" t="s">
-        <v>334</v>
-      </c>
-      <c r="AU25" s="190" t="str">
+      <c r="AT25" s="190" t="s">
+        <v>335</v>
+      </c>
+      <c r="AU25" s="191" t="str">
         <f>=IFERROR(ROUND($AU$18-$AU$21-$AU$22-$AU$23,2),0)</f>
       </c>
-      <c r="AV25" s="191" t="str">
+      <c r="AV25" s="192" t="str">
         <f>=IFERROR(ROUND($AV$18-$AV$21-$AV$22-$AV$23,2),0)</f>
       </c>
-      <c r="AX25" s="189" t="s">
-        <v>334</v>
-      </c>
-      <c r="AY25" s="190" t="str">
+      <c r="AX25" s="190" t="s">
+        <v>335</v>
+      </c>
+      <c r="AY25" s="191" t="str">
         <f>=IFERROR(ROUND($AY$18-$AY$21-$AY$22-$AY$23,2),0)</f>
       </c>
-      <c r="AZ25" s="191" t="str">
+      <c r="AZ25" s="192" t="str">
         <f>=IFERROR(ROUND($AZ$18-$AZ$21-$AZ$22-$AZ$23,2),0)</f>
       </c>
-      <c r="BB25" s="189" t="s">
-        <v>334</v>
-      </c>
-      <c r="BC25" s="190" t="str">
+      <c r="BB25" s="190" t="s">
+        <v>335</v>
+      </c>
+      <c r="BC25" s="191" t="str">
         <f>=IFERROR(ROUND($BC$18-$BC$21-$BC$22-$BC$23,2),0)</f>
       </c>
-      <c r="BD25" s="191" t="str">
+      <c r="BD25" s="192" t="str">
         <f>=IFERROR(ROUND($BD$18-$BD$21-$BD$22-$BD$23,2),0)</f>
       </c>
-      <c r="BF25" s="189" t="s">
-        <v>334</v>
-      </c>
-      <c r="BG25" s="190" t="str">
+      <c r="BF25" s="190" t="s">
+        <v>335</v>
+      </c>
+      <c r="BG25" s="191" t="str">
         <f>=IFERROR(ROUND($BG$18-$BG$21-$BG$22-$BG$23,2),0)</f>
       </c>
-      <c r="BH25" s="191" t="str">
+      <c r="BH25" s="192" t="str">
         <f>=IFERROR(ROUND($BH$18-$BH$21-$BH$22-$BH$23,2),0)</f>
       </c>
-      <c r="BJ25" s="189" t="s">
-        <v>334</v>
-      </c>
-      <c r="BK25" s="190" t="str">
+      <c r="BJ25" s="190" t="s">
+        <v>335</v>
+      </c>
+      <c r="BK25" s="191" t="str">
         <f>=IFERROR(ROUND($BK$18-$BK$21-$BK$22-$BK$23,2),0)</f>
       </c>
-      <c r="BL25" s="191" t="str">
+      <c r="BL25" s="192" t="str">
         <f>=IFERROR(ROUND($BL$18-$BL$21-$BL$22-$BL$23,2),0)</f>
       </c>
-      <c r="BN25" s="189" t="s">
-        <v>334</v>
-      </c>
-      <c r="BO25" s="190" t="str">
+      <c r="BN25" s="190" t="s">
+        <v>335</v>
+      </c>
+      <c r="BO25" s="191" t="str">
         <f>=IFERROR(ROUND($BO$18-$BO$21-$BO$22-$BO$23,2),0)</f>
       </c>
-      <c r="BP25" s="191" t="str">
+      <c r="BP25" s="192" t="str">
         <f>=IFERROR(ROUND($BP$18-$BP$21-$BP$22-$BP$23,2),0)</f>
       </c>
-      <c r="BR25" s="189" t="s">
-        <v>334</v>
-      </c>
-      <c r="BS25" s="190" t="str">
+      <c r="BR25" s="190" t="s">
+        <v>335</v>
+      </c>
+      <c r="BS25" s="191" t="str">
         <f>=IFERROR(ROUND($BS$18-$BS$21-$BS$22-$BS$23,2),0)</f>
       </c>
-      <c r="BT25" s="191" t="str">
+      <c r="BT25" s="192" t="str">
         <f>=IFERROR(ROUND($BT$18-$BT$21-$BT$22-$BT$23,2),0)</f>
       </c>
     </row>
@@ -21389,64 +21502,64 @@
   </cols>
   <sheetData>
     <row r="2" ht="30" customHeight="true">
-      <c r="B2" s="192" t="s">
-        <v>336</v>
-      </c>
-      <c r="C2" s="192"/>
-      <c r="D2" s="192"/>
-      <c r="E2" s="192"/>
-      <c r="F2" s="192"/>
-      <c r="G2" s="192"/>
-      <c r="H2" s="192"/>
-      <c r="I2" s="192"/>
-      <c r="J2" s="192"/>
+      <c r="B2" s="193" t="s">
+        <v>337</v>
+      </c>
+      <c r="C2" s="193"/>
+      <c r="D2" s="193"/>
+      <c r="E2" s="193"/>
+      <c r="F2" s="193"/>
+      <c r="G2" s="193"/>
+      <c r="H2" s="193"/>
+      <c r="I2" s="193"/>
+      <c r="J2" s="193"/>
     </row>
     <row r="3" ht="18" customHeight="true">
-      <c r="B3" s="193" t="s">
-        <v>337</v>
-      </c>
-      <c r="C3" s="193"/>
-      <c r="D3" s="193"/>
-      <c r="E3" s="193"/>
-      <c r="F3" s="193"/>
-      <c r="G3" s="193"/>
-      <c r="H3" s="193"/>
-      <c r="I3" s="193"/>
-      <c r="J3" s="193"/>
+      <c r="B3" s="194" t="s">
+        <v>338</v>
+      </c>
+      <c r="C3" s="194"/>
+      <c r="D3" s="194"/>
+      <c r="E3" s="194"/>
+      <c r="F3" s="194"/>
+      <c r="G3" s="194"/>
+      <c r="H3" s="194"/>
+      <c r="I3" s="194"/>
+      <c r="J3" s="194"/>
     </row>
     <row r="5" ht="22" customHeight="true">
-      <c r="B5" s="194" t="s">
-        <v>338</v>
-      </c>
-      <c r="C5" s="194"/>
-      <c r="D5" s="194"/>
-      <c r="E5" s="194"/>
-      <c r="F5" s="194"/>
-      <c r="G5" s="194"/>
-      <c r="H5" s="194"/>
-      <c r="I5" s="194"/>
-      <c r="J5" s="194"/>
-      <c r="L5" s="202" t="str">
+      <c r="B5" s="195" t="s">
+        <v>339</v>
+      </c>
+      <c r="C5" s="195"/>
+      <c r="D5" s="195"/>
+      <c r="E5" s="195"/>
+      <c r="F5" s="195"/>
+      <c r="G5" s="195"/>
+      <c r="H5" s="195"/>
+      <c r="I5" s="195"/>
+      <c r="J5" s="195"/>
+      <c r="L5" s="203" t="str">
         <f>=IF(E11=0,"Aktuelle Mittelanforderung (keine gewählt)","Aktuelle Mittelanforderung – Periode "&amp;E10&amp;" (#"&amp;E11&amp;")")</f>
       </c>
-      <c r="M5" s="203"/>
-      <c r="N5" s="204"/>
+      <c r="M5" s="204"/>
+      <c r="N5" s="205"/>
       <c r="AD5" t="str">
         <f>=IFERROR(SUMPRODUCT('Daten'!$BA$1:$BA$18,('Daten'!$BB$1:$BB$18=E10)*('Daten'!$BD$1:$BD$18=E11)),0)</f>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="195" t="s">
-        <v>339</v>
-      </c>
-      <c r="C6" s="195"/>
-      <c r="D6" s="195"/>
-      <c r="E6" s="195"/>
-      <c r="F6" s="195"/>
-      <c r="G6" s="195"/>
-      <c r="H6" s="195"/>
-      <c r="I6" s="195"/>
-      <c r="J6" s="195"/>
+      <c r="B6" s="196" t="s">
+        <v>340</v>
+      </c>
+      <c r="C6" s="196"/>
+      <c r="D6" s="196"/>
+      <c r="E6" s="196"/>
+      <c r="F6" s="196"/>
+      <c r="G6" s="196"/>
+      <c r="H6" s="196"/>
+      <c r="I6" s="196"/>
+      <c r="J6" s="196"/>
       <c r="L6" s="315" t="s">
         <v>288</v>
       </c>
@@ -21465,13 +21578,13 @@
       <c r="N7" s="317"/>
     </row>
     <row r="8" ht="22" customHeight="true">
-      <c r="C8" s="202" t="s">
-        <v>340</v>
-      </c>
-      <c r="D8" s="203"/>
-      <c r="E8" s="203"/>
-      <c r="F8" s="203"/>
-      <c r="G8" s="204"/>
+      <c r="C8" s="203" t="s">
+        <v>341</v>
+      </c>
+      <c r="D8" s="204"/>
+      <c r="E8" s="204"/>
+      <c r="F8" s="204"/>
+      <c r="G8" s="205"/>
       <c r="L8" s="315" t="s">
         <v>290</v>
       </c>
@@ -21481,15 +21594,15 @@
       <c r="N8" s="317"/>
     </row>
     <row r="9">
-      <c r="C9" s="205" t="s">
-        <v>341</v>
-      </c>
-      <c r="D9" s="197"/>
+      <c r="C9" s="206" t="s">
+        <v>342</v>
+      </c>
+      <c r="D9" s="198"/>
       <c r="E9" s="63" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="F9" s="63"/>
-      <c r="G9" s="206"/>
+      <c r="G9" s="207"/>
       <c r="L9" s="315" t="s">
         <v>291</v>
       </c>
@@ -21499,16 +21612,16 @@
       <c r="N9" s="318"/>
     </row>
     <row r="10">
-      <c r="C10" s="205" t="s">
-        <v>343</v>
-      </c>
-      <c r="D10" s="197"/>
-      <c r="E10" s="198" t="str">
+      <c r="C10" s="206" t="s">
+        <v>344</v>
+      </c>
+      <c r="D10" s="198"/>
+      <c r="E10" s="199" t="str">
         <f>=E81+1</f>
         <v>0</v>
       </c>
-      <c r="F10" s="198"/>
-      <c r="G10" s="207"/>
+      <c r="F10" s="199"/>
+      <c r="G10" s="208"/>
       <c r="L10" s="315" t="s">
         <v>326</v>
       </c>
@@ -21518,26 +21631,26 @@
       <c r="N10" s="319"/>
     </row>
     <row r="11">
-      <c r="C11" s="205" t="s">
-        <v>344</v>
-      </c>
-      <c r="D11" s="197"/>
-      <c r="E11" s="198" t="str">
+      <c r="C11" s="206" t="s">
+        <v>345</v>
+      </c>
+      <c r="D11" s="198"/>
+      <c r="E11" s="199" t="str">
         <f>=IF(E9="Neuste MA",IFERROR(SUMPRODUCT(MAX(('Daten'!$BB$1:$BB$18=E10)*('Daten'!$BC$1:$BC$18=1)*'Daten'!$BD$1:$BD$18)),0),IFERROR(VALUE(MID(E9,FIND("(#",E9)+2,FIND(")",E9)-FIND("(#",E9)-2)),0))</f>
       </c>
-      <c r="F11" s="198"/>
-      <c r="G11" s="208"/>
+      <c r="F11" s="199"/>
+      <c r="G11" s="209"/>
       <c r="L11" s="47"/>
       <c r="N11" s="48"/>
     </row>
     <row r="12">
-      <c r="C12" s="209" t="s">
-        <v>345</v>
-      </c>
-      <c r="D12" s="199"/>
-      <c r="E12" s="199"/>
-      <c r="F12" s="199"/>
-      <c r="G12" s="210"/>
+      <c r="C12" s="210" t="s">
+        <v>346</v>
+      </c>
+      <c r="D12" s="200"/>
+      <c r="E12" s="200"/>
+      <c r="F12" s="200"/>
+      <c r="G12" s="211"/>
       <c r="L12" s="320" t="s">
         <v>202</v>
       </c>
@@ -21549,15 +21662,15 @@
       </c>
     </row>
     <row r="13">
-      <c r="C13" s="211" t="str">
+      <c r="C13" s="212" t="str">
         <f>=IF(1&lt;=E11,"Periode "&amp;E10&amp;" (#1)","")</f>
       </c>
-      <c r="D13" s="200"/>
-      <c r="E13" s="201" t="str">
+      <c r="D13" s="201"/>
+      <c r="E13" s="202" t="str">
         <f>=IF(1&lt;=E11,IFERROR(SUMIFS('Daten'!$BF$1:$BF$18,'Daten'!$BB$1:$BB$18,E10,'Daten'!$BD$1:$BD$18,1),0),"")</f>
       </c>
-      <c r="F13" s="201"/>
-      <c r="G13" s="212" t="str">
+      <c r="F13" s="202"/>
+      <c r="G13" s="213" t="str">
         <f>=IF(1&lt;=E11,IFERROR(SUMIFS('Daten'!$BG$1:$BG$18,'Daten'!$BB$1:$BB$18,E10,'Daten'!$BD$1:$BD$18,1),0),"")</f>
       </c>
       <c r="L13" s="143" t="s">
@@ -21571,15 +21684,15 @@
       </c>
     </row>
     <row r="14">
-      <c r="C14" s="211" t="str">
+      <c r="C14" s="212" t="str">
         <f>=IF(2&lt;=E11,"Periode "&amp;E10&amp;" (#2)","")</f>
       </c>
-      <c r="D14" s="200"/>
-      <c r="E14" s="201" t="str">
+      <c r="D14" s="201"/>
+      <c r="E14" s="202" t="str">
         <f>=IF(2&lt;=E11,IFERROR(SUMIFS('Daten'!$BF$1:$BF$18,'Daten'!$BB$1:$BB$18,E10,'Daten'!$BD$1:$BD$18,2),0),"")</f>
       </c>
-      <c r="F14" s="201"/>
-      <c r="G14" s="212" t="str">
+      <c r="F14" s="202"/>
+      <c r="G14" s="213" t="str">
         <f>=IF(2&lt;=E11,IFERROR(SUMIFS('Daten'!$BG$1:$BG$18,'Daten'!$BB$1:$BB$18,E10,'Daten'!$BD$1:$BD$18,2),0),"")</f>
       </c>
       <c r="L14" s="143" t="s">
@@ -21593,15 +21706,15 @@
       </c>
     </row>
     <row r="15">
-      <c r="C15" s="211" t="str">
+      <c r="C15" s="212" t="str">
         <f>=IF(3&lt;=E11,"Periode "&amp;E10&amp;" (#3)","")</f>
       </c>
-      <c r="D15" s="200"/>
-      <c r="E15" s="201" t="str">
+      <c r="D15" s="201"/>
+      <c r="E15" s="202" t="str">
         <f>=IF(3&lt;=E11,IFERROR(SUMIFS('Daten'!$BF$1:$BF$18,'Daten'!$BB$1:$BB$18,E10,'Daten'!$BD$1:$BD$18,3),0),"")</f>
       </c>
-      <c r="F15" s="201"/>
-      <c r="G15" s="212" t="str">
+      <c r="F15" s="202"/>
+      <c r="G15" s="213" t="str">
         <f>=IF(3&lt;=E11,IFERROR(SUMIFS('Daten'!$BG$1:$BG$18,'Daten'!$BB$1:$BB$18,E10,'Daten'!$BD$1:$BD$18,3),0),"")</f>
       </c>
       <c r="L15" s="143" t="s">
@@ -21615,15 +21728,15 @@
       </c>
     </row>
     <row r="16">
-      <c r="C16" s="211" t="str">
+      <c r="C16" s="212" t="str">
         <f>=IF(4&lt;=E11,"Periode "&amp;E10&amp;" (#4)","")</f>
       </c>
-      <c r="D16" s="200"/>
-      <c r="E16" s="201" t="str">
+      <c r="D16" s="201"/>
+      <c r="E16" s="202" t="str">
         <f>=IF(4&lt;=E11,IFERROR(SUMIFS('Daten'!$BF$1:$BF$18,'Daten'!$BB$1:$BB$18,E10,'Daten'!$BD$1:$BD$18,4),0),"")</f>
       </c>
-      <c r="F16" s="201"/>
-      <c r="G16" s="212" t="str">
+      <c r="F16" s="202"/>
+      <c r="G16" s="213" t="str">
         <f>=IF(4&lt;=E11,IFERROR(SUMIFS('Daten'!$BG$1:$BG$18,'Daten'!$BB$1:$BB$18,E10,'Daten'!$BD$1:$BD$18,4),0),"")</f>
       </c>
       <c r="L16" s="143" t="s">
@@ -21637,15 +21750,15 @@
       </c>
     </row>
     <row r="17">
-      <c r="C17" s="211" t="str">
+      <c r="C17" s="212" t="str">
         <f>=IF(5&lt;=E11,"Periode "&amp;E10&amp;" (#5)","")</f>
       </c>
-      <c r="D17" s="200"/>
-      <c r="E17" s="201" t="str">
+      <c r="D17" s="201"/>
+      <c r="E17" s="202" t="str">
         <f>=IF(5&lt;=E11,IFERROR(SUMIFS('Daten'!$BF$1:$BF$18,'Daten'!$BB$1:$BB$18,E10,'Daten'!$BD$1:$BD$18,5),0),"")</f>
       </c>
-      <c r="F17" s="201"/>
-      <c r="G17" s="212" t="str">
+      <c r="F17" s="202"/>
+      <c r="G17" s="213" t="str">
         <f>=IF(5&lt;=E11,IFERROR(SUMIFS('Daten'!$BG$1:$BG$18,'Daten'!$BB$1:$BB$18,E10,'Daten'!$BD$1:$BD$18,5),0),"")</f>
       </c>
       <c r="L17" s="143" t="s">
@@ -21659,15 +21772,15 @@
       </c>
     </row>
     <row r="18">
-      <c r="C18" s="213" t="str">
+      <c r="C18" s="214" t="str">
         <f>=IF(6&lt;=E11,"Periode "&amp;E10&amp;" (#6)","")</f>
       </c>
-      <c r="D18" s="214"/>
-      <c r="E18" s="215" t="str">
+      <c r="D18" s="215"/>
+      <c r="E18" s="216" t="str">
         <f>=IF(6&lt;=E11,IFERROR(SUMIFS('Daten'!$BF$1:$BF$18,'Daten'!$BB$1:$BB$18,E10,'Daten'!$BD$1:$BD$18,6),0),"")</f>
       </c>
-      <c r="F18" s="215"/>
-      <c r="G18" s="216" t="str">
+      <c r="F18" s="216"/>
+      <c r="G18" s="217" t="str">
         <f>=IF(6&lt;=E11,IFERROR(SUMIFS('Daten'!$BG$1:$BG$18,'Daten'!$BB$1:$BB$18,E10,'Daten'!$BD$1:$BD$18,6),0),"")</f>
       </c>
       <c r="L18" s="143" t="s">
@@ -21693,7 +21806,7 @@
     </row>
     <row r="20" ht="22" customHeight="true">
       <c r="B20" s="18" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C20" s="18"/>
       <c r="D20" s="18"/>
@@ -21720,43 +21833,43 @@
       <c r="M21" s="243" t="str">
         <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$C$18,'IV. MA'!$G$18,'IV. MA'!$K$18,'IV. MA'!$O$18,'IV. MA'!$S$18,'IV. MA'!$W$18,'IV. MA'!$AA$18,'IV. MA'!$AE$18,'IV. MA'!$AI$18,'IV. MA'!$AM$18,'IV. MA'!$AQ$18,'IV. MA'!$AU$18,'IV. MA'!$AY$18,'IV. MA'!$BC$18,'IV. MA'!$BG$18,'IV. MA'!$BK$18,'IV. MA'!$BO$18,'IV. MA'!$BS$18),"")</f>
       </c>
-      <c r="N21" s="235" t="str">
+      <c r="N21" s="236" t="str">
         <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$D$18,'IV. MA'!$H$18,'IV. MA'!$L$18,'IV. MA'!$P$18,'IV. MA'!$T$18,'IV. MA'!$X$18,'IV. MA'!$AB$18,'IV. MA'!$AF$18,'IV. MA'!$AJ$18,'IV. MA'!$AN$18,'IV. MA'!$AR$18,'IV. MA'!$AV$18,'IV. MA'!$AZ$18,'IV. MA'!$BD$18,'IV. MA'!$BH$18,'IV. MA'!$BL$18,'IV. MA'!$BP$18,'IV. MA'!$BT$18),"")</f>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="223" t="s">
-        <v>347</v>
-      </c>
-      <c r="C22" s="224"/>
-      <c r="D22" s="225" t="str">
+      <c r="B22" s="224" t="s">
+        <v>348</v>
+      </c>
+      <c r="C22" s="225"/>
+      <c r="D22" s="226" t="str">
         <f>=IFERROR(ROUND(KMW_Mittel_EUR,2),0)</f>
       </c>
-      <c r="F22" s="230" t="s">
-        <v>351</v>
-      </c>
-      <c r="G22" s="231"/>
-      <c r="H22" s="231"/>
-      <c r="I22" s="232"/>
+      <c r="F22" s="231" t="s">
+        <v>352</v>
+      </c>
+      <c r="G22" s="232"/>
+      <c r="H22" s="232"/>
+      <c r="I22" s="233"/>
       <c r="L22" s="47"/>
       <c r="N22" s="48"/>
     </row>
     <row r="23">
-      <c r="B23" s="205" t="s">
-        <v>348</v>
-      </c>
-      <c r="C23" s="197"/>
-      <c r="D23" s="226" t="str">
+      <c r="B23" s="206" t="s">
+        <v>349</v>
+      </c>
+      <c r="C23" s="198"/>
+      <c r="D23" s="227" t="str">
         <f>=IFERROR(ROUND(Kosten_Reserve_EUR,2),0)</f>
       </c>
-      <c r="F23" s="233" t="s">
-        <v>352</v>
-      </c>
-      <c r="G23" s="197" t="s">
+      <c r="F23" s="234" t="s">
         <v>353</v>
       </c>
-      <c r="H23" s="197"/>
-      <c r="I23" s="234" t="str">
+      <c r="G23" s="198" t="s">
+        <v>354</v>
+      </c>
+      <c r="H23" s="198"/>
+      <c r="I23" s="235" t="str">
         <f>=IFERROR(ROUND(Saldovortrag_EUR,2),0)</f>
       </c>
       <c r="L23" s="143" t="s">
@@ -21770,26 +21883,26 @@
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="205" t="str">
+      <c r="B24" s="206" t="str">
         <f>=IF(Reserve_Freigabe="Ja","Operatives Budget (Reserve freigegeben)","Operatives Budget (abzgl. Reserve)")</f>
       </c>
-      <c r="C24" s="197"/>
-      <c r="D24" s="226" t="str">
+      <c r="C24" s="198"/>
+      <c r="D24" s="227" t="str">
         <f>=IF(Reserve_Freigabe="Ja",ROUND($D$22,2),ROUND($D$22-$D$23,2))</f>
       </c>
-      <c r="F24" s="233" t="s">
-        <v>352</v>
-      </c>
-      <c r="G24" s="197" t="s">
-        <v>354</v>
-      </c>
-      <c r="H24" s="197"/>
-      <c r="I24" s="234" t="str">
+      <c r="F24" s="234" t="s">
+        <v>353</v>
+      </c>
+      <c r="G24" s="198" t="s">
+        <v>355</v>
+      </c>
+      <c r="H24" s="198"/>
+      <c r="I24" s="235" t="str">
         <f>=I87</f>
         <v>0</v>
       </c>
       <c r="L24" s="143" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="M24" s="116" t="str">
         <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$C$21,'IV. MA'!$G$21,'IV. MA'!$K$21,'IV. MA'!$O$21,'IV. MA'!$S$21,'IV. MA'!$W$21,'IV. MA'!$AA$21,'IV. MA'!$AE$21,'IV. MA'!$AI$21,'IV. MA'!$AM$21,'IV. MA'!$AQ$21,'IV. MA'!$AU$21,'IV. MA'!$AY$21,'IV. MA'!$BC$21,'IV. MA'!$BG$21,'IV. MA'!$BK$21,'IV. MA'!$BO$21,'IV. MA'!$BS$21),"")</f>
@@ -21799,26 +21912,26 @@
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="205" t="s">
-        <v>349</v>
-      </c>
-      <c r="C25" s="197"/>
-      <c r="D25" s="226" t="str">
+      <c r="B25" s="206" t="s">
+        <v>350</v>
+      </c>
+      <c r="C25" s="198"/>
+      <c r="D25" s="227" t="str">
         <f>=IFERROR(ROUND(SUBTOTAL(109,TblKMWMittel[Betrag]),2),0)</f>
       </c>
-      <c r="F25" s="233" t="s">
-        <v>352</v>
-      </c>
-      <c r="G25" s="197" t="s">
-        <v>355</v>
-      </c>
-      <c r="H25" s="197"/>
-      <c r="I25" s="234" t="str">
+      <c r="F25" s="234" t="s">
+        <v>353</v>
+      </c>
+      <c r="G25" s="198" t="s">
+        <v>356</v>
+      </c>
+      <c r="H25" s="198"/>
+      <c r="I25" s="235" t="str">
         <f>=ROUND(MAX(0,MAX(0,(SUM($G$96:$G$99)-$G$98)+SUMIFS('Daten'!$BH$1:$BH$18,'Daten'!$BB$1:$BB$18,E10,'Daten'!$BD$1:$BD$18,"&lt;="&amp;E11,'Daten'!$BD$1:$BD$18,"&gt;=1")-(SUM($H$96:$H$99)-$H$98))-I87),2)</f>
         <v>0</v>
       </c>
       <c r="L25" s="143" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="M25" s="116" t="str">
         <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$C$22,'IV. MA'!$G$22,'IV. MA'!$K$22,'IV. MA'!$O$22,'IV. MA'!$S$22,'IV. MA'!$W$22,'IV. MA'!$AA$22,'IV. MA'!$AE$22,'IV. MA'!$AI$22,'IV. MA'!$AM$22,'IV. MA'!$AQ$22,'IV. MA'!$AU$22,'IV. MA'!$AY$22,'IV. MA'!$BC$22,'IV. MA'!$BG$22,'IV. MA'!$BK$22,'IV. MA'!$BO$22,'IV. MA'!$BS$22),"")</f>
@@ -21828,19 +21941,19 @@
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="227" t="s">
-        <v>350</v>
-      </c>
-      <c r="C26" s="228"/>
-      <c r="D26" s="229" t="str">
+      <c r="B26" s="228" t="s">
+        <v>351</v>
+      </c>
+      <c r="C26" s="229"/>
+      <c r="D26" s="230" t="str">
         <f>=ROUND($D$24-$D$25,2)</f>
       </c>
       <c r="F26" s="47"/>
-      <c r="G26" s="218" t="s">
-        <v>356</v>
-      </c>
-      <c r="H26" s="218"/>
-      <c r="I26" s="235" t="str">
+      <c r="G26" s="219" t="s">
+        <v>357</v>
+      </c>
+      <c r="H26" s="219"/>
+      <c r="I26" s="236" t="str">
         <f>=ROUND(IF($F$23="Abzug",MAX(0,$I$23),0)+IF($F$24="Abzug",MAX(0,$I$24),0)+IF($F$25="Abzug",MAX(0,$I$25),0),2)</f>
       </c>
       <c r="L26" s="143" t="str">
@@ -21854,12 +21967,12 @@
       </c>
     </row>
     <row r="27">
-      <c r="F27" s="236"/>
-      <c r="G27" s="228" t="s">
-        <v>357</v>
-      </c>
-      <c r="H27" s="228"/>
-      <c r="I27" s="229" t="str">
+      <c r="F27" s="237"/>
+      <c r="G27" s="229" t="s">
+        <v>358</v>
+      </c>
+      <c r="H27" s="229"/>
+      <c r="I27" s="230" t="str">
         <f>=ROUND($D$26-$I$26,2)</f>
       </c>
       <c r="L27" s="47"/>
@@ -21867,7 +21980,7 @@
     </row>
     <row r="28">
       <c r="L28" s="323" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="M28" s="324" t="str">
         <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$C$25,'IV. MA'!$G$25,'IV. MA'!$K$25,'IV. MA'!$O$25,'IV. MA'!$S$25,'IV. MA'!$W$25,'IV. MA'!$AA$25,'IV. MA'!$AE$25,'IV. MA'!$AI$25,'IV. MA'!$AM$25,'IV. MA'!$AQ$25,'IV. MA'!$AU$25,'IV. MA'!$AY$25,'IV. MA'!$BC$25,'IV. MA'!$BG$25,'IV. MA'!$BK$25,'IV. MA'!$BO$25,'IV. MA'!$BS$25),"")</f>
@@ -21877,72 +21990,76 @@
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="223" t="s">
-        <v>358</v>
-      </c>
-      <c r="C29" s="224"/>
-      <c r="D29" s="225" t="str">
+      <c r="B29" s="224" t="s">
+        <v>359</v>
+      </c>
+      <c r="C29" s="225"/>
+      <c r="D29" s="226" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"KMW-Mittel",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,E11),2),0)</f>
       </c>
-      <c r="F29" s="223" t="s">
-        <v>358</v>
-      </c>
-      <c r="G29" s="224"/>
-      <c r="H29" s="224"/>
-      <c r="I29" s="225" t="str">
+      <c r="F29" s="224" t="s">
+        <v>359</v>
+      </c>
+      <c r="G29" s="225"/>
+      <c r="H29" s="225"/>
+      <c r="I29" s="226" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"KMW-Mittel",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,E11),2),0)</f>
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="227" t="s">
-        <v>359</v>
-      </c>
-      <c r="C30" s="228"/>
-      <c r="D30" s="229" t="str">
+      <c r="B30" s="228" t="s">
+        <v>360</v>
+      </c>
+      <c r="C30" s="229"/>
+      <c r="D30" s="230" t="str">
         <f>=ROUND($D$26-MAX(0,$D$29),2)</f>
       </c>
-      <c r="F30" s="227" t="s">
+      <c r="F30" s="228" t="s">
+        <v>361</v>
+      </c>
+      <c r="G30" s="229"/>
+      <c r="H30" s="229"/>
+      <c r="I30" s="230" t="str">
+        <f>=ROUND($I$27-MAX(0,$I$29),2)</f>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="224" t="s">
+        <v>362</v>
+      </c>
+      <c r="C32" s="225"/>
+      <c r="D32" s="238" t="str">
+        <f>=IFERROR(CHOOSE(E10,MA_ManBetrag_1,MA_ManBetrag_2,MA_ManBetrag_3,MA_ManBetrag_4,MA_ManBetrag_5,MA_ManBetrag_6,MA_ManBetrag_7,MA_ManBetrag_8,MA_ManBetrag_9,MA_ManBetrag_10,MA_ManBetrag_11,MA_ManBetrag_12,MA_ManBetrag_13,MA_ManBetrag_14,MA_ManBetrag_15,MA_ManBetrag_16,MA_ManBetrag_17,MA_ManBetrag_18),0)</f>
+      </c>
+      <c r="F32" s="224" t="s">
+        <v>362</v>
+      </c>
+      <c r="G32" s="225"/>
+      <c r="H32" s="225"/>
+      <c r="I32" s="238" t="str">
+        <f>=IFERROR(CHOOSE(E10,MA_ManBetrag_1,MA_ManBetrag_2,MA_ManBetrag_3,MA_ManBetrag_4,MA_ManBetrag_5,MA_ManBetrag_6,MA_ManBetrag_7,MA_ManBetrag_8,MA_ManBetrag_9,MA_ManBetrag_10,MA_ManBetrag_11,MA_ManBetrag_12,MA_ManBetrag_13,MA_ManBetrag_14,MA_ManBetrag_15,MA_ManBetrag_16,MA_ManBetrag_17,MA_ManBetrag_18),0)</f>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="228" t="s">
         <v>360</v>
       </c>
-      <c r="G30" s="228"/>
-      <c r="H30" s="228"/>
-      <c r="I30" s="229" t="str">
-        <f>=ROUND($I$27-MAX(0,$I$29),2)</f>
-      </c>
-    </row>
-    <row r="32">
-      <c r="B32" s="223" t="s">
+      <c r="C33" s="229"/>
+      <c r="D33" s="230" t="str">
+        <f>=ROUND($D$26-MAX(0,$D$29)-MAX(0,$D$32),2)</f>
+      </c>
+      <c r="F33" s="228" t="s">
         <v>361</v>
       </c>
-      <c r="C32" s="224"/>
-      <c r="D32" s="237"/>
-      <c r="F32" s="223" t="s">
-        <v>361</v>
-      </c>
-      <c r="G32" s="224"/>
-      <c r="H32" s="224"/>
-      <c r="I32" s="237"/>
-    </row>
-    <row r="33">
-      <c r="B33" s="227" t="s">
-        <v>359</v>
-      </c>
-      <c r="C33" s="228"/>
-      <c r="D33" s="229" t="str">
-        <f>=ROUND($D$26-MAX(0,$D$29)-MAX(0,$D$32),2)</f>
-      </c>
-      <c r="F33" s="227" t="s">
-        <v>360</v>
-      </c>
-      <c r="G33" s="228"/>
-      <c r="H33" s="228"/>
-      <c r="I33" s="229" t="str">
+      <c r="G33" s="229"/>
+      <c r="H33" s="229"/>
+      <c r="I33" s="230" t="str">
         <f>=ROUND($I$27-MAX(0,$I$29)-MAX(0,$I$32),2)</f>
       </c>
     </row>
     <row r="36" ht="22" customHeight="true">
       <c r="B36" s="18" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C36" s="18"/>
       <c r="D36" s="18"/>
@@ -21958,72 +22075,72 @@
         <v>158</v>
       </c>
       <c r="C38" s="247" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="D38" s="247" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="E38" s="248" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="205" t="s">
-        <v>366</v>
-      </c>
-      <c r="C39" s="239" t="str">
+      <c r="B39" s="206" t="s">
+        <v>367</v>
+      </c>
+      <c r="C39" s="240" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BF$1:$BF$18,'Daten'!$BB$1:$BB$18,E10,'Daten'!$BD$1:$BD$18,"&lt;="&amp;E11,'Daten'!$BD$1:$BD$18,"&gt;=1"),2),0)</f>
       </c>
-      <c r="D39" s="240"/>
-      <c r="E39" s="226" t="str">
+      <c r="D39" s="189"/>
+      <c r="E39" s="227" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BG$1:$BG$18,'Daten'!$BB$1:$BB$18,E10,'Daten'!$BD$1:$BD$18,"&lt;="&amp;E11,'Daten'!$BD$1:$BD$18,"&gt;=1"),2),0)</f>
       </c>
     </row>
     <row r="40">
-      <c r="B40" s="205" t="s">
-        <v>367</v>
-      </c>
-      <c r="C40" s="239" t="str">
+      <c r="B40" s="206" t="s">
+        <v>368</v>
+      </c>
+      <c r="C40" s="240" t="str">
         <f>=IFERROR(ROUND(SUBTOTAL(109,TblBudgetAusgaben[Jahr 1]),2),0)</f>
       </c>
       <c r="D40" s="241">
         <v>8</v>
       </c>
-      <c r="E40" s="226" t="str">
+      <c r="E40" s="227" t="str">
         <f>=IFERROR(ROUND($C$40/Budget_Kurs,2),0)</f>
       </c>
     </row>
     <row r="41">
-      <c r="B41" s="205" t="s">
-        <v>368</v>
-      </c>
-      <c r="C41" s="239" t="str">
+      <c r="B41" s="206" t="s">
+        <v>369</v>
+      </c>
+      <c r="C41" s="240" t="str">
         <f>=IFERROR(ROUND(SUBTOTAL(109,TblBudgetAusgaben[Jahr 2]),2),0)</f>
       </c>
       <c r="D41" s="241">
         <v>0</v>
       </c>
-      <c r="E41" s="226" t="str">
+      <c r="E41" s="227" t="str">
         <f>=IFERROR(ROUND($C$41/Budget_Kurs,2),0)</f>
       </c>
     </row>
     <row r="42">
-      <c r="B42" s="205" t="s">
-        <v>369</v>
-      </c>
-      <c r="C42" s="239" t="str">
+      <c r="B42" s="206" t="s">
+        <v>370</v>
+      </c>
+      <c r="C42" s="240" t="str">
         <f>=IFERROR(ROUND(SUBTOTAL(109,TblBudgetAusgaben[Jahr 3]),2),0)</f>
       </c>
       <c r="D42" s="241">
         <v>0</v>
       </c>
-      <c r="E42" s="226" t="str">
+      <c r="E42" s="227" t="str">
         <f>=IFERROR(ROUND($C$42/Budget_Kurs,2),0)</f>
       </c>
     </row>
     <row r="43">
-      <c r="B43" s="205" t="s">
-        <v>370</v>
+      <c r="B43" s="206" t="s">
+        <v>371</v>
       </c>
       <c r="C43" s="242" t="str">
         <f>=$D$40+$D$41+$D$42</f>
@@ -22032,8 +22149,8 @@
       <c r="E43" s="249"/>
     </row>
     <row r="44">
-      <c r="B44" s="205" t="s">
-        <v>371</v>
+      <c r="B44" s="206" t="s">
+        <v>372</v>
       </c>
       <c r="C44" s="242" t="str">
         <f>=IFERROR(CHOOSE(IFERROR(SUMPRODUCT('Daten'!$BA$1:$BA$18,('Daten'!$BB$1:$BB$18=E10)*('Daten'!$BD$1:$BD$18=E11)),0),'IV. MA'!$C$7,'IV. MA'!$G$7,'IV. MA'!$K$7,'IV. MA'!$O$7,'IV. MA'!$S$7,'IV. MA'!$W$7,'IV. MA'!$AA$7,'IV. MA'!$AE$7,'IV. MA'!$AI$7,'IV. MA'!$AM$7,'IV. MA'!$AQ$7,'IV. MA'!$AU$7,'IV. MA'!$AY$7,'IV. MA'!$BC$7,'IV. MA'!$BG$7,'IV. MA'!$BK$7,'IV. MA'!$BO$7,'IV. MA'!$BS$7),0)</f>
@@ -22043,43 +22160,43 @@
     </row>
     <row r="45">
       <c r="B45" s="251" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C45" s="243" t="str">
         <f>=IFERROR(ROUND($C$40*$D$40/12+$C$41*$D$41/12+$C$42*$D$42/12,2),0)</f>
       </c>
-      <c r="D45" s="240"/>
-      <c r="E45" s="235" t="str">
+      <c r="D45" s="189"/>
+      <c r="E45" s="236" t="str">
         <f>=IFERROR(ROUND($E$40*$D$40/12+$E$41*$D$41/12+$E$42*$D$42/12,2),0)</f>
       </c>
     </row>
     <row r="46">
       <c r="B46" s="251" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C46" s="244" t="str">
         <f>=IF($C$39&lt;=$C$45,"OK","ÜBERSCHRITTEN")</f>
       </c>
-      <c r="D46" s="240"/>
+      <c r="D46" s="189"/>
       <c r="E46" s="252" t="str">
         <f>=IF($E$39&lt;=$E$45,"OK","ÜBERSCHRITTEN")</f>
       </c>
     </row>
     <row r="47">
-      <c r="B47" s="205" t="s">
-        <v>374</v>
-      </c>
-      <c r="C47" s="239" t="str">
+      <c r="B47" s="206" t="s">
+        <v>375</v>
+      </c>
+      <c r="C47" s="240" t="str">
         <f>=ROUND(MAX(0,$C$39-$C$45),2)</f>
       </c>
-      <c r="D47" s="240"/>
-      <c r="E47" s="226" t="str">
+      <c r="D47" s="189"/>
+      <c r="E47" s="227" t="str">
         <f>=ROUND(MAX(0,$E$39-$E$45),2)</f>
       </c>
     </row>
     <row r="48">
       <c r="B48" s="253" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C48" s="254" t="str">
         <f>=IFERROR($C$39/$C$45,0)</f>
@@ -22091,7 +22208,7 @@
     </row>
     <row r="50" ht="22" customHeight="true">
       <c r="B50" s="18" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C50" s="18"/>
       <c r="D50" s="18"/>
@@ -22104,53 +22221,53 @@
     </row>
     <row r="52" ht="28" customHeight="true">
       <c r="B52" s="263" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C52" s="264" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="D52" s="264" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="E52" s="264" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="F52" s="264" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="G52" s="264" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="H52" s="264" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="I52" s="264" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="J52" s="265" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="53">
       <c r="B53" s="266" t="s">
         <v>194</v>
       </c>
-      <c r="C53" s="239" t="str">
+      <c r="C53" s="240" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"Eigenmittel",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="D53" s="239" t="str">
+      <c r="D53" s="240" t="str">
         <f>=IFERROR(ROUND(Eigenmittel_LW,2),0)</f>
       </c>
-      <c r="E53" s="201" t="str">
+      <c r="E53" s="202" t="str">
         <f>=ROUND(IFERROR($C$53-$D$53,0),2)</f>
       </c>
       <c r="F53" s="258" t="str">
         <f>=ROUND(IFERROR(($C$53/$D$53)-1,0),4)</f>
       </c>
-      <c r="G53" s="217" t="str">
+      <c r="G53" s="218" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"Eigenmittel",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="H53" s="217" t="str">
+      <c r="H53" s="218" t="str">
         <f>=IFERROR(ROUND(Eigenmittel_EUR,2),0)</f>
       </c>
       <c r="I53" s="182" t="str">
@@ -22164,22 +22281,22 @@
       <c r="B54" s="266" t="s">
         <v>300</v>
       </c>
-      <c r="C54" s="239" t="str">
+      <c r="C54" s="240" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"Drittmittel",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="D54" s="239" t="str">
+      <c r="D54" s="240" t="str">
         <f>=IFERROR(ROUND(Drittmittel_LW,2),0)</f>
       </c>
-      <c r="E54" s="201" t="str">
+      <c r="E54" s="202" t="str">
         <f>=ROUND(IFERROR($C$54-$D$54,0),2)</f>
       </c>
       <c r="F54" s="258" t="str">
         <f>=ROUND(IFERROR(($C$54/$D$54)-1,0),4)</f>
       </c>
-      <c r="G54" s="217" t="str">
+      <c r="G54" s="218" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"Drittmittel",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="H54" s="217" t="str">
+      <c r="H54" s="218" t="str">
         <f>=IFERROR(ROUND(Drittmittel_EUR,2),0)</f>
       </c>
       <c r="I54" s="182" t="str">
@@ -22193,22 +22310,22 @@
       <c r="B55" s="266" t="s">
         <v>199</v>
       </c>
-      <c r="C55" s="239" t="str">
+      <c r="C55" s="240" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"KMW-Mittel",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="D55" s="239" t="str">
+      <c r="D55" s="240" t="str">
         <f>=IFERROR(ROUND(KMW_Mittel_LW,2),0)</f>
       </c>
-      <c r="E55" s="201" t="str">
+      <c r="E55" s="202" t="str">
         <f>=ROUND(IFERROR($C$55-$D$55,0),2)</f>
       </c>
       <c r="F55" s="258" t="str">
         <f>=ROUND(IFERROR(($C$55/$D$55)-1,0),4)</f>
       </c>
-      <c r="G55" s="217" t="str">
+      <c r="G55" s="218" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"KMW-Mittel",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="H55" s="217" t="str">
+      <c r="H55" s="218" t="str">
         <f>=IFERROR(ROUND(KMW_Mittel_EUR,2),0)</f>
       </c>
       <c r="I55" s="182" t="str">
@@ -22222,22 +22339,22 @@
       <c r="B56" s="266" t="s">
         <v>301</v>
       </c>
-      <c r="C56" s="239" t="str">
+      <c r="C56" s="240" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"Zinsertraege",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="D56" s="239" t="str">
+      <c r="D56" s="240" t="str">
         <f>=IFERROR(ROUND(0,2),0)</f>
       </c>
-      <c r="E56" s="201" t="str">
+      <c r="E56" s="202" t="str">
         <f>=ROUND(IFERROR($C$56-$D$56,0),2)</f>
       </c>
       <c r="F56" s="258" t="str">
         <f>=ROUND(IFERROR(($C$56/$D$56)-1,0),4)</f>
       </c>
-      <c r="G56" s="217" t="str">
+      <c r="G56" s="218" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"Zinsertraege",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="H56" s="217" t="str">
+      <c r="H56" s="218" t="str">
         <f>=IFERROR(ROUND(0,2),0)</f>
       </c>
       <c r="I56" s="182" t="str">
@@ -22278,7 +22395,7 @@
     </row>
     <row r="59" ht="22" customHeight="true">
       <c r="B59" s="18" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C59" s="18"/>
       <c r="D59" s="18"/>
@@ -22291,53 +22408,53 @@
     </row>
     <row r="61" ht="28" customHeight="true">
       <c r="B61" s="263" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C61" s="264" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="D61" s="264" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="E61" s="264" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="F61" s="264" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="G61" s="264" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="H61" s="264" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="I61" s="264" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="J61" s="265" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="62">
       <c r="B62" s="266" t="s">
         <v>205</v>
       </c>
-      <c r="C62" s="239" t="str">
+      <c r="C62" s="240" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"Bauausgaben",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="D62" s="239" t="str">
+      <c r="D62" s="240" t="str">
         <f>=IFERROR(ROUND(Kosten_Bauausgaben_LW,2),0)</f>
       </c>
-      <c r="E62" s="201" t="str">
+      <c r="E62" s="202" t="str">
         <f>=ROUND(IFERROR($C$62-$D$62,0),2)</f>
       </c>
       <c r="F62" s="258" t="str">
         <f>=ROUND(IFERROR(($C$62/$D$62)-1,0),4)</f>
       </c>
-      <c r="G62" s="217" t="str">
+      <c r="G62" s="218" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"Bauausgaben",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="H62" s="217" t="str">
+      <c r="H62" s="218" t="str">
         <f>=IFERROR(ROUND(Kosten_Bauausgaben_EUR,2),0)</f>
       </c>
       <c r="I62" s="182" t="str">
@@ -22351,22 +22468,22 @@
       <c r="B63" s="266" t="s">
         <v>210</v>
       </c>
-      <c r="C63" s="239" t="str">
+      <c r="C63" s="240" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"Investitionen",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="D63" s="239" t="str">
+      <c r="D63" s="240" t="str">
         <f>=IFERROR(ROUND(Kosten_Investitionen_LW,2),0)</f>
       </c>
-      <c r="E63" s="201" t="str">
+      <c r="E63" s="202" t="str">
         <f>=ROUND(IFERROR($C$63-$D$63,0),2)</f>
       </c>
       <c r="F63" s="258" t="str">
         <f>=ROUND(IFERROR(($C$63/$D$63)-1,0),4)</f>
       </c>
-      <c r="G63" s="217" t="str">
+      <c r="G63" s="218" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"Investitionen",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="H63" s="217" t="str">
+      <c r="H63" s="218" t="str">
         <f>=IFERROR(ROUND(Kosten_Investitionen_EUR,2),0)</f>
       </c>
       <c r="I63" s="182" t="str">
@@ -22380,22 +22497,22 @@
       <c r="B64" s="266" t="s">
         <v>213</v>
       </c>
-      <c r="C64" s="239" t="str">
+      <c r="C64" s="240" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"Personalkosten",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="D64" s="239" t="str">
+      <c r="D64" s="240" t="str">
         <f>=IFERROR(ROUND(Kosten_Personalkosten_LW,2),0)</f>
       </c>
-      <c r="E64" s="201" t="str">
+      <c r="E64" s="202" t="str">
         <f>=ROUND(IFERROR($C$64-$D$64,0),2)</f>
       </c>
       <c r="F64" s="258" t="str">
         <f>=ROUND(IFERROR(($C$64/$D$64)-1,0),4)</f>
       </c>
-      <c r="G64" s="217" t="str">
+      <c r="G64" s="218" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"Personalkosten",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="H64" s="217" t="str">
+      <c r="H64" s="218" t="str">
         <f>=IFERROR(ROUND(Kosten_Personalkosten_EUR,2),0)</f>
       </c>
       <c r="I64" s="182" t="str">
@@ -22409,22 +22526,22 @@
       <c r="B65" s="266" t="s">
         <v>218</v>
       </c>
-      <c r="C65" s="239" t="str">
+      <c r="C65" s="240" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"Projektaktivitaeten",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="D65" s="239" t="str">
+      <c r="D65" s="240" t="str">
         <f>=IFERROR(ROUND(Kosten_Projektaktivitaeten_LW,2),0)</f>
       </c>
-      <c r="E65" s="201" t="str">
+      <c r="E65" s="202" t="str">
         <f>=ROUND(IFERROR($C$65-$D$65,0),2)</f>
       </c>
       <c r="F65" s="258" t="str">
         <f>=ROUND(IFERROR(($C$65/$D$65)-1,0),4)</f>
       </c>
-      <c r="G65" s="217" t="str">
+      <c r="G65" s="218" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"Projektaktivitaeten",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="H65" s="217" t="str">
+      <c r="H65" s="218" t="str">
         <f>=IFERROR(ROUND(Kosten_Projektaktivitaeten_EUR,2),0)</f>
       </c>
       <c r="I65" s="182" t="str">
@@ -22438,22 +22555,22 @@
       <c r="B66" s="266" t="s">
         <v>221</v>
       </c>
-      <c r="C66" s="239" t="str">
+      <c r="C66" s="240" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"Projektverwaltung",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="D66" s="239" t="str">
+      <c r="D66" s="240" t="str">
         <f>=IFERROR(ROUND(Kosten_Projektverwaltung_LW,2),0)</f>
       </c>
-      <c r="E66" s="201" t="str">
+      <c r="E66" s="202" t="str">
         <f>=ROUND(IFERROR($C$66-$D$66,0),2)</f>
       </c>
       <c r="F66" s="258" t="str">
         <f>=ROUND(IFERROR(($C$66/$D$66)-1,0),4)</f>
       </c>
-      <c r="G66" s="217" t="str">
+      <c r="G66" s="218" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"Projektverwaltung",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="H66" s="217" t="str">
+      <c r="H66" s="218" t="str">
         <f>=IFERROR(ROUND(Kosten_Projektverwaltung_EUR,2),0)</f>
       </c>
       <c r="I66" s="182" t="str">
@@ -22467,22 +22584,22 @@
       <c r="B67" s="266" t="s">
         <v>224</v>
       </c>
-      <c r="C67" s="239" t="str">
+      <c r="C67" s="240" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"Evaluierung",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="D67" s="239" t="str">
+      <c r="D67" s="240" t="str">
         <f>=IFERROR(ROUND(Kosten_Evaluierung_LW,2),0)</f>
       </c>
-      <c r="E67" s="201" t="str">
+      <c r="E67" s="202" t="str">
         <f>=ROUND(IFERROR($C$67-$D$67,0),2)</f>
       </c>
       <c r="F67" s="258" t="str">
         <f>=ROUND(IFERROR(($C$67/$D$67)-1,0),4)</f>
       </c>
-      <c r="G67" s="217" t="str">
+      <c r="G67" s="218" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"Evaluierung",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="H67" s="217" t="str">
+      <c r="H67" s="218" t="str">
         <f>=IFERROR(ROUND(Kosten_Evaluierung_EUR,2),0)</f>
       </c>
       <c r="I67" s="182" t="str">
@@ -22496,22 +22613,22 @@
       <c r="B68" s="266" t="s">
         <v>227</v>
       </c>
-      <c r="C68" s="239" t="str">
+      <c r="C68" s="240" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"Audit",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="D68" s="239" t="str">
+      <c r="D68" s="240" t="str">
         <f>=IFERROR(ROUND(Kosten_Audit_LW,2),0)</f>
       </c>
-      <c r="E68" s="201" t="str">
+      <c r="E68" s="202" t="str">
         <f>=ROUND(IFERROR($C$68-$D$68,0),2)</f>
       </c>
       <c r="F68" s="258" t="str">
         <f>=ROUND(IFERROR(($C$68/$D$68)-1,0),4)</f>
       </c>
-      <c r="G68" s="217" t="str">
+      <c r="G68" s="218" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"Audit",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="H68" s="217" t="str">
+      <c r="H68" s="218" t="str">
         <f>=IFERROR(ROUND(Kosten_Audit_EUR,2),0)</f>
       </c>
       <c r="I68" s="182" t="str">
@@ -22525,22 +22642,22 @@
       <c r="B69" s="266" t="s">
         <v>230</v>
       </c>
-      <c r="C69" s="239" t="str">
+      <c r="C69" s="240" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"Reserve",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="D69" s="239" t="str">
+      <c r="D69" s="240" t="str">
         <f>=IFERROR(ROUND(Kosten_Reserve_LW,2),0)</f>
       </c>
-      <c r="E69" s="201" t="str">
+      <c r="E69" s="202" t="str">
         <f>=ROUND(IFERROR($C$69-$D$69,0),2)</f>
       </c>
       <c r="F69" s="258" t="str">
         <f>=ROUND(IFERROR(($C$69/$D$69)-1,0),4)</f>
       </c>
-      <c r="G69" s="217" t="str">
+      <c r="G69" s="218" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"Reserve",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="H69" s="217" t="str">
+      <c r="H69" s="218" t="str">
         <f>=IFERROR(ROUND(Kosten_Reserve_EUR,2),0)</f>
       </c>
       <c r="I69" s="182" t="str">
@@ -22580,37 +22697,37 @@
       </c>
     </row>
     <row r="76" ht="22" customHeight="true">
-      <c r="B76" s="194" t="s">
-        <v>387</v>
-      </c>
-      <c r="C76" s="194"/>
-      <c r="D76" s="194"/>
-      <c r="E76" s="194"/>
-      <c r="F76" s="194"/>
-      <c r="G76" s="194"/>
-      <c r="H76" s="194"/>
-      <c r="I76" s="194"/>
-      <c r="J76" s="194"/>
-      <c r="L76" s="202" t="str">
+      <c r="B76" s="195" t="s">
+        <v>388</v>
+      </c>
+      <c r="C76" s="195"/>
+      <c r="D76" s="195"/>
+      <c r="E76" s="195"/>
+      <c r="F76" s="195"/>
+      <c r="G76" s="195"/>
+      <c r="H76" s="195"/>
+      <c r="I76" s="195"/>
+      <c r="J76" s="195"/>
+      <c r="L76" s="203" t="str">
         <f>=IF(E81=0,"Aktueller Finanzbericht (keiner gewählt)","Aktueller Finanzbericht – Periode "&amp;E81)</f>
       </c>
-      <c r="M76" s="203"/>
-      <c r="N76" s="203"/>
-      <c r="O76" s="203"/>
-      <c r="P76" s="204"/>
+      <c r="M76" s="204"/>
+      <c r="N76" s="204"/>
+      <c r="O76" s="204"/>
+      <c r="P76" s="205"/>
     </row>
     <row r="77">
-      <c r="B77" s="195" t="s">
-        <v>388</v>
-      </c>
-      <c r="C77" s="195"/>
-      <c r="D77" s="195"/>
-      <c r="E77" s="195"/>
-      <c r="F77" s="195"/>
-      <c r="G77" s="195"/>
-      <c r="H77" s="195"/>
-      <c r="I77" s="195"/>
-      <c r="J77" s="195"/>
+      <c r="B77" s="196" t="s">
+        <v>389</v>
+      </c>
+      <c r="C77" s="196"/>
+      <c r="D77" s="196"/>
+      <c r="E77" s="196"/>
+      <c r="F77" s="196"/>
+      <c r="G77" s="196"/>
+      <c r="H77" s="196"/>
+      <c r="I77" s="196"/>
+      <c r="J77" s="196"/>
       <c r="L77" s="315" t="s">
         <v>288</v>
       </c>
@@ -22633,13 +22750,13 @@
       <c r="P78" s="338"/>
     </row>
     <row r="79" ht="22" customHeight="true">
-      <c r="C79" s="202" t="s">
-        <v>389</v>
-      </c>
-      <c r="D79" s="203"/>
-      <c r="E79" s="203"/>
-      <c r="F79" s="203"/>
-      <c r="G79" s="204"/>
+      <c r="C79" s="203" t="s">
+        <v>390</v>
+      </c>
+      <c r="D79" s="204"/>
+      <c r="E79" s="204"/>
+      <c r="F79" s="204"/>
+      <c r="G79" s="205"/>
       <c r="L79" s="315" t="s">
         <v>290</v>
       </c>
@@ -22651,15 +22768,15 @@
       <c r="P79" s="338"/>
     </row>
     <row r="80">
-      <c r="C80" s="205" t="s">
-        <v>341</v>
-      </c>
-      <c r="D80" s="197"/>
+      <c r="C80" s="206" t="s">
+        <v>342</v>
+      </c>
+      <c r="D80" s="198"/>
       <c r="E80" s="63" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="F80" s="63"/>
-      <c r="G80" s="206"/>
+      <c r="G80" s="207"/>
       <c r="L80" s="315" t="s">
         <v>291</v>
       </c>
@@ -22672,7 +22789,7 @@
     </row>
     <row r="81">
       <c r="C81" s="253" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="D81" s="286"/>
       <c r="E81" s="287" t="str">
@@ -22696,7 +22813,7 @@
     </row>
     <row r="83" ht="22" customHeight="true">
       <c r="B83" s="18" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C83" s="18"/>
       <c r="D83" s="18"/>
@@ -22732,19 +22849,19 @@
       </c>
     </row>
     <row r="85">
-      <c r="B85" s="223" t="s">
-        <v>347</v>
-      </c>
-      <c r="C85" s="224"/>
-      <c r="D85" s="225" t="str">
+      <c r="B85" s="224" t="s">
+        <v>348</v>
+      </c>
+      <c r="C85" s="225"/>
+      <c r="D85" s="226" t="str">
         <f>=IFERROR(ROUND(KMW_Mittel_EUR,2),0)</f>
       </c>
-      <c r="F85" s="230" t="s">
-        <v>351</v>
-      </c>
-      <c r="G85" s="231"/>
-      <c r="H85" s="231"/>
-      <c r="I85" s="232"/>
+      <c r="F85" s="231" t="s">
+        <v>352</v>
+      </c>
+      <c r="G85" s="232"/>
+      <c r="H85" s="232"/>
+      <c r="I85" s="233"/>
       <c r="L85" s="143" t="str">
         <f>=IFERROR(CHOOSE(E81,'III. Finanzberichte'!$B$11,'III. Finanzberichte'!$I$11,'III. Finanzberichte'!$P$11,'III. Finanzberichte'!$W$11,'III. Finanzberichte'!$AD$11,'III. Finanzberichte'!$AK$11,'III. Finanzberichte'!$AR$11,'III. Finanzberichte'!$AY$11,'III. Finanzberichte'!$BF$11,'III. Finanzberichte'!$BM$11,'III. Finanzberichte'!$BT$11,'III. Finanzberichte'!$CA$11,'III. Finanzberichte'!$CH$11,'III. Finanzberichte'!$CO$11,'III. Finanzberichte'!$CV$11,'III. Finanzberichte'!$DC$11,'III. Finanzberichte'!$DJ$11,'III. Finanzberichte'!$DQ$11),"")</f>
       </c>
@@ -22762,21 +22879,21 @@
       </c>
     </row>
     <row r="86">
-      <c r="B86" s="205" t="s">
-        <v>348</v>
-      </c>
-      <c r="C86" s="197"/>
-      <c r="D86" s="226" t="str">
+      <c r="B86" s="206" t="s">
+        <v>349</v>
+      </c>
+      <c r="C86" s="198"/>
+      <c r="D86" s="227" t="str">
         <f>=IFERROR(ROUND(Kosten_Reserve_EUR,2),0)</f>
       </c>
-      <c r="F86" s="233" t="s">
-        <v>352</v>
-      </c>
-      <c r="G86" s="197" t="s">
+      <c r="F86" s="234" t="s">
         <v>353</v>
       </c>
-      <c r="H86" s="197"/>
-      <c r="I86" s="234" t="str">
+      <c r="G86" s="198" t="s">
+        <v>354</v>
+      </c>
+      <c r="H86" s="198"/>
+      <c r="I86" s="235" t="str">
         <f>=IFERROR(ROUND(Saldovortrag_EUR,2),0)</f>
       </c>
       <c r="L86" s="143" t="s">
@@ -22796,21 +22913,21 @@
       </c>
     </row>
     <row r="87">
-      <c r="B87" s="205" t="str">
+      <c r="B87" s="206" t="str">
         <f>=IF(Reserve_Freigabe="Ja","Operatives Budget (Reserve freigegeben)","Operatives Budget (abzgl. Reserve)")</f>
       </c>
-      <c r="C87" s="197"/>
-      <c r="D87" s="226" t="str">
+      <c r="C87" s="198"/>
+      <c r="D87" s="227" t="str">
         <f>=IF(Reserve_Freigabe="Ja",ROUND($D$85,2),ROUND($D$85-$D$86,2))</f>
       </c>
-      <c r="F87" s="233" t="s">
-        <v>352</v>
-      </c>
-      <c r="G87" s="197" t="s">
-        <v>354</v>
-      </c>
-      <c r="H87" s="197"/>
-      <c r="I87" s="234" t="str">
+      <c r="F87" s="234" t="s">
+        <v>353</v>
+      </c>
+      <c r="G87" s="198" t="s">
+        <v>355</v>
+      </c>
+      <c r="H87" s="198"/>
+      <c r="I87" s="235" t="str">
         <f>=IFERROR(ROUND(MAX(0,(SUM($G$96:$G$99)-$G$98)-(SUM($H$96:$H$99)-$H$98)),2),0)</f>
         <v>0</v>
       </c>
@@ -22831,19 +22948,19 @@
       </c>
     </row>
     <row r="88">
-      <c r="B88" s="205" t="s">
-        <v>349</v>
-      </c>
-      <c r="C88" s="197"/>
-      <c r="D88" s="226" t="str">
+      <c r="B88" s="206" t="s">
+        <v>350</v>
+      </c>
+      <c r="C88" s="198"/>
+      <c r="D88" s="227" t="str">
         <f>=IFERROR(ROUND(SUBTOTAL(109,TblKMWMittel[Betrag]),2),0)</f>
       </c>
       <c r="F88" s="47"/>
-      <c r="G88" s="218" t="s">
-        <v>356</v>
-      </c>
-      <c r="H88" s="218"/>
-      <c r="I88" s="235" t="str">
+      <c r="G88" s="219" t="s">
+        <v>357</v>
+      </c>
+      <c r="H88" s="219"/>
+      <c r="I88" s="236" t="str">
         <f>=ROUND(IF($F$86="Abzug",MAX(0,$I$86),0)+IF($F$87="Abzug",MAX(0,$I$87),0),2)</f>
       </c>
       <c r="L88" s="143" t="s">
@@ -22863,19 +22980,19 @@
       </c>
     </row>
     <row r="89">
-      <c r="B89" s="227" t="s">
-        <v>350</v>
-      </c>
-      <c r="C89" s="228"/>
-      <c r="D89" s="229" t="str">
+      <c r="B89" s="228" t="s">
+        <v>351</v>
+      </c>
+      <c r="C89" s="229"/>
+      <c r="D89" s="230" t="str">
         <f>=ROUND($D$87-$D$88,2)</f>
       </c>
-      <c r="F89" s="236"/>
-      <c r="G89" s="228" t="s">
-        <v>357</v>
-      </c>
-      <c r="H89" s="228"/>
-      <c r="I89" s="229" t="str">
+      <c r="F89" s="237"/>
+      <c r="G89" s="229" t="s">
+        <v>358</v>
+      </c>
+      <c r="H89" s="229"/>
+      <c r="I89" s="230" t="str">
         <f>=ROUND($D$89-$I$88,2)</f>
       </c>
       <c r="L89" s="143" t="s">
@@ -22939,7 +23056,7 @@
     </row>
     <row r="93" ht="22" customHeight="true">
       <c r="B93" s="18" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C93" s="18"/>
       <c r="D93" s="18"/>
@@ -22984,31 +23101,31 @@
     </row>
     <row r="95" ht="28" customHeight="true">
       <c r="B95" s="263" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C95" s="264" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="D95" s="264" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="E95" s="264" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="F95" s="264" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="G95" s="264" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="H95" s="264" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="I95" s="264" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="J95" s="265" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="L95" s="143" t="str">
         <f>=IFERROR(CHOOSE(E81,'III. Finanzberichte'!$B$21,'III. Finanzberichte'!$I$21,'III. Finanzberichte'!$P$21,'III. Finanzberichte'!$W$21,'III. Finanzberichte'!$AD$21,'III. Finanzberichte'!$AK$21,'III. Finanzberichte'!$AR$21,'III. Finanzberichte'!$AY$21,'III. Finanzberichte'!$BF$21,'III. Finanzberichte'!$BM$21,'III. Finanzberichte'!$BT$21,'III. Finanzberichte'!$CA$21,'III. Finanzberichte'!$CH$21,'III. Finanzberichte'!$CO$21,'III. Finanzberichte'!$CV$21,'III. Finanzberichte'!$DC$21,'III. Finanzberichte'!$DJ$21,'III. Finanzberichte'!$DQ$21),"")</f>
@@ -23030,22 +23147,22 @@
       <c r="B96" s="266" t="s">
         <v>194</v>
       </c>
-      <c r="C96" s="239" t="str">
+      <c r="C96" s="240" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$E$12,'III. Finanzberichte'!$L$12,'III. Finanzberichte'!$S$12,'III. Finanzberichte'!$Z$12,'III. Finanzberichte'!$AG$12,'III. Finanzberichte'!$AN$12,'III. Finanzberichte'!$AU$12,'III. Finanzberichte'!$BB$12,'III. Finanzberichte'!$BI$12,'III. Finanzberichte'!$BP$12,'III. Finanzberichte'!$BW$12,'III. Finanzberichte'!$CD$12,'III. Finanzberichte'!$CK$12,'III. Finanzberichte'!$CR$12,'III. Finanzberichte'!$CY$12,'III. Finanzberichte'!$DF$12,'III. Finanzberichte'!$DM$12,'III. Finanzberichte'!$DT$12),2),0)</f>
       </c>
-      <c r="D96" s="239" t="str">
+      <c r="D96" s="240" t="str">
         <f>=IFERROR(ROUND(Eigenmittel_LW,2),0)</f>
       </c>
-      <c r="E96" s="201" t="str">
+      <c r="E96" s="202" t="str">
         <f>=ROUND(IFERROR($C$96-$D$96,0),2)</f>
       </c>
       <c r="F96" s="258" t="str">
         <f>=ROUND(IFERROR(($C$96/$D$96)-1,0),4)</f>
       </c>
-      <c r="G96" s="217" t="str">
+      <c r="G96" s="218" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$F$12,'III. Finanzberichte'!$M$12,'III. Finanzberichte'!$T$12,'III. Finanzberichte'!$AA$12,'III. Finanzberichte'!$AH$12,'III. Finanzberichte'!$AO$12,'III. Finanzberichte'!$AV$12,'III. Finanzberichte'!$BC$12,'III. Finanzberichte'!$BJ$12,'III. Finanzberichte'!$BQ$12,'III. Finanzberichte'!$BX$12,'III. Finanzberichte'!$CE$12,'III. Finanzberichte'!$CL$12,'III. Finanzberichte'!$CS$12,'III. Finanzberichte'!$CZ$12,'III. Finanzberichte'!$DG$12,'III. Finanzberichte'!$DN$12,'III. Finanzberichte'!$DU$12),2),0)</f>
       </c>
-      <c r="H96" s="217" t="str">
+      <c r="H96" s="218" t="str">
         <f>=IFERROR(ROUND(Eigenmittel_EUR,2),0)</f>
       </c>
       <c r="I96" s="182" t="str">
@@ -23074,22 +23191,22 @@
       <c r="B97" s="266" t="s">
         <v>300</v>
       </c>
-      <c r="C97" s="239" t="str">
+      <c r="C97" s="240" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$E$13,'III. Finanzberichte'!$L$13,'III. Finanzberichte'!$S$13,'III. Finanzberichte'!$Z$13,'III. Finanzberichte'!$AG$13,'III. Finanzberichte'!$AN$13,'III. Finanzberichte'!$AU$13,'III. Finanzberichte'!$BB$13,'III. Finanzberichte'!$BI$13,'III. Finanzberichte'!$BP$13,'III. Finanzberichte'!$BW$13,'III. Finanzberichte'!$CD$13,'III. Finanzberichte'!$CK$13,'III. Finanzberichte'!$CR$13,'III. Finanzberichte'!$CY$13,'III. Finanzberichte'!$DF$13,'III. Finanzberichte'!$DM$13,'III. Finanzberichte'!$DT$13),2),0)</f>
       </c>
-      <c r="D97" s="239" t="str">
+      <c r="D97" s="240" t="str">
         <f>=IFERROR(ROUND(Drittmittel_LW,2),0)</f>
       </c>
-      <c r="E97" s="201" t="str">
+      <c r="E97" s="202" t="str">
         <f>=ROUND(IFERROR($C$97-$D$97,0),2)</f>
       </c>
       <c r="F97" s="258" t="str">
         <f>=ROUND(IFERROR(($C$97/$D$97)-1,0),4)</f>
       </c>
-      <c r="G97" s="217" t="str">
+      <c r="G97" s="218" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$F$13,'III. Finanzberichte'!$M$13,'III. Finanzberichte'!$T$13,'III. Finanzberichte'!$AA$13,'III. Finanzberichte'!$AH$13,'III. Finanzberichte'!$AO$13,'III. Finanzberichte'!$AV$13,'III. Finanzberichte'!$BC$13,'III. Finanzberichte'!$BJ$13,'III. Finanzberichte'!$BQ$13,'III. Finanzberichte'!$BX$13,'III. Finanzberichte'!$CE$13,'III. Finanzberichte'!$CL$13,'III. Finanzberichte'!$CS$13,'III. Finanzberichte'!$CZ$13,'III. Finanzberichte'!$DG$13,'III. Finanzberichte'!$DN$13,'III. Finanzberichte'!$DU$13),2),0)</f>
       </c>
-      <c r="H97" s="217" t="str">
+      <c r="H97" s="218" t="str">
         <f>=IFERROR(ROUND(Drittmittel_EUR,2),0)</f>
       </c>
       <c r="I97" s="182" t="str">
@@ -23118,22 +23235,22 @@
       <c r="B98" s="266" t="s">
         <v>199</v>
       </c>
-      <c r="C98" s="239" t="str">
+      <c r="C98" s="240" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$E$14,'III. Finanzberichte'!$L$14,'III. Finanzberichte'!$S$14,'III. Finanzberichte'!$Z$14,'III. Finanzberichte'!$AG$14,'III. Finanzberichte'!$AN$14,'III. Finanzberichte'!$AU$14,'III. Finanzberichte'!$BB$14,'III. Finanzberichte'!$BI$14,'III. Finanzberichte'!$BP$14,'III. Finanzberichte'!$BW$14,'III. Finanzberichte'!$CD$14,'III. Finanzberichte'!$CK$14,'III. Finanzberichte'!$CR$14,'III. Finanzberichte'!$CY$14,'III. Finanzberichte'!$DF$14,'III. Finanzberichte'!$DM$14,'III. Finanzberichte'!$DT$14),2),0)</f>
       </c>
-      <c r="D98" s="239" t="str">
+      <c r="D98" s="240" t="str">
         <f>=IFERROR(ROUND(KMW_Mittel_LW,2),0)</f>
       </c>
-      <c r="E98" s="201" t="str">
+      <c r="E98" s="202" t="str">
         <f>=ROUND(IFERROR($C$98-$D$98,0),2)</f>
       </c>
       <c r="F98" s="258" t="str">
         <f>=ROUND(IFERROR(($C$98/$D$98)-1,0),4)</f>
       </c>
-      <c r="G98" s="217" t="str">
+      <c r="G98" s="218" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$F$14,'III. Finanzberichte'!$M$14,'III. Finanzberichte'!$T$14,'III. Finanzberichte'!$AA$14,'III. Finanzberichte'!$AH$14,'III. Finanzberichte'!$AO$14,'III. Finanzberichte'!$AV$14,'III. Finanzberichte'!$BC$14,'III. Finanzberichte'!$BJ$14,'III. Finanzberichte'!$BQ$14,'III. Finanzberichte'!$BX$14,'III. Finanzberichte'!$CE$14,'III. Finanzberichte'!$CL$14,'III. Finanzberichte'!$CS$14,'III. Finanzberichte'!$CZ$14,'III. Finanzberichte'!$DG$14,'III. Finanzberichte'!$DN$14,'III. Finanzberichte'!$DU$14),2),0)</f>
       </c>
-      <c r="H98" s="217" t="str">
+      <c r="H98" s="218" t="str">
         <f>=IFERROR(ROUND(KMW_Mittel_EUR,2),0)</f>
       </c>
       <c r="I98" s="182" t="str">
@@ -23162,22 +23279,22 @@
       <c r="B99" s="266" t="s">
         <v>301</v>
       </c>
-      <c r="C99" s="239" t="str">
+      <c r="C99" s="240" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$E$15,'III. Finanzberichte'!$L$15,'III. Finanzberichte'!$S$15,'III. Finanzberichte'!$Z$15,'III. Finanzberichte'!$AG$15,'III. Finanzberichte'!$AN$15,'III. Finanzberichte'!$AU$15,'III. Finanzberichte'!$BB$15,'III. Finanzberichte'!$BI$15,'III. Finanzberichte'!$BP$15,'III. Finanzberichte'!$BW$15,'III. Finanzberichte'!$CD$15,'III. Finanzberichte'!$CK$15,'III. Finanzberichte'!$CR$15,'III. Finanzberichte'!$CY$15,'III. Finanzberichte'!$DF$15,'III. Finanzberichte'!$DM$15,'III. Finanzberichte'!$DT$15),2),0)</f>
       </c>
-      <c r="D99" s="239" t="str">
+      <c r="D99" s="240" t="str">
         <f>=IFERROR(ROUND(0,2),0)</f>
       </c>
-      <c r="E99" s="201" t="str">
+      <c r="E99" s="202" t="str">
         <f>=ROUND(IFERROR($C$99-$D$99,0),2)</f>
       </c>
       <c r="F99" s="258" t="str">
         <f>=ROUND(IFERROR(($C$99/$D$99)-1,0),4)</f>
       </c>
-      <c r="G99" s="217" t="str">
+      <c r="G99" s="218" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$F$15,'III. Finanzberichte'!$M$15,'III. Finanzberichte'!$T$15,'III. Finanzberichte'!$AA$15,'III. Finanzberichte'!$AH$15,'III. Finanzberichte'!$AO$15,'III. Finanzberichte'!$AV$15,'III. Finanzberichte'!$BC$15,'III. Finanzberichte'!$BJ$15,'III. Finanzberichte'!$BQ$15,'III. Finanzberichte'!$BX$15,'III. Finanzberichte'!$CE$15,'III. Finanzberichte'!$CL$15,'III. Finanzberichte'!$CS$15,'III. Finanzberichte'!$CZ$15,'III. Finanzberichte'!$DG$15,'III. Finanzberichte'!$DN$15,'III. Finanzberichte'!$DU$15),2),0)</f>
       </c>
-      <c r="H99" s="217" t="str">
+      <c r="H99" s="218" t="str">
         <f>=IFERROR(ROUND(0,2),0)</f>
       </c>
       <c r="I99" s="182" t="str">
@@ -23265,7 +23382,7 @@
     </row>
     <row r="102" ht="22" customHeight="true">
       <c r="B102" s="18" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C102" s="18"/>
       <c r="D102" s="18"/>
@@ -23310,31 +23427,31 @@
     </row>
     <row r="104" ht="28" customHeight="true">
       <c r="B104" s="263" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C104" s="264" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="D104" s="264" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="E104" s="264" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="F104" s="264" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="G104" s="264" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="H104" s="264" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="I104" s="264" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="J104" s="265" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="L104" s="47"/>
       <c r="P104" s="48"/>
@@ -23343,22 +23460,22 @@
       <c r="B105" s="266" t="s">
         <v>205</v>
       </c>
-      <c r="C105" s="239" t="str">
+      <c r="C105" s="240" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$E$19+'III. Finanzberichte'!$E$20,'III. Finanzberichte'!$L$19+'III. Finanzberichte'!$L$20,'III. Finanzberichte'!$S$19+'III. Finanzberichte'!$S$20,'III. Finanzberichte'!$Z$19+'III. Finanzberichte'!$Z$20,'III. Finanzberichte'!$AG$19+'III. Finanzberichte'!$AG$20,'III. Finanzberichte'!$AN$19+'III. Finanzberichte'!$AN$20,'III. Finanzberichte'!$AU$19+'III. Finanzberichte'!$AU$20,'III. Finanzberichte'!$BB$19+'III. Finanzberichte'!$BB$20,'III. Finanzberichte'!$BI$19+'III. Finanzberichte'!$BI$20,'III. Finanzberichte'!$BP$19+'III. Finanzberichte'!$BP$20,'III. Finanzberichte'!$BW$19+'III. Finanzberichte'!$BW$20,'III. Finanzberichte'!$CD$19+'III. Finanzberichte'!$CD$20,'III. Finanzberichte'!$CK$19+'III. Finanzberichte'!$CK$20,'III. Finanzberichte'!$CR$19+'III. Finanzberichte'!$CR$20,'III. Finanzberichte'!$CY$19+'III. Finanzberichte'!$CY$20,'III. Finanzberichte'!$DF$19+'III. Finanzberichte'!$DF$20,'III. Finanzberichte'!$DM$19+'III. Finanzberichte'!$DM$20,'III. Finanzberichte'!$DT$19+'III. Finanzberichte'!$DT$20),2),0)</f>
       </c>
-      <c r="D105" s="239" t="str">
+      <c r="D105" s="240" t="str">
         <f>=IFERROR(ROUND(Kosten_Bauausgaben_LW,2),0)</f>
       </c>
-      <c r="E105" s="201" t="str">
+      <c r="E105" s="202" t="str">
         <f>=ROUND(IFERROR($C$105-$D$105,0),2)</f>
       </c>
       <c r="F105" s="258" t="str">
         <f>=ROUND(IFERROR(($C$105/$D$105)-1,0),4)</f>
       </c>
-      <c r="G105" s="217" t="str">
+      <c r="G105" s="218" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$F$19+'III. Finanzberichte'!$F$20,'III. Finanzberichte'!$M$19+'III. Finanzberichte'!$M$20,'III. Finanzberichte'!$T$19+'III. Finanzberichte'!$T$20,'III. Finanzberichte'!$AA$19+'III. Finanzberichte'!$AA$20,'III. Finanzberichte'!$AH$19+'III. Finanzberichte'!$AH$20,'III. Finanzberichte'!$AO$19+'III. Finanzberichte'!$AO$20,'III. Finanzberichte'!$AV$19+'III. Finanzberichte'!$AV$20,'III. Finanzberichte'!$BC$19+'III. Finanzberichte'!$BC$20,'III. Finanzberichte'!$BJ$19+'III. Finanzberichte'!$BJ$20,'III. Finanzberichte'!$BQ$19+'III. Finanzberichte'!$BQ$20,'III. Finanzberichte'!$BX$19+'III. Finanzberichte'!$BX$20,'III. Finanzberichte'!$CE$19+'III. Finanzberichte'!$CE$20,'III. Finanzberichte'!$CL$19+'III. Finanzberichte'!$CL$20,'III. Finanzberichte'!$CS$19+'III. Finanzberichte'!$CS$20,'III. Finanzberichte'!$CZ$19+'III. Finanzberichte'!$CZ$20,'III. Finanzberichte'!$DG$19+'III. Finanzberichte'!$DG$20,'III. Finanzberichte'!$DN$19+'III. Finanzberichte'!$DN$20,'III. Finanzberichte'!$DU$19+'III. Finanzberichte'!$DU$20),2),0)</f>
       </c>
-      <c r="H105" s="217" t="str">
+      <c r="H105" s="218" t="str">
         <f>=IFERROR(ROUND(Kosten_Bauausgaben_EUR,2),0)</f>
       </c>
       <c r="I105" s="182" t="str">
@@ -23387,22 +23504,22 @@
       <c r="B106" s="266" t="s">
         <v>210</v>
       </c>
-      <c r="C106" s="239" t="str">
+      <c r="C106" s="240" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$E$21,'III. Finanzberichte'!$L$21,'III. Finanzberichte'!$S$21,'III. Finanzberichte'!$Z$21,'III. Finanzberichte'!$AG$21,'III. Finanzberichte'!$AN$21,'III. Finanzberichte'!$AU$21,'III. Finanzberichte'!$BB$21,'III. Finanzberichte'!$BI$21,'III. Finanzberichte'!$BP$21,'III. Finanzberichte'!$BW$21,'III. Finanzberichte'!$CD$21,'III. Finanzberichte'!$CK$21,'III. Finanzberichte'!$CR$21,'III. Finanzberichte'!$CY$21,'III. Finanzberichte'!$DF$21,'III. Finanzberichte'!$DM$21,'III. Finanzberichte'!$DT$21),2),0)</f>
       </c>
-      <c r="D106" s="239" t="str">
+      <c r="D106" s="240" t="str">
         <f>=IFERROR(ROUND(Kosten_Investitionen_LW,2),0)</f>
       </c>
-      <c r="E106" s="201" t="str">
+      <c r="E106" s="202" t="str">
         <f>=ROUND(IFERROR($C$106-$D$106,0),2)</f>
       </c>
       <c r="F106" s="258" t="str">
         <f>=ROUND(IFERROR(($C$106/$D$106)-1,0),4)</f>
       </c>
-      <c r="G106" s="217" t="str">
+      <c r="G106" s="218" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$F$21,'III. Finanzberichte'!$M$21,'III. Finanzberichte'!$T$21,'III. Finanzberichte'!$AA$21,'III. Finanzberichte'!$AH$21,'III. Finanzberichte'!$AO$21,'III. Finanzberichte'!$AV$21,'III. Finanzberichte'!$BC$21,'III. Finanzberichte'!$BJ$21,'III. Finanzberichte'!$BQ$21,'III. Finanzberichte'!$BX$21,'III. Finanzberichte'!$CE$21,'III. Finanzberichte'!$CL$21,'III. Finanzberichte'!$CS$21,'III. Finanzberichte'!$CZ$21,'III. Finanzberichte'!$DG$21,'III. Finanzberichte'!$DN$21,'III. Finanzberichte'!$DU$21),2),0)</f>
       </c>
-      <c r="H106" s="217" t="str">
+      <c r="H106" s="218" t="str">
         <f>=IFERROR(ROUND(Kosten_Investitionen_EUR,2),0)</f>
       </c>
       <c r="I106" s="182" t="str">
@@ -23416,22 +23533,22 @@
       <c r="B107" s="266" t="s">
         <v>213</v>
       </c>
-      <c r="C107" s="239" t="str">
+      <c r="C107" s="240" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$E$22+'III. Finanzberichte'!$E$23,'III. Finanzberichte'!$L$22+'III. Finanzberichte'!$L$23,'III. Finanzberichte'!$S$22+'III. Finanzberichte'!$S$23,'III. Finanzberichte'!$Z$22+'III. Finanzberichte'!$Z$23,'III. Finanzberichte'!$AG$22+'III. Finanzberichte'!$AG$23,'III. Finanzberichte'!$AN$22+'III. Finanzberichte'!$AN$23,'III. Finanzberichte'!$AU$22+'III. Finanzberichte'!$AU$23,'III. Finanzberichte'!$BB$22+'III. Finanzberichte'!$BB$23,'III. Finanzberichte'!$BI$22+'III. Finanzberichte'!$BI$23,'III. Finanzberichte'!$BP$22+'III. Finanzberichte'!$BP$23,'III. Finanzberichte'!$BW$22+'III. Finanzberichte'!$BW$23,'III. Finanzberichte'!$CD$22+'III. Finanzberichte'!$CD$23,'III. Finanzberichte'!$CK$22+'III. Finanzberichte'!$CK$23,'III. Finanzberichte'!$CR$22+'III. Finanzberichte'!$CR$23,'III. Finanzberichte'!$CY$22+'III. Finanzberichte'!$CY$23,'III. Finanzberichte'!$DF$22+'III. Finanzberichte'!$DF$23,'III. Finanzberichte'!$DM$22+'III. Finanzberichte'!$DM$23,'III. Finanzberichte'!$DT$22+'III. Finanzberichte'!$DT$23),2),0)</f>
       </c>
-      <c r="D107" s="239" t="str">
+      <c r="D107" s="240" t="str">
         <f>=IFERROR(ROUND(Kosten_Personalkosten_LW,2),0)</f>
       </c>
-      <c r="E107" s="201" t="str">
+      <c r="E107" s="202" t="str">
         <f>=ROUND(IFERROR($C$107-$D$107,0),2)</f>
       </c>
       <c r="F107" s="258" t="str">
         <f>=ROUND(IFERROR(($C$107/$D$107)-1,0),4)</f>
       </c>
-      <c r="G107" s="217" t="str">
+      <c r="G107" s="218" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$F$22+'III. Finanzberichte'!$F$23,'III. Finanzberichte'!$M$22+'III. Finanzberichte'!$M$23,'III. Finanzberichte'!$T$22+'III. Finanzberichte'!$T$23,'III. Finanzberichte'!$AA$22+'III. Finanzberichte'!$AA$23,'III. Finanzberichte'!$AH$22+'III. Finanzberichte'!$AH$23,'III. Finanzberichte'!$AO$22+'III. Finanzberichte'!$AO$23,'III. Finanzberichte'!$AV$22+'III. Finanzberichte'!$AV$23,'III. Finanzberichte'!$BC$22+'III. Finanzberichte'!$BC$23,'III. Finanzberichte'!$BJ$22+'III. Finanzberichte'!$BJ$23,'III. Finanzberichte'!$BQ$22+'III. Finanzberichte'!$BQ$23,'III. Finanzberichte'!$BX$22+'III. Finanzberichte'!$BX$23,'III. Finanzberichte'!$CE$22+'III. Finanzberichte'!$CE$23,'III. Finanzberichte'!$CL$22+'III. Finanzberichte'!$CL$23,'III. Finanzberichte'!$CS$22+'III. Finanzberichte'!$CS$23,'III. Finanzberichte'!$CZ$22+'III. Finanzberichte'!$CZ$23,'III. Finanzberichte'!$DG$22+'III. Finanzberichte'!$DG$23,'III. Finanzberichte'!$DN$22+'III. Finanzberichte'!$DN$23,'III. Finanzberichte'!$DU$22+'III. Finanzberichte'!$DU$23),2),0)</f>
       </c>
-      <c r="H107" s="217" t="str">
+      <c r="H107" s="218" t="str">
         <f>=IFERROR(ROUND(Kosten_Personalkosten_EUR,2),0)</f>
       </c>
       <c r="I107" s="182" t="str">
@@ -23445,22 +23562,22 @@
       <c r="B108" s="266" t="s">
         <v>218</v>
       </c>
-      <c r="C108" s="239" t="str">
+      <c r="C108" s="240" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$E$24,'III. Finanzberichte'!$L$24,'III. Finanzberichte'!$S$24,'III. Finanzberichte'!$Z$24,'III. Finanzberichte'!$AG$24,'III. Finanzberichte'!$AN$24,'III. Finanzberichte'!$AU$24,'III. Finanzberichte'!$BB$24,'III. Finanzberichte'!$BI$24,'III. Finanzberichte'!$BP$24,'III. Finanzberichte'!$BW$24,'III. Finanzberichte'!$CD$24,'III. Finanzberichte'!$CK$24,'III. Finanzberichte'!$CR$24,'III. Finanzberichte'!$CY$24,'III. Finanzberichte'!$DF$24,'III. Finanzberichte'!$DM$24,'III. Finanzberichte'!$DT$24),2),0)</f>
       </c>
-      <c r="D108" s="239" t="str">
+      <c r="D108" s="240" t="str">
         <f>=IFERROR(ROUND(Kosten_Projektaktivitaeten_LW,2),0)</f>
       </c>
-      <c r="E108" s="201" t="str">
+      <c r="E108" s="202" t="str">
         <f>=ROUND(IFERROR($C$108-$D$108,0),2)</f>
       </c>
       <c r="F108" s="258" t="str">
         <f>=ROUND(IFERROR(($C$108/$D$108)-1,0),4)</f>
       </c>
-      <c r="G108" s="217" t="str">
+      <c r="G108" s="218" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$F$24,'III. Finanzberichte'!$M$24,'III. Finanzberichte'!$T$24,'III. Finanzberichte'!$AA$24,'III. Finanzberichte'!$AH$24,'III. Finanzberichte'!$AO$24,'III. Finanzberichte'!$AV$24,'III. Finanzberichte'!$BC$24,'III. Finanzberichte'!$BJ$24,'III. Finanzberichte'!$BQ$24,'III. Finanzberichte'!$BX$24,'III. Finanzberichte'!$CE$24,'III. Finanzberichte'!$CL$24,'III. Finanzberichte'!$CS$24,'III. Finanzberichte'!$CZ$24,'III. Finanzberichte'!$DG$24,'III. Finanzberichte'!$DN$24,'III. Finanzberichte'!$DU$24),2),0)</f>
       </c>
-      <c r="H108" s="217" t="str">
+      <c r="H108" s="218" t="str">
         <f>=IFERROR(ROUND(Kosten_Projektaktivitaeten_EUR,2),0)</f>
       </c>
       <c r="I108" s="182" t="str">
@@ -23474,22 +23591,22 @@
       <c r="B109" s="266" t="s">
         <v>221</v>
       </c>
-      <c r="C109" s="239" t="str">
+      <c r="C109" s="240" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$E$25,'III. Finanzberichte'!$L$25,'III. Finanzberichte'!$S$25,'III. Finanzberichte'!$Z$25,'III. Finanzberichte'!$AG$25,'III. Finanzberichte'!$AN$25,'III. Finanzberichte'!$AU$25,'III. Finanzberichte'!$BB$25,'III. Finanzberichte'!$BI$25,'III. Finanzberichte'!$BP$25,'III. Finanzberichte'!$BW$25,'III. Finanzberichte'!$CD$25,'III. Finanzberichte'!$CK$25,'III. Finanzberichte'!$CR$25,'III. Finanzberichte'!$CY$25,'III. Finanzberichte'!$DF$25,'III. Finanzberichte'!$DM$25,'III. Finanzberichte'!$DT$25),2),0)</f>
       </c>
-      <c r="D109" s="239" t="str">
+      <c r="D109" s="240" t="str">
         <f>=IFERROR(ROUND(Kosten_Projektverwaltung_LW,2),0)</f>
       </c>
-      <c r="E109" s="201" t="str">
+      <c r="E109" s="202" t="str">
         <f>=ROUND(IFERROR($C$109-$D$109,0),2)</f>
       </c>
       <c r="F109" s="258" t="str">
         <f>=ROUND(IFERROR(($C$109/$D$109)-1,0),4)</f>
       </c>
-      <c r="G109" s="217" t="str">
+      <c r="G109" s="218" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$F$25,'III. Finanzberichte'!$M$25,'III. Finanzberichte'!$T$25,'III. Finanzberichte'!$AA$25,'III. Finanzberichte'!$AH$25,'III. Finanzberichte'!$AO$25,'III. Finanzberichte'!$AV$25,'III. Finanzberichte'!$BC$25,'III. Finanzberichte'!$BJ$25,'III. Finanzberichte'!$BQ$25,'III. Finanzberichte'!$BX$25,'III. Finanzberichte'!$CE$25,'III. Finanzberichte'!$CL$25,'III. Finanzberichte'!$CS$25,'III. Finanzberichte'!$CZ$25,'III. Finanzberichte'!$DG$25,'III. Finanzberichte'!$DN$25,'III. Finanzberichte'!$DU$25),2),0)</f>
       </c>
-      <c r="H109" s="217" t="str">
+      <c r="H109" s="218" t="str">
         <f>=IFERROR(ROUND(Kosten_Projektverwaltung_EUR,2),0)</f>
       </c>
       <c r="I109" s="182" t="str">
@@ -23503,22 +23620,22 @@
       <c r="B110" s="266" t="s">
         <v>224</v>
       </c>
-      <c r="C110" s="239" t="str">
+      <c r="C110" s="240" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$E$26,'III. Finanzberichte'!$L$26,'III. Finanzberichte'!$S$26,'III. Finanzberichte'!$Z$26,'III. Finanzberichte'!$AG$26,'III. Finanzberichte'!$AN$26,'III. Finanzberichte'!$AU$26,'III. Finanzberichte'!$BB$26,'III. Finanzberichte'!$BI$26,'III. Finanzberichte'!$BP$26,'III. Finanzberichte'!$BW$26,'III. Finanzberichte'!$CD$26,'III. Finanzberichte'!$CK$26,'III. Finanzberichte'!$CR$26,'III. Finanzberichte'!$CY$26,'III. Finanzberichte'!$DF$26,'III. Finanzberichte'!$DM$26,'III. Finanzberichte'!$DT$26),2),0)</f>
       </c>
-      <c r="D110" s="239" t="str">
+      <c r="D110" s="240" t="str">
         <f>=IFERROR(ROUND(Kosten_Evaluierung_LW,2),0)</f>
       </c>
-      <c r="E110" s="201" t="str">
+      <c r="E110" s="202" t="str">
         <f>=ROUND(IFERROR($C$110-$D$110,0),2)</f>
       </c>
       <c r="F110" s="258" t="str">
         <f>=ROUND(IFERROR(($C$110/$D$110)-1,0),4)</f>
       </c>
-      <c r="G110" s="217" t="str">
+      <c r="G110" s="218" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$F$26,'III. Finanzberichte'!$M$26,'III. Finanzberichte'!$T$26,'III. Finanzberichte'!$AA$26,'III. Finanzberichte'!$AH$26,'III. Finanzberichte'!$AO$26,'III. Finanzberichte'!$AV$26,'III. Finanzberichte'!$BC$26,'III. Finanzberichte'!$BJ$26,'III. Finanzberichte'!$BQ$26,'III. Finanzberichte'!$BX$26,'III. Finanzberichte'!$CE$26,'III. Finanzberichte'!$CL$26,'III. Finanzberichte'!$CS$26,'III. Finanzberichte'!$CZ$26,'III. Finanzberichte'!$DG$26,'III. Finanzberichte'!$DN$26,'III. Finanzberichte'!$DU$26),2),0)</f>
       </c>
-      <c r="H110" s="217" t="str">
+      <c r="H110" s="218" t="str">
         <f>=IFERROR(ROUND(Kosten_Evaluierung_EUR,2),0)</f>
       </c>
       <c r="I110" s="182" t="str">
@@ -23532,22 +23649,22 @@
       <c r="B111" s="266" t="s">
         <v>227</v>
       </c>
-      <c r="C111" s="239" t="str">
+      <c r="C111" s="240" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$E$27,'III. Finanzberichte'!$L$27,'III. Finanzberichte'!$S$27,'III. Finanzberichte'!$Z$27,'III. Finanzberichte'!$AG$27,'III. Finanzberichte'!$AN$27,'III. Finanzberichte'!$AU$27,'III. Finanzberichte'!$BB$27,'III. Finanzberichte'!$BI$27,'III. Finanzberichte'!$BP$27,'III. Finanzberichte'!$BW$27,'III. Finanzberichte'!$CD$27,'III. Finanzberichte'!$CK$27,'III. Finanzberichte'!$CR$27,'III. Finanzberichte'!$CY$27,'III. Finanzberichte'!$DF$27,'III. Finanzberichte'!$DM$27,'III. Finanzberichte'!$DT$27),2),0)</f>
       </c>
-      <c r="D111" s="239" t="str">
+      <c r="D111" s="240" t="str">
         <f>=IFERROR(ROUND(Kosten_Audit_LW,2),0)</f>
       </c>
-      <c r="E111" s="201" t="str">
+      <c r="E111" s="202" t="str">
         <f>=ROUND(IFERROR($C$111-$D$111,0),2)</f>
       </c>
       <c r="F111" s="258" t="str">
         <f>=ROUND(IFERROR(($C$111/$D$111)-1,0),4)</f>
       </c>
-      <c r="G111" s="217" t="str">
+      <c r="G111" s="218" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$F$27,'III. Finanzberichte'!$M$27,'III. Finanzberichte'!$T$27,'III. Finanzberichte'!$AA$27,'III. Finanzberichte'!$AH$27,'III. Finanzberichte'!$AO$27,'III. Finanzberichte'!$AV$27,'III. Finanzberichte'!$BC$27,'III. Finanzberichte'!$BJ$27,'III. Finanzberichte'!$BQ$27,'III. Finanzberichte'!$BX$27,'III. Finanzberichte'!$CE$27,'III. Finanzberichte'!$CL$27,'III. Finanzberichte'!$CS$27,'III. Finanzberichte'!$CZ$27,'III. Finanzberichte'!$DG$27,'III. Finanzberichte'!$DN$27,'III. Finanzberichte'!$DU$27),2),0)</f>
       </c>
-      <c r="H111" s="217" t="str">
+      <c r="H111" s="218" t="str">
         <f>=IFERROR(ROUND(Kosten_Audit_EUR,2),0)</f>
       </c>
       <c r="I111" s="182" t="str">
@@ -23561,22 +23678,22 @@
       <c r="B112" s="266" t="s">
         <v>230</v>
       </c>
-      <c r="C112" s="239" t="str">
+      <c r="C112" s="240" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$E$28,'III. Finanzberichte'!$L$28,'III. Finanzberichte'!$S$28,'III. Finanzberichte'!$Z$28,'III. Finanzberichte'!$AG$28,'III. Finanzberichte'!$AN$28,'III. Finanzberichte'!$AU$28,'III. Finanzberichte'!$BB$28,'III. Finanzberichte'!$BI$28,'III. Finanzberichte'!$BP$28,'III. Finanzberichte'!$BW$28,'III. Finanzberichte'!$CD$28,'III. Finanzberichte'!$CK$28,'III. Finanzberichte'!$CR$28,'III. Finanzberichte'!$CY$28,'III. Finanzberichte'!$DF$28,'III. Finanzberichte'!$DM$28,'III. Finanzberichte'!$DT$28),2),0)</f>
       </c>
-      <c r="D112" s="239" t="str">
+      <c r="D112" s="240" t="str">
         <f>=IFERROR(ROUND(Kosten_Reserve_LW,2),0)</f>
       </c>
-      <c r="E112" s="201" t="str">
+      <c r="E112" s="202" t="str">
         <f>=ROUND(IFERROR($C$112-$D$112,0),2)</f>
       </c>
       <c r="F112" s="258" t="str">
         <f>=ROUND(IFERROR(($C$112/$D$112)-1,0),4)</f>
       </c>
-      <c r="G112" s="217" t="str">
+      <c r="G112" s="218" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$F$28,'III. Finanzberichte'!$M$28,'III. Finanzberichte'!$T$28,'III. Finanzberichte'!$AA$28,'III. Finanzberichte'!$AH$28,'III. Finanzberichte'!$AO$28,'III. Finanzberichte'!$AV$28,'III. Finanzberichte'!$BC$28,'III. Finanzberichte'!$BJ$28,'III. Finanzberichte'!$BQ$28,'III. Finanzberichte'!$BX$28,'III. Finanzberichte'!$CE$28,'III. Finanzberichte'!$CL$28,'III. Finanzberichte'!$CS$28,'III. Finanzberichte'!$CZ$28,'III. Finanzberichte'!$DG$28,'III. Finanzberichte'!$DN$28,'III. Finanzberichte'!$DU$28),2),0)</f>
       </c>
-      <c r="H112" s="217" t="str">
+      <c r="H112" s="218" t="str">
         <f>=IFERROR(ROUND(Kosten_Reserve_EUR,2),0)</f>
       </c>
       <c r="I112" s="182" t="str">
@@ -23957,16 +24074,16 @@
         <v>247</v>
       </c>
       <c r="C1" s="351" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="I1" s="351" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="O1" s="351" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="U1" s="351" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="BA1">
         <v>1</v>

</xml_diff>

<commit_message>
feat: add manual amount field to mittelanforderung report
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_befuellt.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_befuellt.xlsx
@@ -103,41 +103,41 @@
     <definedName name="FB_SaldoLC_18">'III. Finanzberichte'!$DR$31</definedName>
     <definedName name="FB_SaldoEUR_18">'III. Finanzberichte'!$DS$31</definedName>
     <definedName name="MA_Kurs_1">'IV. MA'!$C$8</definedName>
-    <definedName name="MA_ManBetrag_1">'IV. MA'!$D$24</definedName>
+    <definedName name="MA_ManBetrag_1">'IV. MA'!$D$27</definedName>
     <definedName name="MA_Kurs_2">'IV. MA'!$G$8</definedName>
-    <definedName name="MA_ManBetrag_2">'IV. MA'!$H$24</definedName>
+    <definedName name="MA_ManBetrag_2">'IV. MA'!$H$27</definedName>
     <definedName name="MA_Kurs_3">'IV. MA'!$K$8</definedName>
-    <definedName name="MA_ManBetrag_3">'IV. MA'!$L$24</definedName>
+    <definedName name="MA_ManBetrag_3">'IV. MA'!$L$27</definedName>
     <definedName name="MA_Kurs_4">'IV. MA'!$O$8</definedName>
-    <definedName name="MA_ManBetrag_4">'IV. MA'!$P$24</definedName>
+    <definedName name="MA_ManBetrag_4">'IV. MA'!$P$27</definedName>
     <definedName name="MA_Kurs_5">'IV. MA'!$S$8</definedName>
-    <definedName name="MA_ManBetrag_5">'IV. MA'!$T$24</definedName>
+    <definedName name="MA_ManBetrag_5">'IV. MA'!$T$27</definedName>
     <definedName name="MA_Kurs_6">'IV. MA'!$W$8</definedName>
-    <definedName name="MA_ManBetrag_6">'IV. MA'!$X$24</definedName>
+    <definedName name="MA_ManBetrag_6">'IV. MA'!$X$27</definedName>
     <definedName name="MA_Kurs_7">'IV. MA'!$AA$8</definedName>
-    <definedName name="MA_ManBetrag_7">'IV. MA'!$AB$24</definedName>
+    <definedName name="MA_ManBetrag_7">'IV. MA'!$AB$27</definedName>
     <definedName name="MA_Kurs_8">'IV. MA'!$AE$8</definedName>
-    <definedName name="MA_ManBetrag_8">'IV. MA'!$AF$24</definedName>
+    <definedName name="MA_ManBetrag_8">'IV. MA'!$AF$27</definedName>
     <definedName name="MA_Kurs_9">'IV. MA'!$AI$8</definedName>
-    <definedName name="MA_ManBetrag_9">'IV. MA'!$AJ$24</definedName>
+    <definedName name="MA_ManBetrag_9">'IV. MA'!$AJ$27</definedName>
     <definedName name="MA_Kurs_10">'IV. MA'!$AM$8</definedName>
-    <definedName name="MA_ManBetrag_10">'IV. MA'!$AN$24</definedName>
+    <definedName name="MA_ManBetrag_10">'IV. MA'!$AN$27</definedName>
     <definedName name="MA_Kurs_11">'IV. MA'!$AQ$8</definedName>
-    <definedName name="MA_ManBetrag_11">'IV. MA'!$AR$24</definedName>
+    <definedName name="MA_ManBetrag_11">'IV. MA'!$AR$27</definedName>
     <definedName name="MA_Kurs_12">'IV. MA'!$AU$8</definedName>
-    <definedName name="MA_ManBetrag_12">'IV. MA'!$AV$24</definedName>
+    <definedName name="MA_ManBetrag_12">'IV. MA'!$AV$27</definedName>
     <definedName name="MA_Kurs_13">'IV. MA'!$AY$8</definedName>
-    <definedName name="MA_ManBetrag_13">'IV. MA'!$AZ$24</definedName>
+    <definedName name="MA_ManBetrag_13">'IV. MA'!$AZ$27</definedName>
     <definedName name="MA_Kurs_14">'IV. MA'!$BC$8</definedName>
-    <definedName name="MA_ManBetrag_14">'IV. MA'!$BD$24</definedName>
+    <definedName name="MA_ManBetrag_14">'IV. MA'!$BD$27</definedName>
     <definedName name="MA_Kurs_15">'IV. MA'!$BG$8</definedName>
-    <definedName name="MA_ManBetrag_15">'IV. MA'!$BH$24</definedName>
+    <definedName name="MA_ManBetrag_15">'IV. MA'!$BH$27</definedName>
     <definedName name="MA_Kurs_16">'IV. MA'!$BK$8</definedName>
-    <definedName name="MA_ManBetrag_16">'IV. MA'!$BL$24</definedName>
+    <definedName name="MA_ManBetrag_16">'IV. MA'!$BL$27</definedName>
     <definedName name="MA_Kurs_17">'IV. MA'!$BO$8</definedName>
-    <definedName name="MA_ManBetrag_17">'IV. MA'!$BP$24</definedName>
+    <definedName name="MA_ManBetrag_17">'IV. MA'!$BP$27</definedName>
     <definedName name="MA_Kurs_18">'IV. MA'!$BS$8</definedName>
-    <definedName name="MA_ManBetrag_18">'IV. MA'!$BT$24</definedName>
+    <definedName name="MA_ManBetrag_18">'IV. MA'!$BT$27</definedName>
     <definedName name="FB_Auswahl_Liste">OFFSET('Daten'!$BP$1,0,0,COUNTA('Daten'!$BP:$BP),1)</definedName>
     <definedName name="MA_Auswahl_Liste">OFFSET('Daten'!$BN$1,0,0,COUNTA('Daten'!$BN:$BN),1)</definedName>
   </definedNames>
@@ -1172,10 +1172,10 @@
     <t>abzueglich Saldo Vorprojekt:</t>
   </si>
   <si>
-    <t>Manueller Betrag:</t>
-  </si>
-  <si>
     <t>KMW-Mittel Anforderung:</t>
+  </si>
+  <si>
+    <t>Manueller Betrag (EUR):</t>
   </si>
   <si>
     <t>abzueglich Saldo Vorperiode (FB):</t>
@@ -2827,161 +2827,161 @@
     <xf numFmtId="166" fontId="8" fillId="0" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="50" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="19" fillId="10" borderId="49" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="19" fillId="10" borderId="49" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="12" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="51" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="7" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="52" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="18" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="12" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="12" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="17" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="18" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="20" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="21" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="12" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="38" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="39" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="8" borderId="40" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="8" borderId="21" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="51" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="7" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="52" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="17" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="12" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="true" applyAlignment="false">
+      <alignment/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="12" borderId="40" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="50" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="19" fillId="10" borderId="49" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="19" fillId="10" borderId="49" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="172" fontId="12" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="51" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="7" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="52" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="18" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="172" fontId="12" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="172" fontId="12" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="17" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="18" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="20" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="21" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="12" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="12" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="38" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="39" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="8" borderId="40" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="12" fillId="8" borderId="21" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="51" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="7" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="52" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="17" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="12" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="12" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="true" applyAlignment="false">
-      <alignment/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="12" borderId="40" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="172" fontId="3" fillId="5" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
@@ -21056,354 +21056,372 @@
         <f>=IFERROR(ROUND($BS$23/$BS$8,2),0)</f>
       </c>
     </row>
-    <row r="24">
-      <c r="B24" t="s">
+    <row r="25">
+      <c r="B25" s="189" t="s">
         <v>334</v>
       </c>
-      <c r="C24" s="189"/>
-      <c r="D24" s="25"/>
-      <c r="F24" t="s">
+      <c r="C25" s="190" t="str">
+        <f>=IFERROR(ROUND($C$18-$C$21-$C$22-$C$23,2),0)</f>
+      </c>
+      <c r="D25" s="191" t="str">
+        <f>=IFERROR(ROUND($D$18-$D$21-$D$22-$D$23,2),0)</f>
+      </c>
+      <c r="F25" s="189" t="s">
         <v>334</v>
       </c>
-      <c r="G24" s="189"/>
-      <c r="H24" s="25"/>
-      <c r="J24" t="s">
+      <c r="G25" s="190" t="str">
+        <f>=IFERROR(ROUND($G$18-$G$21-$G$22-$G$23,2),0)</f>
+      </c>
+      <c r="H25" s="191" t="str">
+        <f>=IFERROR(ROUND($H$18-$H$21-$H$22-$H$23,2),0)</f>
+      </c>
+      <c r="J25" s="189" t="s">
         <v>334</v>
       </c>
-      <c r="K24" s="189"/>
-      <c r="L24" s="25"/>
-      <c r="N24" t="s">
+      <c r="K25" s="190" t="str">
+        <f>=IFERROR(ROUND($K$18-$K$21-$K$22-$K$23,2),0)</f>
+      </c>
+      <c r="L25" s="191" t="str">
+        <f>=IFERROR(ROUND($L$18-$L$21-$L$22-$L$23,2),0)</f>
+      </c>
+      <c r="N25" s="189" t="s">
         <v>334</v>
       </c>
-      <c r="O24" s="189"/>
-      <c r="P24" s="25"/>
-      <c r="R24" t="s">
+      <c r="O25" s="190" t="str">
+        <f>=IFERROR(ROUND($O$18-$O$21-$O$22-$O$23,2),0)</f>
+      </c>
+      <c r="P25" s="191" t="str">
+        <f>=IFERROR(ROUND($P$18-$P$21-$P$22-$P$23,2),0)</f>
+      </c>
+      <c r="R25" s="189" t="s">
         <v>334</v>
       </c>
-      <c r="S24" s="189"/>
-      <c r="T24" s="25"/>
-      <c r="V24" t="s">
+      <c r="S25" s="190" t="str">
+        <f>=IFERROR(ROUND($S$18-$S$21-$S$22-$S$23,2),0)</f>
+      </c>
+      <c r="T25" s="191" t="str">
+        <f>=IFERROR(ROUND($T$18-$T$21-$T$22-$T$23,2),0)</f>
+      </c>
+      <c r="V25" s="189" t="s">
         <v>334</v>
       </c>
-      <c r="W24" s="189"/>
-      <c r="X24" s="25"/>
-      <c r="Z24" t="s">
+      <c r="W25" s="190" t="str">
+        <f>=IFERROR(ROUND($W$18-$W$21-$W$22-$W$23,2),0)</f>
+      </c>
+      <c r="X25" s="191" t="str">
+        <f>=IFERROR(ROUND($X$18-$X$21-$X$22-$X$23,2),0)</f>
+      </c>
+      <c r="Z25" s="189" t="s">
         <v>334</v>
       </c>
-      <c r="AA24" s="189"/>
-      <c r="AB24" s="25"/>
-      <c r="AD24" t="s">
+      <c r="AA25" s="190" t="str">
+        <f>=IFERROR(ROUND($AA$18-$AA$21-$AA$22-$AA$23,2),0)</f>
+      </c>
+      <c r="AB25" s="191" t="str">
+        <f>=IFERROR(ROUND($AB$18-$AB$21-$AB$22-$AB$23,2),0)</f>
+      </c>
+      <c r="AD25" s="189" t="s">
         <v>334</v>
       </c>
-      <c r="AE24" s="189"/>
-      <c r="AF24" s="25"/>
-      <c r="AH24" t="s">
+      <c r="AE25" s="190" t="str">
+        <f>=IFERROR(ROUND($AE$18-$AE$21-$AE$22-$AE$23,2),0)</f>
+      </c>
+      <c r="AF25" s="191" t="str">
+        <f>=IFERROR(ROUND($AF$18-$AF$21-$AF$22-$AF$23,2),0)</f>
+      </c>
+      <c r="AH25" s="189" t="s">
         <v>334</v>
       </c>
-      <c r="AI24" s="189"/>
-      <c r="AJ24" s="25"/>
-      <c r="AL24" t="s">
+      <c r="AI25" s="190" t="str">
+        <f>=IFERROR(ROUND($AI$18-$AI$21-$AI$22-$AI$23,2),0)</f>
+      </c>
+      <c r="AJ25" s="191" t="str">
+        <f>=IFERROR(ROUND($AJ$18-$AJ$21-$AJ$22-$AJ$23,2),0)</f>
+      </c>
+      <c r="AL25" s="189" t="s">
         <v>334</v>
       </c>
-      <c r="AM24" s="189"/>
-      <c r="AN24" s="25"/>
-      <c r="AP24" t="s">
+      <c r="AM25" s="190" t="str">
+        <f>=IFERROR(ROUND($AM$18-$AM$21-$AM$22-$AM$23,2),0)</f>
+      </c>
+      <c r="AN25" s="191" t="str">
+        <f>=IFERROR(ROUND($AN$18-$AN$21-$AN$22-$AN$23,2),0)</f>
+      </c>
+      <c r="AP25" s="189" t="s">
         <v>334</v>
       </c>
-      <c r="AQ24" s="189"/>
-      <c r="AR24" s="25"/>
-      <c r="AT24" t="s">
+      <c r="AQ25" s="190" t="str">
+        <f>=IFERROR(ROUND($AQ$18-$AQ$21-$AQ$22-$AQ$23,2),0)</f>
+      </c>
+      <c r="AR25" s="191" t="str">
+        <f>=IFERROR(ROUND($AR$18-$AR$21-$AR$22-$AR$23,2),0)</f>
+      </c>
+      <c r="AT25" s="189" t="s">
         <v>334</v>
       </c>
-      <c r="AU24" s="189"/>
-      <c r="AV24" s="25"/>
-      <c r="AX24" t="s">
+      <c r="AU25" s="190" t="str">
+        <f>=IFERROR(ROUND($AU$18-$AU$21-$AU$22-$AU$23,2),0)</f>
+      </c>
+      <c r="AV25" s="191" t="str">
+        <f>=IFERROR(ROUND($AV$18-$AV$21-$AV$22-$AV$23,2),0)</f>
+      </c>
+      <c r="AX25" s="189" t="s">
         <v>334</v>
       </c>
-      <c r="AY24" s="189"/>
-      <c r="AZ24" s="25"/>
-      <c r="BB24" t="s">
+      <c r="AY25" s="190" t="str">
+        <f>=IFERROR(ROUND($AY$18-$AY$21-$AY$22-$AY$23,2),0)</f>
+      </c>
+      <c r="AZ25" s="191" t="str">
+        <f>=IFERROR(ROUND($AZ$18-$AZ$21-$AZ$22-$AZ$23,2),0)</f>
+      </c>
+      <c r="BB25" s="189" t="s">
         <v>334</v>
       </c>
-      <c r="BC24" s="189"/>
-      <c r="BD24" s="25"/>
-      <c r="BF24" t="s">
+      <c r="BC25" s="190" t="str">
+        <f>=IFERROR(ROUND($BC$18-$BC$21-$BC$22-$BC$23,2),0)</f>
+      </c>
+      <c r="BD25" s="191" t="str">
+        <f>=IFERROR(ROUND($BD$18-$BD$21-$BD$22-$BD$23,2),0)</f>
+      </c>
+      <c r="BF25" s="189" t="s">
         <v>334</v>
       </c>
-      <c r="BG24" s="189"/>
-      <c r="BH24" s="25"/>
-      <c r="BJ24" t="s">
+      <c r="BG25" s="190" t="str">
+        <f>=IFERROR(ROUND($BG$18-$BG$21-$BG$22-$BG$23,2),0)</f>
+      </c>
+      <c r="BH25" s="191" t="str">
+        <f>=IFERROR(ROUND($BH$18-$BH$21-$BH$22-$BH$23,2),0)</f>
+      </c>
+      <c r="BJ25" s="189" t="s">
         <v>334</v>
       </c>
-      <c r="BK24" s="189"/>
-      <c r="BL24" s="25"/>
-      <c r="BN24" t="s">
+      <c r="BK25" s="190" t="str">
+        <f>=IFERROR(ROUND($BK$18-$BK$21-$BK$22-$BK$23,2),0)</f>
+      </c>
+      <c r="BL25" s="191" t="str">
+        <f>=IFERROR(ROUND($BL$18-$BL$21-$BL$22-$BL$23,2),0)</f>
+      </c>
+      <c r="BN25" s="189" t="s">
         <v>334</v>
       </c>
-      <c r="BO24" s="189"/>
-      <c r="BP24" s="25"/>
-      <c r="BR24" t="s">
+      <c r="BO25" s="190" t="str">
+        <f>=IFERROR(ROUND($BO$18-$BO$21-$BO$22-$BO$23,2),0)</f>
+      </c>
+      <c r="BP25" s="191" t="str">
+        <f>=IFERROR(ROUND($BP$18-$BP$21-$BP$22-$BP$23,2),0)</f>
+      </c>
+      <c r="BR25" s="189" t="s">
         <v>334</v>
       </c>
-      <c r="BS24" s="189"/>
-      <c r="BT24" s="25"/>
-    </row>
-    <row r="25">
-      <c r="B25" s="190" t="s">
+      <c r="BS25" s="190" t="str">
+        <f>=IFERROR(ROUND($BS$18-$BS$21-$BS$22-$BS$23,2),0)</f>
+      </c>
+      <c r="BT25" s="191" t="str">
+        <f>=IFERROR(ROUND($BT$18-$BT$21-$BT$22-$BT$23,2),0)</f>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="181" t="s">
         <v>335</v>
       </c>
-      <c r="C25" s="191" t="str">
-        <f>=IFERROR(ROUND($C$18-$C$21-$C$22-$C$23,2),0)</f>
-      </c>
-      <c r="D25" s="192" t="str">
-        <f>=IFERROR(ROUND($D$18-$D$21-$D$22-$D$23,2),0)</f>
-      </c>
-      <c r="F25" s="190" t="s">
+      <c r="C27" s="181"/>
+      <c r="D27" s="25"/>
+      <c r="F27" s="181" t="s">
         <v>335</v>
       </c>
-      <c r="G25" s="191" t="str">
-        <f>=IFERROR(ROUND($G$18-$G$21-$G$22-$G$23,2),0)</f>
-      </c>
-      <c r="H25" s="192" t="str">
-        <f>=IFERROR(ROUND($H$18-$H$21-$H$22-$H$23,2),0)</f>
-      </c>
-      <c r="J25" s="190" t="s">
+      <c r="G27" s="181"/>
+      <c r="H27" s="25"/>
+      <c r="J27" s="181" t="s">
         <v>335</v>
       </c>
-      <c r="K25" s="191" t="str">
-        <f>=IFERROR(ROUND($K$18-$K$21-$K$22-$K$23,2),0)</f>
-      </c>
-      <c r="L25" s="192" t="str">
-        <f>=IFERROR(ROUND($L$18-$L$21-$L$22-$L$23,2),0)</f>
-      </c>
-      <c r="N25" s="190" t="s">
+      <c r="K27" s="181"/>
+      <c r="L27" s="25"/>
+      <c r="N27" s="181" t="s">
         <v>335</v>
       </c>
-      <c r="O25" s="191" t="str">
-        <f>=IFERROR(ROUND($O$18-$O$21-$O$22-$O$23,2),0)</f>
-      </c>
-      <c r="P25" s="192" t="str">
-        <f>=IFERROR(ROUND($P$18-$P$21-$P$22-$P$23,2),0)</f>
-      </c>
-      <c r="R25" s="190" t="s">
+      <c r="O27" s="181"/>
+      <c r="P27" s="25"/>
+      <c r="R27" s="181" t="s">
         <v>335</v>
       </c>
-      <c r="S25" s="191" t="str">
-        <f>=IFERROR(ROUND($S$18-$S$21-$S$22-$S$23,2),0)</f>
-      </c>
-      <c r="T25" s="192" t="str">
-        <f>=IFERROR(ROUND($T$18-$T$21-$T$22-$T$23,2),0)</f>
-      </c>
-      <c r="V25" s="190" t="s">
+      <c r="S27" s="181"/>
+      <c r="T27" s="25"/>
+      <c r="V27" s="181" t="s">
         <v>335</v>
       </c>
-      <c r="W25" s="191" t="str">
-        <f>=IFERROR(ROUND($W$18-$W$21-$W$22-$W$23,2),0)</f>
-      </c>
-      <c r="X25" s="192" t="str">
-        <f>=IFERROR(ROUND($X$18-$X$21-$X$22-$X$23,2),0)</f>
-      </c>
-      <c r="Z25" s="190" t="s">
+      <c r="W27" s="181"/>
+      <c r="X27" s="25"/>
+      <c r="Z27" s="181" t="s">
         <v>335</v>
       </c>
-      <c r="AA25" s="191" t="str">
-        <f>=IFERROR(ROUND($AA$18-$AA$21-$AA$22-$AA$23,2),0)</f>
-      </c>
-      <c r="AB25" s="192" t="str">
-        <f>=IFERROR(ROUND($AB$18-$AB$21-$AB$22-$AB$23,2),0)</f>
-      </c>
-      <c r="AD25" s="190" t="s">
+      <c r="AA27" s="181"/>
+      <c r="AB27" s="25"/>
+      <c r="AD27" s="181" t="s">
         <v>335</v>
       </c>
-      <c r="AE25" s="191" t="str">
-        <f>=IFERROR(ROUND($AE$18-$AE$21-$AE$22-$AE$23,2),0)</f>
-      </c>
-      <c r="AF25" s="192" t="str">
-        <f>=IFERROR(ROUND($AF$18-$AF$21-$AF$22-$AF$23,2),0)</f>
-      </c>
-      <c r="AH25" s="190" t="s">
+      <c r="AE27" s="181"/>
+      <c r="AF27" s="25"/>
+      <c r="AH27" s="181" t="s">
         <v>335</v>
       </c>
-      <c r="AI25" s="191" t="str">
-        <f>=IFERROR(ROUND($AI$18-$AI$21-$AI$22-$AI$23,2),0)</f>
-      </c>
-      <c r="AJ25" s="192" t="str">
-        <f>=IFERROR(ROUND($AJ$18-$AJ$21-$AJ$22-$AJ$23,2),0)</f>
-      </c>
-      <c r="AL25" s="190" t="s">
+      <c r="AI27" s="181"/>
+      <c r="AJ27" s="25"/>
+      <c r="AL27" s="181" t="s">
         <v>335</v>
       </c>
-      <c r="AM25" s="191" t="str">
-        <f>=IFERROR(ROUND($AM$18-$AM$21-$AM$22-$AM$23,2),0)</f>
-      </c>
-      <c r="AN25" s="192" t="str">
-        <f>=IFERROR(ROUND($AN$18-$AN$21-$AN$22-$AN$23,2),0)</f>
-      </c>
-      <c r="AP25" s="190" t="s">
+      <c r="AM27" s="181"/>
+      <c r="AN27" s="25"/>
+      <c r="AP27" s="181" t="s">
         <v>335</v>
       </c>
-      <c r="AQ25" s="191" t="str">
-        <f>=IFERROR(ROUND($AQ$18-$AQ$21-$AQ$22-$AQ$23,2),0)</f>
-      </c>
-      <c r="AR25" s="192" t="str">
-        <f>=IFERROR(ROUND($AR$18-$AR$21-$AR$22-$AR$23,2),0)</f>
-      </c>
-      <c r="AT25" s="190" t="s">
+      <c r="AQ27" s="181"/>
+      <c r="AR27" s="25"/>
+      <c r="AT27" s="181" t="s">
         <v>335</v>
       </c>
-      <c r="AU25" s="191" t="str">
-        <f>=IFERROR(ROUND($AU$18-$AU$21-$AU$22-$AU$23,2),0)</f>
-      </c>
-      <c r="AV25" s="192" t="str">
-        <f>=IFERROR(ROUND($AV$18-$AV$21-$AV$22-$AV$23,2),0)</f>
-      </c>
-      <c r="AX25" s="190" t="s">
+      <c r="AU27" s="181"/>
+      <c r="AV27" s="25"/>
+      <c r="AX27" s="181" t="s">
         <v>335</v>
       </c>
-      <c r="AY25" s="191" t="str">
-        <f>=IFERROR(ROUND($AY$18-$AY$21-$AY$22-$AY$23,2),0)</f>
-      </c>
-      <c r="AZ25" s="192" t="str">
-        <f>=IFERROR(ROUND($AZ$18-$AZ$21-$AZ$22-$AZ$23,2),0)</f>
-      </c>
-      <c r="BB25" s="190" t="s">
+      <c r="AY27" s="181"/>
+      <c r="AZ27" s="25"/>
+      <c r="BB27" s="181" t="s">
         <v>335</v>
       </c>
-      <c r="BC25" s="191" t="str">
-        <f>=IFERROR(ROUND($BC$18-$BC$21-$BC$22-$BC$23,2),0)</f>
-      </c>
-      <c r="BD25" s="192" t="str">
-        <f>=IFERROR(ROUND($BD$18-$BD$21-$BD$22-$BD$23,2),0)</f>
-      </c>
-      <c r="BF25" s="190" t="s">
+      <c r="BC27" s="181"/>
+      <c r="BD27" s="25"/>
+      <c r="BF27" s="181" t="s">
         <v>335</v>
       </c>
-      <c r="BG25" s="191" t="str">
-        <f>=IFERROR(ROUND($BG$18-$BG$21-$BG$22-$BG$23,2),0)</f>
-      </c>
-      <c r="BH25" s="192" t="str">
-        <f>=IFERROR(ROUND($BH$18-$BH$21-$BH$22-$BH$23,2),0)</f>
-      </c>
-      <c r="BJ25" s="190" t="s">
+      <c r="BG27" s="181"/>
+      <c r="BH27" s="25"/>
+      <c r="BJ27" s="181" t="s">
         <v>335</v>
       </c>
-      <c r="BK25" s="191" t="str">
-        <f>=IFERROR(ROUND($BK$18-$BK$21-$BK$22-$BK$23,2),0)</f>
-      </c>
-      <c r="BL25" s="192" t="str">
-        <f>=IFERROR(ROUND($BL$18-$BL$21-$BL$22-$BL$23,2),0)</f>
-      </c>
-      <c r="BN25" s="190" t="s">
+      <c r="BK27" s="181"/>
+      <c r="BL27" s="25"/>
+      <c r="BN27" s="181" t="s">
         <v>335</v>
       </c>
-      <c r="BO25" s="191" t="str">
-        <f>=IFERROR(ROUND($BO$18-$BO$21-$BO$22-$BO$23,2),0)</f>
-      </c>
-      <c r="BP25" s="192" t="str">
-        <f>=IFERROR(ROUND($BP$18-$BP$21-$BP$22-$BP$23,2),0)</f>
-      </c>
-      <c r="BR25" s="190" t="s">
+      <c r="BO27" s="181"/>
+      <c r="BP27" s="25"/>
+      <c r="BR27" s="181" t="s">
         <v>335</v>
       </c>
-      <c r="BS25" s="191" t="str">
-        <f>=IFERROR(ROUND($BS$18-$BS$21-$BS$22-$BS$23,2),0)</f>
-      </c>
-      <c r="BT25" s="192" t="str">
-        <f>=IFERROR(ROUND($BT$18-$BT$21-$BT$22-$BT$23,2),0)</f>
-      </c>
+      <c r="BS27" s="181"/>
+      <c r="BT27" s="25"/>
     </row>
   </sheetData>
-  <mergeCells count="90">
+  <mergeCells count="108">
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="C8:D8"/>
+    <mergeCell ref="B27:C27"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="G5:H5"/>
     <mergeCell ref="G6:H6"/>
     <mergeCell ref="G7:H7"/>
     <mergeCell ref="G8:H8"/>
+    <mergeCell ref="F27:G27"/>
     <mergeCell ref="K4:L4"/>
     <mergeCell ref="K5:L5"/>
     <mergeCell ref="K6:L6"/>
     <mergeCell ref="K7:L7"/>
     <mergeCell ref="K8:L8"/>
+    <mergeCell ref="J27:K27"/>
     <mergeCell ref="O4:P4"/>
     <mergeCell ref="O5:P5"/>
     <mergeCell ref="O6:P6"/>
     <mergeCell ref="O7:P7"/>
     <mergeCell ref="O8:P8"/>
+    <mergeCell ref="N27:O27"/>
     <mergeCell ref="S4:T4"/>
     <mergeCell ref="S5:T5"/>
     <mergeCell ref="S6:T6"/>
     <mergeCell ref="S7:T7"/>
     <mergeCell ref="S8:T8"/>
+    <mergeCell ref="R27:S27"/>
     <mergeCell ref="W4:X4"/>
     <mergeCell ref="W5:X5"/>
     <mergeCell ref="W6:X6"/>
     <mergeCell ref="W7:X7"/>
     <mergeCell ref="W8:X8"/>
+    <mergeCell ref="V27:W27"/>
     <mergeCell ref="AA4:AB4"/>
     <mergeCell ref="AA5:AB5"/>
     <mergeCell ref="AA6:AB6"/>
     <mergeCell ref="AA7:AB7"/>
     <mergeCell ref="AA8:AB8"/>
+    <mergeCell ref="Z27:AA27"/>
     <mergeCell ref="AE4:AF4"/>
     <mergeCell ref="AE5:AF5"/>
     <mergeCell ref="AE6:AF6"/>
     <mergeCell ref="AE7:AF7"/>
     <mergeCell ref="AE8:AF8"/>
+    <mergeCell ref="AD27:AE27"/>
     <mergeCell ref="AI4:AJ4"/>
     <mergeCell ref="AI5:AJ5"/>
     <mergeCell ref="AI6:AJ6"/>
     <mergeCell ref="AI7:AJ7"/>
     <mergeCell ref="AI8:AJ8"/>
+    <mergeCell ref="AH27:AI27"/>
     <mergeCell ref="AM4:AN4"/>
     <mergeCell ref="AM5:AN5"/>
     <mergeCell ref="AM6:AN6"/>
     <mergeCell ref="AM7:AN7"/>
     <mergeCell ref="AM8:AN8"/>
+    <mergeCell ref="AL27:AM27"/>
     <mergeCell ref="AQ4:AR4"/>
     <mergeCell ref="AQ5:AR5"/>
     <mergeCell ref="AQ6:AR6"/>
     <mergeCell ref="AQ7:AR7"/>
     <mergeCell ref="AQ8:AR8"/>
+    <mergeCell ref="AP27:AQ27"/>
     <mergeCell ref="AU4:AV4"/>
     <mergeCell ref="AU5:AV5"/>
     <mergeCell ref="AU6:AV6"/>
     <mergeCell ref="AU7:AV7"/>
     <mergeCell ref="AU8:AV8"/>
+    <mergeCell ref="AT27:AU27"/>
     <mergeCell ref="AY4:AZ4"/>
     <mergeCell ref="AY5:AZ5"/>
     <mergeCell ref="AY6:AZ6"/>
     <mergeCell ref="AY7:AZ7"/>
     <mergeCell ref="AY8:AZ8"/>
+    <mergeCell ref="AX27:AY27"/>
     <mergeCell ref="BC4:BD4"/>
     <mergeCell ref="BC5:BD5"/>
     <mergeCell ref="BC6:BD6"/>
     <mergeCell ref="BC7:BD7"/>
     <mergeCell ref="BC8:BD8"/>
+    <mergeCell ref="BB27:BC27"/>
     <mergeCell ref="BG4:BH4"/>
     <mergeCell ref="BG5:BH5"/>
     <mergeCell ref="BG6:BH6"/>
     <mergeCell ref="BG7:BH7"/>
     <mergeCell ref="BG8:BH8"/>
+    <mergeCell ref="BF27:BG27"/>
     <mergeCell ref="BK4:BL4"/>
     <mergeCell ref="BK5:BL5"/>
     <mergeCell ref="BK6:BL6"/>
     <mergeCell ref="BK7:BL7"/>
     <mergeCell ref="BK8:BL8"/>
+    <mergeCell ref="BJ27:BK27"/>
     <mergeCell ref="BO4:BP4"/>
     <mergeCell ref="BO5:BP5"/>
     <mergeCell ref="BO6:BP6"/>
     <mergeCell ref="BO7:BP7"/>
     <mergeCell ref="BO8:BP8"/>
+    <mergeCell ref="BN27:BO27"/>
     <mergeCell ref="BS4:BT4"/>
     <mergeCell ref="BS5:BT5"/>
     <mergeCell ref="BS6:BT6"/>
     <mergeCell ref="BS7:BT7"/>
     <mergeCell ref="BS8:BT8"/>
+    <mergeCell ref="BR27:BS27"/>
   </mergeCells>
   <dataValidations count="18">
     <dataValidation allowBlank="true" sqref="C4" type="list">
@@ -21502,64 +21520,64 @@
   </cols>
   <sheetData>
     <row r="2" ht="30" customHeight="true">
-      <c r="B2" s="193" t="s">
+      <c r="B2" s="192" t="s">
         <v>337</v>
       </c>
-      <c r="C2" s="193"/>
-      <c r="D2" s="193"/>
-      <c r="E2" s="193"/>
-      <c r="F2" s="193"/>
-      <c r="G2" s="193"/>
-      <c r="H2" s="193"/>
-      <c r="I2" s="193"/>
-      <c r="J2" s="193"/>
+      <c r="C2" s="192"/>
+      <c r="D2" s="192"/>
+      <c r="E2" s="192"/>
+      <c r="F2" s="192"/>
+      <c r="G2" s="192"/>
+      <c r="H2" s="192"/>
+      <c r="I2" s="192"/>
+      <c r="J2" s="192"/>
     </row>
     <row r="3" ht="18" customHeight="true">
-      <c r="B3" s="194" t="s">
+      <c r="B3" s="193" t="s">
         <v>338</v>
       </c>
-      <c r="C3" s="194"/>
-      <c r="D3" s="194"/>
-      <c r="E3" s="194"/>
-      <c r="F3" s="194"/>
-      <c r="G3" s="194"/>
-      <c r="H3" s="194"/>
-      <c r="I3" s="194"/>
-      <c r="J3" s="194"/>
+      <c r="C3" s="193"/>
+      <c r="D3" s="193"/>
+      <c r="E3" s="193"/>
+      <c r="F3" s="193"/>
+      <c r="G3" s="193"/>
+      <c r="H3" s="193"/>
+      <c r="I3" s="193"/>
+      <c r="J3" s="193"/>
     </row>
     <row r="5" ht="22" customHeight="true">
-      <c r="B5" s="195" t="s">
+      <c r="B5" s="194" t="s">
         <v>339</v>
       </c>
-      <c r="C5" s="195"/>
-      <c r="D5" s="195"/>
-      <c r="E5" s="195"/>
-      <c r="F5" s="195"/>
-      <c r="G5" s="195"/>
-      <c r="H5" s="195"/>
-      <c r="I5" s="195"/>
-      <c r="J5" s="195"/>
-      <c r="L5" s="203" t="str">
+      <c r="C5" s="194"/>
+      <c r="D5" s="194"/>
+      <c r="E5" s="194"/>
+      <c r="F5" s="194"/>
+      <c r="G5" s="194"/>
+      <c r="H5" s="194"/>
+      <c r="I5" s="194"/>
+      <c r="J5" s="194"/>
+      <c r="L5" s="202" t="str">
         <f>=IF(E11=0,"Aktuelle Mittelanforderung (keine gewählt)","Aktuelle Mittelanforderung – Periode "&amp;E10&amp;" (#"&amp;E11&amp;")")</f>
       </c>
-      <c r="M5" s="204"/>
-      <c r="N5" s="205"/>
+      <c r="M5" s="203"/>
+      <c r="N5" s="204"/>
       <c r="AD5" t="str">
         <f>=IFERROR(SUMPRODUCT('Daten'!$BA$1:$BA$18,('Daten'!$BB$1:$BB$18=E10)*('Daten'!$BD$1:$BD$18=E11)),0)</f>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="196" t="s">
+      <c r="B6" s="195" t="s">
         <v>340</v>
       </c>
-      <c r="C6" s="196"/>
-      <c r="D6" s="196"/>
-      <c r="E6" s="196"/>
-      <c r="F6" s="196"/>
-      <c r="G6" s="196"/>
-      <c r="H6" s="196"/>
-      <c r="I6" s="196"/>
-      <c r="J6" s="196"/>
+      <c r="C6" s="195"/>
+      <c r="D6" s="195"/>
+      <c r="E6" s="195"/>
+      <c r="F6" s="195"/>
+      <c r="G6" s="195"/>
+      <c r="H6" s="195"/>
+      <c r="I6" s="195"/>
+      <c r="J6" s="195"/>
       <c r="L6" s="315" t="s">
         <v>288</v>
       </c>
@@ -21578,13 +21596,13 @@
       <c r="N7" s="317"/>
     </row>
     <row r="8" ht="22" customHeight="true">
-      <c r="C8" s="203" t="s">
+      <c r="C8" s="202" t="s">
         <v>341</v>
       </c>
-      <c r="D8" s="204"/>
-      <c r="E8" s="204"/>
-      <c r="F8" s="204"/>
-      <c r="G8" s="205"/>
+      <c r="D8" s="203"/>
+      <c r="E8" s="203"/>
+      <c r="F8" s="203"/>
+      <c r="G8" s="204"/>
       <c r="L8" s="315" t="s">
         <v>290</v>
       </c>
@@ -21594,15 +21612,15 @@
       <c r="N8" s="317"/>
     </row>
     <row r="9">
-      <c r="C9" s="206" t="s">
+      <c r="C9" s="205" t="s">
         <v>342</v>
       </c>
-      <c r="D9" s="198"/>
+      <c r="D9" s="197"/>
       <c r="E9" s="63" t="s">
         <v>343</v>
       </c>
       <c r="F9" s="63"/>
-      <c r="G9" s="207"/>
+      <c r="G9" s="206"/>
       <c r="L9" s="315" t="s">
         <v>291</v>
       </c>
@@ -21612,16 +21630,16 @@
       <c r="N9" s="318"/>
     </row>
     <row r="10">
-      <c r="C10" s="206" t="s">
+      <c r="C10" s="205" t="s">
         <v>344</v>
       </c>
-      <c r="D10" s="198"/>
-      <c r="E10" s="199" t="str">
+      <c r="D10" s="197"/>
+      <c r="E10" s="198" t="str">
         <f>=E81+1</f>
         <v>0</v>
       </c>
-      <c r="F10" s="199"/>
-      <c r="G10" s="208"/>
+      <c r="F10" s="198"/>
+      <c r="G10" s="207"/>
       <c r="L10" s="315" t="s">
         <v>326</v>
       </c>
@@ -21631,26 +21649,26 @@
       <c r="N10" s="319"/>
     </row>
     <row r="11">
-      <c r="C11" s="206" t="s">
+      <c r="C11" s="205" t="s">
         <v>345</v>
       </c>
-      <c r="D11" s="198"/>
-      <c r="E11" s="199" t="str">
+      <c r="D11" s="197"/>
+      <c r="E11" s="198" t="str">
         <f>=IF(E9="Neuste MA",IFERROR(SUMPRODUCT(MAX(('Daten'!$BB$1:$BB$18=E10)*('Daten'!$BC$1:$BC$18=1)*'Daten'!$BD$1:$BD$18)),0),IFERROR(VALUE(MID(E9,FIND("(#",E9)+2,FIND(")",E9)-FIND("(#",E9)-2)),0))</f>
       </c>
-      <c r="F11" s="199"/>
-      <c r="G11" s="209"/>
+      <c r="F11" s="198"/>
+      <c r="G11" s="208"/>
       <c r="L11" s="47"/>
       <c r="N11" s="48"/>
     </row>
     <row r="12">
-      <c r="C12" s="210" t="s">
+      <c r="C12" s="209" t="s">
         <v>346</v>
       </c>
-      <c r="D12" s="200"/>
-      <c r="E12" s="200"/>
-      <c r="F12" s="200"/>
-      <c r="G12" s="211"/>
+      <c r="D12" s="199"/>
+      <c r="E12" s="199"/>
+      <c r="F12" s="199"/>
+      <c r="G12" s="210"/>
       <c r="L12" s="320" t="s">
         <v>202</v>
       </c>
@@ -21662,15 +21680,15 @@
       </c>
     </row>
     <row r="13">
-      <c r="C13" s="212" t="str">
+      <c r="C13" s="211" t="str">
         <f>=IF(1&lt;=E11,"Periode "&amp;E10&amp;" (#1)","")</f>
       </c>
-      <c r="D13" s="201"/>
-      <c r="E13" s="202" t="str">
+      <c r="D13" s="200"/>
+      <c r="E13" s="201" t="str">
         <f>=IF(1&lt;=E11,IFERROR(SUMIFS('Daten'!$BF$1:$BF$18,'Daten'!$BB$1:$BB$18,E10,'Daten'!$BD$1:$BD$18,1),0),"")</f>
       </c>
-      <c r="F13" s="202"/>
-      <c r="G13" s="213" t="str">
+      <c r="F13" s="201"/>
+      <c r="G13" s="212" t="str">
         <f>=IF(1&lt;=E11,IFERROR(SUMIFS('Daten'!$BG$1:$BG$18,'Daten'!$BB$1:$BB$18,E10,'Daten'!$BD$1:$BD$18,1),0),"")</f>
       </c>
       <c r="L13" s="143" t="s">
@@ -21684,15 +21702,15 @@
       </c>
     </row>
     <row r="14">
-      <c r="C14" s="212" t="str">
+      <c r="C14" s="211" t="str">
         <f>=IF(2&lt;=E11,"Periode "&amp;E10&amp;" (#2)","")</f>
       </c>
-      <c r="D14" s="201"/>
-      <c r="E14" s="202" t="str">
+      <c r="D14" s="200"/>
+      <c r="E14" s="201" t="str">
         <f>=IF(2&lt;=E11,IFERROR(SUMIFS('Daten'!$BF$1:$BF$18,'Daten'!$BB$1:$BB$18,E10,'Daten'!$BD$1:$BD$18,2),0),"")</f>
       </c>
-      <c r="F14" s="202"/>
-      <c r="G14" s="213" t="str">
+      <c r="F14" s="201"/>
+      <c r="G14" s="212" t="str">
         <f>=IF(2&lt;=E11,IFERROR(SUMIFS('Daten'!$BG$1:$BG$18,'Daten'!$BB$1:$BB$18,E10,'Daten'!$BD$1:$BD$18,2),0),"")</f>
       </c>
       <c r="L14" s="143" t="s">
@@ -21706,15 +21724,15 @@
       </c>
     </row>
     <row r="15">
-      <c r="C15" s="212" t="str">
+      <c r="C15" s="211" t="str">
         <f>=IF(3&lt;=E11,"Periode "&amp;E10&amp;" (#3)","")</f>
       </c>
-      <c r="D15" s="201"/>
-      <c r="E15" s="202" t="str">
+      <c r="D15" s="200"/>
+      <c r="E15" s="201" t="str">
         <f>=IF(3&lt;=E11,IFERROR(SUMIFS('Daten'!$BF$1:$BF$18,'Daten'!$BB$1:$BB$18,E10,'Daten'!$BD$1:$BD$18,3),0),"")</f>
       </c>
-      <c r="F15" s="202"/>
-      <c r="G15" s="213" t="str">
+      <c r="F15" s="201"/>
+      <c r="G15" s="212" t="str">
         <f>=IF(3&lt;=E11,IFERROR(SUMIFS('Daten'!$BG$1:$BG$18,'Daten'!$BB$1:$BB$18,E10,'Daten'!$BD$1:$BD$18,3),0),"")</f>
       </c>
       <c r="L15" s="143" t="s">
@@ -21728,15 +21746,15 @@
       </c>
     </row>
     <row r="16">
-      <c r="C16" s="212" t="str">
+      <c r="C16" s="211" t="str">
         <f>=IF(4&lt;=E11,"Periode "&amp;E10&amp;" (#4)","")</f>
       </c>
-      <c r="D16" s="201"/>
-      <c r="E16" s="202" t="str">
+      <c r="D16" s="200"/>
+      <c r="E16" s="201" t="str">
         <f>=IF(4&lt;=E11,IFERROR(SUMIFS('Daten'!$BF$1:$BF$18,'Daten'!$BB$1:$BB$18,E10,'Daten'!$BD$1:$BD$18,4),0),"")</f>
       </c>
-      <c r="F16" s="202"/>
-      <c r="G16" s="213" t="str">
+      <c r="F16" s="201"/>
+      <c r="G16" s="212" t="str">
         <f>=IF(4&lt;=E11,IFERROR(SUMIFS('Daten'!$BG$1:$BG$18,'Daten'!$BB$1:$BB$18,E10,'Daten'!$BD$1:$BD$18,4),0),"")</f>
       </c>
       <c r="L16" s="143" t="s">
@@ -21750,15 +21768,15 @@
       </c>
     </row>
     <row r="17">
-      <c r="C17" s="212" t="str">
+      <c r="C17" s="211" t="str">
         <f>=IF(5&lt;=E11,"Periode "&amp;E10&amp;" (#5)","")</f>
       </c>
-      <c r="D17" s="201"/>
-      <c r="E17" s="202" t="str">
+      <c r="D17" s="200"/>
+      <c r="E17" s="201" t="str">
         <f>=IF(5&lt;=E11,IFERROR(SUMIFS('Daten'!$BF$1:$BF$18,'Daten'!$BB$1:$BB$18,E10,'Daten'!$BD$1:$BD$18,5),0),"")</f>
       </c>
-      <c r="F17" s="202"/>
-      <c r="G17" s="213" t="str">
+      <c r="F17" s="201"/>
+      <c r="G17" s="212" t="str">
         <f>=IF(5&lt;=E11,IFERROR(SUMIFS('Daten'!$BG$1:$BG$18,'Daten'!$BB$1:$BB$18,E10,'Daten'!$BD$1:$BD$18,5),0),"")</f>
       </c>
       <c r="L17" s="143" t="s">
@@ -21772,15 +21790,15 @@
       </c>
     </row>
     <row r="18">
-      <c r="C18" s="214" t="str">
+      <c r="C18" s="213" t="str">
         <f>=IF(6&lt;=E11,"Periode "&amp;E10&amp;" (#6)","")</f>
       </c>
-      <c r="D18" s="215"/>
-      <c r="E18" s="216" t="str">
+      <c r="D18" s="214"/>
+      <c r="E18" s="215" t="str">
         <f>=IF(6&lt;=E11,IFERROR(SUMIFS('Daten'!$BF$1:$BF$18,'Daten'!$BB$1:$BB$18,E10,'Daten'!$BD$1:$BD$18,6),0),"")</f>
       </c>
-      <c r="F18" s="216"/>
-      <c r="G18" s="217" t="str">
+      <c r="F18" s="215"/>
+      <c r="G18" s="216" t="str">
         <f>=IF(6&lt;=E11,IFERROR(SUMIFS('Daten'!$BG$1:$BG$18,'Daten'!$BB$1:$BB$18,E10,'Daten'!$BD$1:$BD$18,6),0),"")</f>
       </c>
       <c r="L18" s="143" t="s">
@@ -21833,43 +21851,43 @@
       <c r="M21" s="243" t="str">
         <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$C$18,'IV. MA'!$G$18,'IV. MA'!$K$18,'IV. MA'!$O$18,'IV. MA'!$S$18,'IV. MA'!$W$18,'IV. MA'!$AA$18,'IV. MA'!$AE$18,'IV. MA'!$AI$18,'IV. MA'!$AM$18,'IV. MA'!$AQ$18,'IV. MA'!$AU$18,'IV. MA'!$AY$18,'IV. MA'!$BC$18,'IV. MA'!$BG$18,'IV. MA'!$BK$18,'IV. MA'!$BO$18,'IV. MA'!$BS$18),"")</f>
       </c>
-      <c r="N21" s="236" t="str">
+      <c r="N21" s="235" t="str">
         <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$D$18,'IV. MA'!$H$18,'IV. MA'!$L$18,'IV. MA'!$P$18,'IV. MA'!$T$18,'IV. MA'!$X$18,'IV. MA'!$AB$18,'IV. MA'!$AF$18,'IV. MA'!$AJ$18,'IV. MA'!$AN$18,'IV. MA'!$AR$18,'IV. MA'!$AV$18,'IV. MA'!$AZ$18,'IV. MA'!$BD$18,'IV. MA'!$BH$18,'IV. MA'!$BL$18,'IV. MA'!$BP$18,'IV. MA'!$BT$18),"")</f>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="224" t="s">
+      <c r="B22" s="223" t="s">
         <v>348</v>
       </c>
-      <c r="C22" s="225"/>
-      <c r="D22" s="226" t="str">
+      <c r="C22" s="224"/>
+      <c r="D22" s="225" t="str">
         <f>=IFERROR(ROUND(KMW_Mittel_EUR,2),0)</f>
       </c>
-      <c r="F22" s="231" t="s">
+      <c r="F22" s="230" t="s">
         <v>352</v>
       </c>
-      <c r="G22" s="232"/>
-      <c r="H22" s="232"/>
-      <c r="I22" s="233"/>
+      <c r="G22" s="231"/>
+      <c r="H22" s="231"/>
+      <c r="I22" s="232"/>
       <c r="L22" s="47"/>
       <c r="N22" s="48"/>
     </row>
     <row r="23">
-      <c r="B23" s="206" t="s">
+      <c r="B23" s="205" t="s">
         <v>349</v>
       </c>
-      <c r="C23" s="198"/>
-      <c r="D23" s="227" t="str">
+      <c r="C23" s="197"/>
+      <c r="D23" s="226" t="str">
         <f>=IFERROR(ROUND(Kosten_Reserve_EUR,2),0)</f>
       </c>
-      <c r="F23" s="234" t="s">
+      <c r="F23" s="233" t="s">
         <v>353</v>
       </c>
-      <c r="G23" s="198" t="s">
+      <c r="G23" s="197" t="s">
         <v>354</v>
       </c>
-      <c r="H23" s="198"/>
-      <c r="I23" s="235" t="str">
+      <c r="H23" s="197"/>
+      <c r="I23" s="234" t="str">
         <f>=IFERROR(ROUND(Saldovortrag_EUR,2),0)</f>
       </c>
       <c r="L23" s="143" t="s">
@@ -21883,21 +21901,21 @@
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="206" t="str">
+      <c r="B24" s="205" t="str">
         <f>=IF(Reserve_Freigabe="Ja","Operatives Budget (Reserve freigegeben)","Operatives Budget (abzgl. Reserve)")</f>
       </c>
-      <c r="C24" s="198"/>
-      <c r="D24" s="227" t="str">
+      <c r="C24" s="197"/>
+      <c r="D24" s="226" t="str">
         <f>=IF(Reserve_Freigabe="Ja",ROUND($D$22,2),ROUND($D$22-$D$23,2))</f>
       </c>
-      <c r="F24" s="234" t="s">
+      <c r="F24" s="233" t="s">
         <v>353</v>
       </c>
-      <c r="G24" s="198" t="s">
+      <c r="G24" s="197" t="s">
         <v>355</v>
       </c>
-      <c r="H24" s="198"/>
-      <c r="I24" s="235" t="str">
+      <c r="H24" s="197"/>
+      <c r="I24" s="234" t="str">
         <f>=I87</f>
         <v>0</v>
       </c>
@@ -21912,21 +21930,21 @@
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="206" t="s">
+      <c r="B25" s="205" t="s">
         <v>350</v>
       </c>
-      <c r="C25" s="198"/>
-      <c r="D25" s="227" t="str">
+      <c r="C25" s="197"/>
+      <c r="D25" s="226" t="str">
         <f>=IFERROR(ROUND(SUBTOTAL(109,TblKMWMittel[Betrag]),2),0)</f>
       </c>
-      <c r="F25" s="234" t="s">
+      <c r="F25" s="233" t="s">
         <v>353</v>
       </c>
-      <c r="G25" s="198" t="s">
+      <c r="G25" s="197" t="s">
         <v>356</v>
       </c>
-      <c r="H25" s="198"/>
-      <c r="I25" s="235" t="str">
+      <c r="H25" s="197"/>
+      <c r="I25" s="234" t="str">
         <f>=ROUND(MAX(0,MAX(0,(SUM($G$96:$G$99)-$G$98)+SUMIFS('Daten'!$BH$1:$BH$18,'Daten'!$BB$1:$BB$18,E10,'Daten'!$BD$1:$BD$18,"&lt;="&amp;E11,'Daten'!$BD$1:$BD$18,"&gt;=1")-(SUM($H$96:$H$99)-$H$98))-I87),2)</f>
         <v>0</v>
       </c>
@@ -21941,19 +21959,19 @@
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="228" t="s">
+      <c r="B26" s="227" t="s">
         <v>351</v>
       </c>
-      <c r="C26" s="229"/>
-      <c r="D26" s="230" t="str">
+      <c r="C26" s="228"/>
+      <c r="D26" s="229" t="str">
         <f>=ROUND($D$24-$D$25,2)</f>
       </c>
       <c r="F26" s="47"/>
-      <c r="G26" s="219" t="s">
+      <c r="G26" s="218" t="s">
         <v>357</v>
       </c>
-      <c r="H26" s="219"/>
-      <c r="I26" s="236" t="str">
+      <c r="H26" s="218"/>
+      <c r="I26" s="235" t="str">
         <f>=ROUND(IF($F$23="Abzug",MAX(0,$I$23),0)+IF($F$24="Abzug",MAX(0,$I$24),0)+IF($F$25="Abzug",MAX(0,$I$25),0),2)</f>
       </c>
       <c r="L26" s="143" t="str">
@@ -21967,12 +21985,12 @@
       </c>
     </row>
     <row r="27">
-      <c r="F27" s="237"/>
-      <c r="G27" s="229" t="s">
+      <c r="F27" s="236"/>
+      <c r="G27" s="228" t="s">
         <v>358</v>
       </c>
-      <c r="H27" s="229"/>
-      <c r="I27" s="230" t="str">
+      <c r="H27" s="228"/>
+      <c r="I27" s="229" t="str">
         <f>=ROUND($D$26-$I$26,2)</f>
       </c>
       <c r="L27" s="47"/>
@@ -21980,7 +21998,7 @@
     </row>
     <row r="28">
       <c r="L28" s="323" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="M28" s="324" t="str">
         <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$C$25,'IV. MA'!$G$25,'IV. MA'!$K$25,'IV. MA'!$O$25,'IV. MA'!$S$25,'IV. MA'!$W$25,'IV. MA'!$AA$25,'IV. MA'!$AE$25,'IV. MA'!$AI$25,'IV. MA'!$AM$25,'IV. MA'!$AQ$25,'IV. MA'!$AU$25,'IV. MA'!$AY$25,'IV. MA'!$BC$25,'IV. MA'!$BG$25,'IV. MA'!$BK$25,'IV. MA'!$BO$25,'IV. MA'!$BS$25),"")</f>
@@ -21990,70 +22008,70 @@
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="224" t="s">
+      <c r="B29" s="223" t="s">
         <v>359</v>
       </c>
-      <c r="C29" s="225"/>
-      <c r="D29" s="226" t="str">
+      <c r="C29" s="224"/>
+      <c r="D29" s="225" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"KMW-Mittel",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,E11),2),0)</f>
       </c>
-      <c r="F29" s="224" t="s">
+      <c r="F29" s="223" t="s">
         <v>359</v>
       </c>
-      <c r="G29" s="225"/>
-      <c r="H29" s="225"/>
-      <c r="I29" s="226" t="str">
+      <c r="G29" s="224"/>
+      <c r="H29" s="224"/>
+      <c r="I29" s="225" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"KMW-Mittel",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,E11),2),0)</f>
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="228" t="s">
+      <c r="B30" s="227" t="s">
         <v>360</v>
       </c>
-      <c r="C30" s="229"/>
-      <c r="D30" s="230" t="str">
+      <c r="C30" s="228"/>
+      <c r="D30" s="229" t="str">
         <f>=ROUND($D$26-MAX(0,$D$29),2)</f>
       </c>
-      <c r="F30" s="228" t="s">
+      <c r="F30" s="227" t="s">
         <v>361</v>
       </c>
-      <c r="G30" s="229"/>
-      <c r="H30" s="229"/>
-      <c r="I30" s="230" t="str">
+      <c r="G30" s="228"/>
+      <c r="H30" s="228"/>
+      <c r="I30" s="229" t="str">
         <f>=ROUND($I$27-MAX(0,$I$29),2)</f>
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="224" t="s">
+      <c r="B32" s="223" t="s">
         <v>362</v>
       </c>
-      <c r="C32" s="225"/>
-      <c r="D32" s="238" t="str">
+      <c r="C32" s="224"/>
+      <c r="D32" s="237" t="str">
         <f>=IFERROR(CHOOSE(E10,MA_ManBetrag_1,MA_ManBetrag_2,MA_ManBetrag_3,MA_ManBetrag_4,MA_ManBetrag_5,MA_ManBetrag_6,MA_ManBetrag_7,MA_ManBetrag_8,MA_ManBetrag_9,MA_ManBetrag_10,MA_ManBetrag_11,MA_ManBetrag_12,MA_ManBetrag_13,MA_ManBetrag_14,MA_ManBetrag_15,MA_ManBetrag_16,MA_ManBetrag_17,MA_ManBetrag_18),0)</f>
       </c>
-      <c r="F32" s="224" t="s">
+      <c r="F32" s="223" t="s">
         <v>362</v>
       </c>
-      <c r="G32" s="225"/>
-      <c r="H32" s="225"/>
-      <c r="I32" s="238" t="str">
+      <c r="G32" s="224"/>
+      <c r="H32" s="224"/>
+      <c r="I32" s="237" t="str">
         <f>=IFERROR(CHOOSE(E10,MA_ManBetrag_1,MA_ManBetrag_2,MA_ManBetrag_3,MA_ManBetrag_4,MA_ManBetrag_5,MA_ManBetrag_6,MA_ManBetrag_7,MA_ManBetrag_8,MA_ManBetrag_9,MA_ManBetrag_10,MA_ManBetrag_11,MA_ManBetrag_12,MA_ManBetrag_13,MA_ManBetrag_14,MA_ManBetrag_15,MA_ManBetrag_16,MA_ManBetrag_17,MA_ManBetrag_18),0)</f>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="228" t="s">
+      <c r="B33" s="227" t="s">
         <v>360</v>
       </c>
-      <c r="C33" s="229"/>
-      <c r="D33" s="230" t="str">
+      <c r="C33" s="228"/>
+      <c r="D33" s="229" t="str">
         <f>=ROUND($D$26-MAX(0,$D$29)-MAX(0,$D$32),2)</f>
       </c>
-      <c r="F33" s="228" t="s">
+      <c r="F33" s="227" t="s">
         <v>361</v>
       </c>
-      <c r="G33" s="229"/>
-      <c r="H33" s="229"/>
-      <c r="I33" s="230" t="str">
+      <c r="G33" s="228"/>
+      <c r="H33" s="228"/>
+      <c r="I33" s="229" t="str">
         <f>=ROUND($I$27-MAX(0,$I$29)-MAX(0,$I$32),2)</f>
       </c>
     </row>
@@ -22085,61 +22103,61 @@
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="206" t="s">
+      <c r="B39" s="205" t="s">
         <v>367</v>
       </c>
-      <c r="C39" s="240" t="str">
+      <c r="C39" s="239" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BF$1:$BF$18,'Daten'!$BB$1:$BB$18,E10,'Daten'!$BD$1:$BD$18,"&lt;="&amp;E11,'Daten'!$BD$1:$BD$18,"&gt;=1"),2),0)</f>
       </c>
-      <c r="D39" s="189"/>
-      <c r="E39" s="227" t="str">
+      <c r="D39" s="240"/>
+      <c r="E39" s="226" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BG$1:$BG$18,'Daten'!$BB$1:$BB$18,E10,'Daten'!$BD$1:$BD$18,"&lt;="&amp;E11,'Daten'!$BD$1:$BD$18,"&gt;=1"),2),0)</f>
       </c>
     </row>
     <row r="40">
-      <c r="B40" s="206" t="s">
+      <c r="B40" s="205" t="s">
         <v>368</v>
       </c>
-      <c r="C40" s="240" t="str">
+      <c r="C40" s="239" t="str">
         <f>=IFERROR(ROUND(SUBTOTAL(109,TblBudgetAusgaben[Jahr 1]),2),0)</f>
       </c>
       <c r="D40" s="241">
         <v>8</v>
       </c>
-      <c r="E40" s="227" t="str">
+      <c r="E40" s="226" t="str">
         <f>=IFERROR(ROUND($C$40/Budget_Kurs,2),0)</f>
       </c>
     </row>
     <row r="41">
-      <c r="B41" s="206" t="s">
+      <c r="B41" s="205" t="s">
         <v>369</v>
       </c>
-      <c r="C41" s="240" t="str">
+      <c r="C41" s="239" t="str">
         <f>=IFERROR(ROUND(SUBTOTAL(109,TblBudgetAusgaben[Jahr 2]),2),0)</f>
       </c>
       <c r="D41" s="241">
         <v>0</v>
       </c>
-      <c r="E41" s="227" t="str">
+      <c r="E41" s="226" t="str">
         <f>=IFERROR(ROUND($C$41/Budget_Kurs,2),0)</f>
       </c>
     </row>
     <row r="42">
-      <c r="B42" s="206" t="s">
+      <c r="B42" s="205" t="s">
         <v>370</v>
       </c>
-      <c r="C42" s="240" t="str">
+      <c r="C42" s="239" t="str">
         <f>=IFERROR(ROUND(SUBTOTAL(109,TblBudgetAusgaben[Jahr 3]),2),0)</f>
       </c>
       <c r="D42" s="241">
         <v>0</v>
       </c>
-      <c r="E42" s="227" t="str">
+      <c r="E42" s="226" t="str">
         <f>=IFERROR(ROUND($C$42/Budget_Kurs,2),0)</f>
       </c>
     </row>
     <row r="43">
-      <c r="B43" s="206" t="s">
+      <c r="B43" s="205" t="s">
         <v>371</v>
       </c>
       <c r="C43" s="242" t="str">
@@ -22149,7 +22167,7 @@
       <c r="E43" s="249"/>
     </row>
     <row r="44">
-      <c r="B44" s="206" t="s">
+      <c r="B44" s="205" t="s">
         <v>372</v>
       </c>
       <c r="C44" s="242" t="str">
@@ -22165,8 +22183,8 @@
       <c r="C45" s="243" t="str">
         <f>=IFERROR(ROUND($C$40*$D$40/12+$C$41*$D$41/12+$C$42*$D$42/12,2),0)</f>
       </c>
-      <c r="D45" s="189"/>
-      <c r="E45" s="236" t="str">
+      <c r="D45" s="240"/>
+      <c r="E45" s="235" t="str">
         <f>=IFERROR(ROUND($E$40*$D$40/12+$E$41*$D$41/12+$E$42*$D$42/12,2),0)</f>
       </c>
     </row>
@@ -22177,20 +22195,20 @@
       <c r="C46" s="244" t="str">
         <f>=IF($C$39&lt;=$C$45,"OK","ÜBERSCHRITTEN")</f>
       </c>
-      <c r="D46" s="189"/>
+      <c r="D46" s="240"/>
       <c r="E46" s="252" t="str">
         <f>=IF($E$39&lt;=$E$45,"OK","ÜBERSCHRITTEN")</f>
       </c>
     </row>
     <row r="47">
-      <c r="B47" s="206" t="s">
+      <c r="B47" s="205" t="s">
         <v>375</v>
       </c>
-      <c r="C47" s="240" t="str">
+      <c r="C47" s="239" t="str">
         <f>=ROUND(MAX(0,$C$39-$C$45),2)</f>
       </c>
-      <c r="D47" s="189"/>
-      <c r="E47" s="227" t="str">
+      <c r="D47" s="240"/>
+      <c r="E47" s="226" t="str">
         <f>=ROUND(MAX(0,$E$39-$E$45),2)</f>
       </c>
     </row>
@@ -22252,22 +22270,22 @@
       <c r="B53" s="266" t="s">
         <v>194</v>
       </c>
-      <c r="C53" s="240" t="str">
+      <c r="C53" s="239" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"Eigenmittel",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="D53" s="240" t="str">
+      <c r="D53" s="239" t="str">
         <f>=IFERROR(ROUND(Eigenmittel_LW,2),0)</f>
       </c>
-      <c r="E53" s="202" t="str">
+      <c r="E53" s="201" t="str">
         <f>=ROUND(IFERROR($C$53-$D$53,0),2)</f>
       </c>
       <c r="F53" s="258" t="str">
         <f>=ROUND(IFERROR(($C$53/$D$53)-1,0),4)</f>
       </c>
-      <c r="G53" s="218" t="str">
+      <c r="G53" s="217" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"Eigenmittel",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="H53" s="218" t="str">
+      <c r="H53" s="217" t="str">
         <f>=IFERROR(ROUND(Eigenmittel_EUR,2),0)</f>
       </c>
       <c r="I53" s="182" t="str">
@@ -22281,22 +22299,22 @@
       <c r="B54" s="266" t="s">
         <v>300</v>
       </c>
-      <c r="C54" s="240" t="str">
+      <c r="C54" s="239" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"Drittmittel",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="D54" s="240" t="str">
+      <c r="D54" s="239" t="str">
         <f>=IFERROR(ROUND(Drittmittel_LW,2),0)</f>
       </c>
-      <c r="E54" s="202" t="str">
+      <c r="E54" s="201" t="str">
         <f>=ROUND(IFERROR($C$54-$D$54,0),2)</f>
       </c>
       <c r="F54" s="258" t="str">
         <f>=ROUND(IFERROR(($C$54/$D$54)-1,0),4)</f>
       </c>
-      <c r="G54" s="218" t="str">
+      <c r="G54" s="217" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"Drittmittel",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="H54" s="218" t="str">
+      <c r="H54" s="217" t="str">
         <f>=IFERROR(ROUND(Drittmittel_EUR,2),0)</f>
       </c>
       <c r="I54" s="182" t="str">
@@ -22310,22 +22328,22 @@
       <c r="B55" s="266" t="s">
         <v>199</v>
       </c>
-      <c r="C55" s="240" t="str">
+      <c r="C55" s="239" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"KMW-Mittel",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="D55" s="240" t="str">
+      <c r="D55" s="239" t="str">
         <f>=IFERROR(ROUND(KMW_Mittel_LW,2),0)</f>
       </c>
-      <c r="E55" s="202" t="str">
+      <c r="E55" s="201" t="str">
         <f>=ROUND(IFERROR($C$55-$D$55,0),2)</f>
       </c>
       <c r="F55" s="258" t="str">
         <f>=ROUND(IFERROR(($C$55/$D$55)-1,0),4)</f>
       </c>
-      <c r="G55" s="218" t="str">
+      <c r="G55" s="217" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"KMW-Mittel",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="H55" s="218" t="str">
+      <c r="H55" s="217" t="str">
         <f>=IFERROR(ROUND(KMW_Mittel_EUR,2),0)</f>
       </c>
       <c r="I55" s="182" t="str">
@@ -22339,22 +22357,22 @@
       <c r="B56" s="266" t="s">
         <v>301</v>
       </c>
-      <c r="C56" s="240" t="str">
+      <c r="C56" s="239" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"Zinsertraege",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="D56" s="240" t="str">
+      <c r="D56" s="239" t="str">
         <f>=IFERROR(ROUND(0,2),0)</f>
       </c>
-      <c r="E56" s="202" t="str">
+      <c r="E56" s="201" t="str">
         <f>=ROUND(IFERROR($C$56-$D$56,0),2)</f>
       </c>
       <c r="F56" s="258" t="str">
         <f>=ROUND(IFERROR(($C$56/$D$56)-1,0),4)</f>
       </c>
-      <c r="G56" s="218" t="str">
+      <c r="G56" s="217" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"Zinsertraege",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="H56" s="218" t="str">
+      <c r="H56" s="217" t="str">
         <f>=IFERROR(ROUND(0,2),0)</f>
       </c>
       <c r="I56" s="182" t="str">
@@ -22439,22 +22457,22 @@
       <c r="B62" s="266" t="s">
         <v>205</v>
       </c>
-      <c r="C62" s="240" t="str">
+      <c r="C62" s="239" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"Bauausgaben",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="D62" s="240" t="str">
+      <c r="D62" s="239" t="str">
         <f>=IFERROR(ROUND(Kosten_Bauausgaben_LW,2),0)</f>
       </c>
-      <c r="E62" s="202" t="str">
+      <c r="E62" s="201" t="str">
         <f>=ROUND(IFERROR($C$62-$D$62,0),2)</f>
       </c>
       <c r="F62" s="258" t="str">
         <f>=ROUND(IFERROR(($C$62/$D$62)-1,0),4)</f>
       </c>
-      <c r="G62" s="218" t="str">
+      <c r="G62" s="217" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"Bauausgaben",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="H62" s="218" t="str">
+      <c r="H62" s="217" t="str">
         <f>=IFERROR(ROUND(Kosten_Bauausgaben_EUR,2),0)</f>
       </c>
       <c r="I62" s="182" t="str">
@@ -22468,22 +22486,22 @@
       <c r="B63" s="266" t="s">
         <v>210</v>
       </c>
-      <c r="C63" s="240" t="str">
+      <c r="C63" s="239" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"Investitionen",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="D63" s="240" t="str">
+      <c r="D63" s="239" t="str">
         <f>=IFERROR(ROUND(Kosten_Investitionen_LW,2),0)</f>
       </c>
-      <c r="E63" s="202" t="str">
+      <c r="E63" s="201" t="str">
         <f>=ROUND(IFERROR($C$63-$D$63,0),2)</f>
       </c>
       <c r="F63" s="258" t="str">
         <f>=ROUND(IFERROR(($C$63/$D$63)-1,0),4)</f>
       </c>
-      <c r="G63" s="218" t="str">
+      <c r="G63" s="217" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"Investitionen",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="H63" s="218" t="str">
+      <c r="H63" s="217" t="str">
         <f>=IFERROR(ROUND(Kosten_Investitionen_EUR,2),0)</f>
       </c>
       <c r="I63" s="182" t="str">
@@ -22497,22 +22515,22 @@
       <c r="B64" s="266" t="s">
         <v>213</v>
       </c>
-      <c r="C64" s="240" t="str">
+      <c r="C64" s="239" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"Personalkosten",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="D64" s="240" t="str">
+      <c r="D64" s="239" t="str">
         <f>=IFERROR(ROUND(Kosten_Personalkosten_LW,2),0)</f>
       </c>
-      <c r="E64" s="202" t="str">
+      <c r="E64" s="201" t="str">
         <f>=ROUND(IFERROR($C$64-$D$64,0),2)</f>
       </c>
       <c r="F64" s="258" t="str">
         <f>=ROUND(IFERROR(($C$64/$D$64)-1,0),4)</f>
       </c>
-      <c r="G64" s="218" t="str">
+      <c r="G64" s="217" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"Personalkosten",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="H64" s="218" t="str">
+      <c r="H64" s="217" t="str">
         <f>=IFERROR(ROUND(Kosten_Personalkosten_EUR,2),0)</f>
       </c>
       <c r="I64" s="182" t="str">
@@ -22526,22 +22544,22 @@
       <c r="B65" s="266" t="s">
         <v>218</v>
       </c>
-      <c r="C65" s="240" t="str">
+      <c r="C65" s="239" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"Projektaktivitaeten",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="D65" s="240" t="str">
+      <c r="D65" s="239" t="str">
         <f>=IFERROR(ROUND(Kosten_Projektaktivitaeten_LW,2),0)</f>
       </c>
-      <c r="E65" s="202" t="str">
+      <c r="E65" s="201" t="str">
         <f>=ROUND(IFERROR($C$65-$D$65,0),2)</f>
       </c>
       <c r="F65" s="258" t="str">
         <f>=ROUND(IFERROR(($C$65/$D$65)-1,0),4)</f>
       </c>
-      <c r="G65" s="218" t="str">
+      <c r="G65" s="217" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"Projektaktivitaeten",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="H65" s="218" t="str">
+      <c r="H65" s="217" t="str">
         <f>=IFERROR(ROUND(Kosten_Projektaktivitaeten_EUR,2),0)</f>
       </c>
       <c r="I65" s="182" t="str">
@@ -22555,22 +22573,22 @@
       <c r="B66" s="266" t="s">
         <v>221</v>
       </c>
-      <c r="C66" s="240" t="str">
+      <c r="C66" s="239" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"Projektverwaltung",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="D66" s="240" t="str">
+      <c r="D66" s="239" t="str">
         <f>=IFERROR(ROUND(Kosten_Projektverwaltung_LW,2),0)</f>
       </c>
-      <c r="E66" s="202" t="str">
+      <c r="E66" s="201" t="str">
         <f>=ROUND(IFERROR($C$66-$D$66,0),2)</f>
       </c>
       <c r="F66" s="258" t="str">
         <f>=ROUND(IFERROR(($C$66/$D$66)-1,0),4)</f>
       </c>
-      <c r="G66" s="218" t="str">
+      <c r="G66" s="217" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"Projektverwaltung",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="H66" s="218" t="str">
+      <c r="H66" s="217" t="str">
         <f>=IFERROR(ROUND(Kosten_Projektverwaltung_EUR,2),0)</f>
       </c>
       <c r="I66" s="182" t="str">
@@ -22584,22 +22602,22 @@
       <c r="B67" s="266" t="s">
         <v>224</v>
       </c>
-      <c r="C67" s="240" t="str">
+      <c r="C67" s="239" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"Evaluierung",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="D67" s="240" t="str">
+      <c r="D67" s="239" t="str">
         <f>=IFERROR(ROUND(Kosten_Evaluierung_LW,2),0)</f>
       </c>
-      <c r="E67" s="202" t="str">
+      <c r="E67" s="201" t="str">
         <f>=ROUND(IFERROR($C$67-$D$67,0),2)</f>
       </c>
       <c r="F67" s="258" t="str">
         <f>=ROUND(IFERROR(($C$67/$D$67)-1,0),4)</f>
       </c>
-      <c r="G67" s="218" t="str">
+      <c r="G67" s="217" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"Evaluierung",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="H67" s="218" t="str">
+      <c r="H67" s="217" t="str">
         <f>=IFERROR(ROUND(Kosten_Evaluierung_EUR,2),0)</f>
       </c>
       <c r="I67" s="182" t="str">
@@ -22613,22 +22631,22 @@
       <c r="B68" s="266" t="s">
         <v>227</v>
       </c>
-      <c r="C68" s="240" t="str">
+      <c r="C68" s="239" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"Audit",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="D68" s="240" t="str">
+      <c r="D68" s="239" t="str">
         <f>=IFERROR(ROUND(Kosten_Audit_LW,2),0)</f>
       </c>
-      <c r="E68" s="202" t="str">
+      <c r="E68" s="201" t="str">
         <f>=ROUND(IFERROR($C$68-$D$68,0),2)</f>
       </c>
       <c r="F68" s="258" t="str">
         <f>=ROUND(IFERROR(($C$68/$D$68)-1,0),4)</f>
       </c>
-      <c r="G68" s="218" t="str">
+      <c r="G68" s="217" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"Audit",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="H68" s="218" t="str">
+      <c r="H68" s="217" t="str">
         <f>=IFERROR(ROUND(Kosten_Audit_EUR,2),0)</f>
       </c>
       <c r="I68" s="182" t="str">
@@ -22642,22 +22660,22 @@
       <c r="B69" s="266" t="s">
         <v>230</v>
       </c>
-      <c r="C69" s="240" t="str">
+      <c r="C69" s="239" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BU$1:$BU$198,'Daten'!$BT$1:$BT$198,"Reserve",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="D69" s="240" t="str">
+      <c r="D69" s="239" t="str">
         <f>=IFERROR(ROUND(Kosten_Reserve_LW,2),0)</f>
       </c>
-      <c r="E69" s="202" t="str">
+      <c r="E69" s="201" t="str">
         <f>=ROUND(IFERROR($C$69-$D$69,0),2)</f>
       </c>
       <c r="F69" s="258" t="str">
         <f>=ROUND(IFERROR(($C$69/$D$69)-1,0),4)</f>
       </c>
-      <c r="G69" s="218" t="str">
+      <c r="G69" s="217" t="str">
         <f>=IFERROR(ROUND(SUMIFS('Daten'!$BV$1:$BV$198,'Daten'!$BT$1:$BT$198,"Reserve",'Daten'!$BR$1:$BR$198,E10,'Daten'!$BS$1:$BS$198,"&lt;="&amp;E11,'Daten'!$BS$1:$BS$198,"&gt;=1"),2),0)</f>
       </c>
-      <c r="H69" s="218" t="str">
+      <c r="H69" s="217" t="str">
         <f>=IFERROR(ROUND(Kosten_Reserve_EUR,2),0)</f>
       </c>
       <c r="I69" s="182" t="str">
@@ -22697,37 +22715,37 @@
       </c>
     </row>
     <row r="76" ht="22" customHeight="true">
-      <c r="B76" s="195" t="s">
+      <c r="B76" s="194" t="s">
         <v>388</v>
       </c>
-      <c r="C76" s="195"/>
-      <c r="D76" s="195"/>
-      <c r="E76" s="195"/>
-      <c r="F76" s="195"/>
-      <c r="G76" s="195"/>
-      <c r="H76" s="195"/>
-      <c r="I76" s="195"/>
-      <c r="J76" s="195"/>
-      <c r="L76" s="203" t="str">
+      <c r="C76" s="194"/>
+      <c r="D76" s="194"/>
+      <c r="E76" s="194"/>
+      <c r="F76" s="194"/>
+      <c r="G76" s="194"/>
+      <c r="H76" s="194"/>
+      <c r="I76" s="194"/>
+      <c r="J76" s="194"/>
+      <c r="L76" s="202" t="str">
         <f>=IF(E81=0,"Aktueller Finanzbericht (keiner gewählt)","Aktueller Finanzbericht – Periode "&amp;E81)</f>
       </c>
-      <c r="M76" s="204"/>
-      <c r="N76" s="204"/>
-      <c r="O76" s="204"/>
-      <c r="P76" s="205"/>
+      <c r="M76" s="203"/>
+      <c r="N76" s="203"/>
+      <c r="O76" s="203"/>
+      <c r="P76" s="204"/>
     </row>
     <row r="77">
-      <c r="B77" s="196" t="s">
+      <c r="B77" s="195" t="s">
         <v>389</v>
       </c>
-      <c r="C77" s="196"/>
-      <c r="D77" s="196"/>
-      <c r="E77" s="196"/>
-      <c r="F77" s="196"/>
-      <c r="G77" s="196"/>
-      <c r="H77" s="196"/>
-      <c r="I77" s="196"/>
-      <c r="J77" s="196"/>
+      <c r="C77" s="195"/>
+      <c r="D77" s="195"/>
+      <c r="E77" s="195"/>
+      <c r="F77" s="195"/>
+      <c r="G77" s="195"/>
+      <c r="H77" s="195"/>
+      <c r="I77" s="195"/>
+      <c r="J77" s="195"/>
       <c r="L77" s="315" t="s">
         <v>288</v>
       </c>
@@ -22750,13 +22768,13 @@
       <c r="P78" s="338"/>
     </row>
     <row r="79" ht="22" customHeight="true">
-      <c r="C79" s="203" t="s">
+      <c r="C79" s="202" t="s">
         <v>390</v>
       </c>
-      <c r="D79" s="204"/>
-      <c r="E79" s="204"/>
-      <c r="F79" s="204"/>
-      <c r="G79" s="205"/>
+      <c r="D79" s="203"/>
+      <c r="E79" s="203"/>
+      <c r="F79" s="203"/>
+      <c r="G79" s="204"/>
       <c r="L79" s="315" t="s">
         <v>290</v>
       </c>
@@ -22768,15 +22786,15 @@
       <c r="P79" s="338"/>
     </row>
     <row r="80">
-      <c r="C80" s="206" t="s">
+      <c r="C80" s="205" t="s">
         <v>342</v>
       </c>
-      <c r="D80" s="198"/>
+      <c r="D80" s="197"/>
       <c r="E80" s="63" t="s">
         <v>391</v>
       </c>
       <c r="F80" s="63"/>
-      <c r="G80" s="207"/>
+      <c r="G80" s="206"/>
       <c r="L80" s="315" t="s">
         <v>291</v>
       </c>
@@ -22849,19 +22867,19 @@
       </c>
     </row>
     <row r="85">
-      <c r="B85" s="224" t="s">
+      <c r="B85" s="223" t="s">
         <v>348</v>
       </c>
-      <c r="C85" s="225"/>
-      <c r="D85" s="226" t="str">
+      <c r="C85" s="224"/>
+      <c r="D85" s="225" t="str">
         <f>=IFERROR(ROUND(KMW_Mittel_EUR,2),0)</f>
       </c>
-      <c r="F85" s="231" t="s">
+      <c r="F85" s="230" t="s">
         <v>352</v>
       </c>
-      <c r="G85" s="232"/>
-      <c r="H85" s="232"/>
-      <c r="I85" s="233"/>
+      <c r="G85" s="231"/>
+      <c r="H85" s="231"/>
+      <c r="I85" s="232"/>
       <c r="L85" s="143" t="str">
         <f>=IFERROR(CHOOSE(E81,'III. Finanzberichte'!$B$11,'III. Finanzberichte'!$I$11,'III. Finanzberichte'!$P$11,'III. Finanzberichte'!$W$11,'III. Finanzberichte'!$AD$11,'III. Finanzberichte'!$AK$11,'III. Finanzberichte'!$AR$11,'III. Finanzberichte'!$AY$11,'III. Finanzberichte'!$BF$11,'III. Finanzberichte'!$BM$11,'III. Finanzberichte'!$BT$11,'III. Finanzberichte'!$CA$11,'III. Finanzberichte'!$CH$11,'III. Finanzberichte'!$CO$11,'III. Finanzberichte'!$CV$11,'III. Finanzberichte'!$DC$11,'III. Finanzberichte'!$DJ$11,'III. Finanzberichte'!$DQ$11),"")</f>
       </c>
@@ -22879,21 +22897,21 @@
       </c>
     </row>
     <row r="86">
-      <c r="B86" s="206" t="s">
+      <c r="B86" s="205" t="s">
         <v>349</v>
       </c>
-      <c r="C86" s="198"/>
-      <c r="D86" s="227" t="str">
+      <c r="C86" s="197"/>
+      <c r="D86" s="226" t="str">
         <f>=IFERROR(ROUND(Kosten_Reserve_EUR,2),0)</f>
       </c>
-      <c r="F86" s="234" t="s">
+      <c r="F86" s="233" t="s">
         <v>353</v>
       </c>
-      <c r="G86" s="198" t="s">
+      <c r="G86" s="197" t="s">
         <v>354</v>
       </c>
-      <c r="H86" s="198"/>
-      <c r="I86" s="235" t="str">
+      <c r="H86" s="197"/>
+      <c r="I86" s="234" t="str">
         <f>=IFERROR(ROUND(Saldovortrag_EUR,2),0)</f>
       </c>
       <c r="L86" s="143" t="s">
@@ -22913,21 +22931,21 @@
       </c>
     </row>
     <row r="87">
-      <c r="B87" s="206" t="str">
+      <c r="B87" s="205" t="str">
         <f>=IF(Reserve_Freigabe="Ja","Operatives Budget (Reserve freigegeben)","Operatives Budget (abzgl. Reserve)")</f>
       </c>
-      <c r="C87" s="198"/>
-      <c r="D87" s="227" t="str">
+      <c r="C87" s="197"/>
+      <c r="D87" s="226" t="str">
         <f>=IF(Reserve_Freigabe="Ja",ROUND($D$85,2),ROUND($D$85-$D$86,2))</f>
       </c>
-      <c r="F87" s="234" t="s">
+      <c r="F87" s="233" t="s">
         <v>353</v>
       </c>
-      <c r="G87" s="198" t="s">
+      <c r="G87" s="197" t="s">
         <v>355</v>
       </c>
-      <c r="H87" s="198"/>
-      <c r="I87" s="235" t="str">
+      <c r="H87" s="197"/>
+      <c r="I87" s="234" t="str">
         <f>=IFERROR(ROUND(MAX(0,(SUM($G$96:$G$99)-$G$98)-(SUM($H$96:$H$99)-$H$98)),2),0)</f>
         <v>0</v>
       </c>
@@ -22948,19 +22966,19 @@
       </c>
     </row>
     <row r="88">
-      <c r="B88" s="206" t="s">
+      <c r="B88" s="205" t="s">
         <v>350</v>
       </c>
-      <c r="C88" s="198"/>
-      <c r="D88" s="227" t="str">
+      <c r="C88" s="197"/>
+      <c r="D88" s="226" t="str">
         <f>=IFERROR(ROUND(SUBTOTAL(109,TblKMWMittel[Betrag]),2),0)</f>
       </c>
       <c r="F88" s="47"/>
-      <c r="G88" s="219" t="s">
+      <c r="G88" s="218" t="s">
         <v>357</v>
       </c>
-      <c r="H88" s="219"/>
-      <c r="I88" s="236" t="str">
+      <c r="H88" s="218"/>
+      <c r="I88" s="235" t="str">
         <f>=ROUND(IF($F$86="Abzug",MAX(0,$I$86),0)+IF($F$87="Abzug",MAX(0,$I$87),0),2)</f>
       </c>
       <c r="L88" s="143" t="s">
@@ -22980,19 +22998,19 @@
       </c>
     </row>
     <row r="89">
-      <c r="B89" s="228" t="s">
+      <c r="B89" s="227" t="s">
         <v>351</v>
       </c>
-      <c r="C89" s="229"/>
-      <c r="D89" s="230" t="str">
+      <c r="C89" s="228"/>
+      <c r="D89" s="229" t="str">
         <f>=ROUND($D$87-$D$88,2)</f>
       </c>
-      <c r="F89" s="237"/>
-      <c r="G89" s="229" t="s">
+      <c r="F89" s="236"/>
+      <c r="G89" s="228" t="s">
         <v>358</v>
       </c>
-      <c r="H89" s="229"/>
-      <c r="I89" s="230" t="str">
+      <c r="H89" s="228"/>
+      <c r="I89" s="229" t="str">
         <f>=ROUND($D$89-$I$88,2)</f>
       </c>
       <c r="L89" s="143" t="s">
@@ -23147,22 +23165,22 @@
       <c r="B96" s="266" t="s">
         <v>194</v>
       </c>
-      <c r="C96" s="240" t="str">
+      <c r="C96" s="239" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$E$12,'III. Finanzberichte'!$L$12,'III. Finanzberichte'!$S$12,'III. Finanzberichte'!$Z$12,'III. Finanzberichte'!$AG$12,'III. Finanzberichte'!$AN$12,'III. Finanzberichte'!$AU$12,'III. Finanzberichte'!$BB$12,'III. Finanzberichte'!$BI$12,'III. Finanzberichte'!$BP$12,'III. Finanzberichte'!$BW$12,'III. Finanzberichte'!$CD$12,'III. Finanzberichte'!$CK$12,'III. Finanzberichte'!$CR$12,'III. Finanzberichte'!$CY$12,'III. Finanzberichte'!$DF$12,'III. Finanzberichte'!$DM$12,'III. Finanzberichte'!$DT$12),2),0)</f>
       </c>
-      <c r="D96" s="240" t="str">
+      <c r="D96" s="239" t="str">
         <f>=IFERROR(ROUND(Eigenmittel_LW,2),0)</f>
       </c>
-      <c r="E96" s="202" t="str">
+      <c r="E96" s="201" t="str">
         <f>=ROUND(IFERROR($C$96-$D$96,0),2)</f>
       </c>
       <c r="F96" s="258" t="str">
         <f>=ROUND(IFERROR(($C$96/$D$96)-1,0),4)</f>
       </c>
-      <c r="G96" s="218" t="str">
+      <c r="G96" s="217" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$F$12,'III. Finanzberichte'!$M$12,'III. Finanzberichte'!$T$12,'III. Finanzberichte'!$AA$12,'III. Finanzberichte'!$AH$12,'III. Finanzberichte'!$AO$12,'III. Finanzberichte'!$AV$12,'III. Finanzberichte'!$BC$12,'III. Finanzberichte'!$BJ$12,'III. Finanzberichte'!$BQ$12,'III. Finanzberichte'!$BX$12,'III. Finanzberichte'!$CE$12,'III. Finanzberichte'!$CL$12,'III. Finanzberichte'!$CS$12,'III. Finanzberichte'!$CZ$12,'III. Finanzberichte'!$DG$12,'III. Finanzberichte'!$DN$12,'III. Finanzberichte'!$DU$12),2),0)</f>
       </c>
-      <c r="H96" s="218" t="str">
+      <c r="H96" s="217" t="str">
         <f>=IFERROR(ROUND(Eigenmittel_EUR,2),0)</f>
       </c>
       <c r="I96" s="182" t="str">
@@ -23191,22 +23209,22 @@
       <c r="B97" s="266" t="s">
         <v>300</v>
       </c>
-      <c r="C97" s="240" t="str">
+      <c r="C97" s="239" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$E$13,'III. Finanzberichte'!$L$13,'III. Finanzberichte'!$S$13,'III. Finanzberichte'!$Z$13,'III. Finanzberichte'!$AG$13,'III. Finanzberichte'!$AN$13,'III. Finanzberichte'!$AU$13,'III. Finanzberichte'!$BB$13,'III. Finanzberichte'!$BI$13,'III. Finanzberichte'!$BP$13,'III. Finanzberichte'!$BW$13,'III. Finanzberichte'!$CD$13,'III. Finanzberichte'!$CK$13,'III. Finanzberichte'!$CR$13,'III. Finanzberichte'!$CY$13,'III. Finanzberichte'!$DF$13,'III. Finanzberichte'!$DM$13,'III. Finanzberichte'!$DT$13),2),0)</f>
       </c>
-      <c r="D97" s="240" t="str">
+      <c r="D97" s="239" t="str">
         <f>=IFERROR(ROUND(Drittmittel_LW,2),0)</f>
       </c>
-      <c r="E97" s="202" t="str">
+      <c r="E97" s="201" t="str">
         <f>=ROUND(IFERROR($C$97-$D$97,0),2)</f>
       </c>
       <c r="F97" s="258" t="str">
         <f>=ROUND(IFERROR(($C$97/$D$97)-1,0),4)</f>
       </c>
-      <c r="G97" s="218" t="str">
+      <c r="G97" s="217" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$F$13,'III. Finanzberichte'!$M$13,'III. Finanzberichte'!$T$13,'III. Finanzberichte'!$AA$13,'III. Finanzberichte'!$AH$13,'III. Finanzberichte'!$AO$13,'III. Finanzberichte'!$AV$13,'III. Finanzberichte'!$BC$13,'III. Finanzberichte'!$BJ$13,'III. Finanzberichte'!$BQ$13,'III. Finanzberichte'!$BX$13,'III. Finanzberichte'!$CE$13,'III. Finanzberichte'!$CL$13,'III. Finanzberichte'!$CS$13,'III. Finanzberichte'!$CZ$13,'III. Finanzberichte'!$DG$13,'III. Finanzberichte'!$DN$13,'III. Finanzberichte'!$DU$13),2),0)</f>
       </c>
-      <c r="H97" s="218" t="str">
+      <c r="H97" s="217" t="str">
         <f>=IFERROR(ROUND(Drittmittel_EUR,2),0)</f>
       </c>
       <c r="I97" s="182" t="str">
@@ -23235,22 +23253,22 @@
       <c r="B98" s="266" t="s">
         <v>199</v>
       </c>
-      <c r="C98" s="240" t="str">
+      <c r="C98" s="239" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$E$14,'III. Finanzberichte'!$L$14,'III. Finanzberichte'!$S$14,'III. Finanzberichte'!$Z$14,'III. Finanzberichte'!$AG$14,'III. Finanzberichte'!$AN$14,'III. Finanzberichte'!$AU$14,'III. Finanzberichte'!$BB$14,'III. Finanzberichte'!$BI$14,'III. Finanzberichte'!$BP$14,'III. Finanzberichte'!$BW$14,'III. Finanzberichte'!$CD$14,'III. Finanzberichte'!$CK$14,'III. Finanzberichte'!$CR$14,'III. Finanzberichte'!$CY$14,'III. Finanzberichte'!$DF$14,'III. Finanzberichte'!$DM$14,'III. Finanzberichte'!$DT$14),2),0)</f>
       </c>
-      <c r="D98" s="240" t="str">
+      <c r="D98" s="239" t="str">
         <f>=IFERROR(ROUND(KMW_Mittel_LW,2),0)</f>
       </c>
-      <c r="E98" s="202" t="str">
+      <c r="E98" s="201" t="str">
         <f>=ROUND(IFERROR($C$98-$D$98,0),2)</f>
       </c>
       <c r="F98" s="258" t="str">
         <f>=ROUND(IFERROR(($C$98/$D$98)-1,0),4)</f>
       </c>
-      <c r="G98" s="218" t="str">
+      <c r="G98" s="217" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$F$14,'III. Finanzberichte'!$M$14,'III. Finanzberichte'!$T$14,'III. Finanzberichte'!$AA$14,'III. Finanzberichte'!$AH$14,'III. Finanzberichte'!$AO$14,'III. Finanzberichte'!$AV$14,'III. Finanzberichte'!$BC$14,'III. Finanzberichte'!$BJ$14,'III. Finanzberichte'!$BQ$14,'III. Finanzberichte'!$BX$14,'III. Finanzberichte'!$CE$14,'III. Finanzberichte'!$CL$14,'III. Finanzberichte'!$CS$14,'III. Finanzberichte'!$CZ$14,'III. Finanzberichte'!$DG$14,'III. Finanzberichte'!$DN$14,'III. Finanzberichte'!$DU$14),2),0)</f>
       </c>
-      <c r="H98" s="218" t="str">
+      <c r="H98" s="217" t="str">
         <f>=IFERROR(ROUND(KMW_Mittel_EUR,2),0)</f>
       </c>
       <c r="I98" s="182" t="str">
@@ -23279,22 +23297,22 @@
       <c r="B99" s="266" t="s">
         <v>301</v>
       </c>
-      <c r="C99" s="240" t="str">
+      <c r="C99" s="239" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$E$15,'III. Finanzberichte'!$L$15,'III. Finanzberichte'!$S$15,'III. Finanzberichte'!$Z$15,'III. Finanzberichte'!$AG$15,'III. Finanzberichte'!$AN$15,'III. Finanzberichte'!$AU$15,'III. Finanzberichte'!$BB$15,'III. Finanzberichte'!$BI$15,'III. Finanzberichte'!$BP$15,'III. Finanzberichte'!$BW$15,'III. Finanzberichte'!$CD$15,'III. Finanzberichte'!$CK$15,'III. Finanzberichte'!$CR$15,'III. Finanzberichte'!$CY$15,'III. Finanzberichte'!$DF$15,'III. Finanzberichte'!$DM$15,'III. Finanzberichte'!$DT$15),2),0)</f>
       </c>
-      <c r="D99" s="240" t="str">
+      <c r="D99" s="239" t="str">
         <f>=IFERROR(ROUND(0,2),0)</f>
       </c>
-      <c r="E99" s="202" t="str">
+      <c r="E99" s="201" t="str">
         <f>=ROUND(IFERROR($C$99-$D$99,0),2)</f>
       </c>
       <c r="F99" s="258" t="str">
         <f>=ROUND(IFERROR(($C$99/$D$99)-1,0),4)</f>
       </c>
-      <c r="G99" s="218" t="str">
+      <c r="G99" s="217" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$F$15,'III. Finanzberichte'!$M$15,'III. Finanzberichte'!$T$15,'III. Finanzberichte'!$AA$15,'III. Finanzberichte'!$AH$15,'III. Finanzberichte'!$AO$15,'III. Finanzberichte'!$AV$15,'III. Finanzberichte'!$BC$15,'III. Finanzberichte'!$BJ$15,'III. Finanzberichte'!$BQ$15,'III. Finanzberichte'!$BX$15,'III. Finanzberichte'!$CE$15,'III. Finanzberichte'!$CL$15,'III. Finanzberichte'!$CS$15,'III. Finanzberichte'!$CZ$15,'III. Finanzberichte'!$DG$15,'III. Finanzberichte'!$DN$15,'III. Finanzberichte'!$DU$15),2),0)</f>
       </c>
-      <c r="H99" s="218" t="str">
+      <c r="H99" s="217" t="str">
         <f>=IFERROR(ROUND(0,2),0)</f>
       </c>
       <c r="I99" s="182" t="str">
@@ -23460,22 +23478,22 @@
       <c r="B105" s="266" t="s">
         <v>205</v>
       </c>
-      <c r="C105" s="240" t="str">
+      <c r="C105" s="239" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$E$19+'III. Finanzberichte'!$E$20,'III. Finanzberichte'!$L$19+'III. Finanzberichte'!$L$20,'III. Finanzberichte'!$S$19+'III. Finanzberichte'!$S$20,'III. Finanzberichte'!$Z$19+'III. Finanzberichte'!$Z$20,'III. Finanzberichte'!$AG$19+'III. Finanzberichte'!$AG$20,'III. Finanzberichte'!$AN$19+'III. Finanzberichte'!$AN$20,'III. Finanzberichte'!$AU$19+'III. Finanzberichte'!$AU$20,'III. Finanzberichte'!$BB$19+'III. Finanzberichte'!$BB$20,'III. Finanzberichte'!$BI$19+'III. Finanzberichte'!$BI$20,'III. Finanzberichte'!$BP$19+'III. Finanzberichte'!$BP$20,'III. Finanzberichte'!$BW$19+'III. Finanzberichte'!$BW$20,'III. Finanzberichte'!$CD$19+'III. Finanzberichte'!$CD$20,'III. Finanzberichte'!$CK$19+'III. Finanzberichte'!$CK$20,'III. Finanzberichte'!$CR$19+'III. Finanzberichte'!$CR$20,'III. Finanzberichte'!$CY$19+'III. Finanzberichte'!$CY$20,'III. Finanzberichte'!$DF$19+'III. Finanzberichte'!$DF$20,'III. Finanzberichte'!$DM$19+'III. Finanzberichte'!$DM$20,'III. Finanzberichte'!$DT$19+'III. Finanzberichte'!$DT$20),2),0)</f>
       </c>
-      <c r="D105" s="240" t="str">
+      <c r="D105" s="239" t="str">
         <f>=IFERROR(ROUND(Kosten_Bauausgaben_LW,2),0)</f>
       </c>
-      <c r="E105" s="202" t="str">
+      <c r="E105" s="201" t="str">
         <f>=ROUND(IFERROR($C$105-$D$105,0),2)</f>
       </c>
       <c r="F105" s="258" t="str">
         <f>=ROUND(IFERROR(($C$105/$D$105)-1,0),4)</f>
       </c>
-      <c r="G105" s="218" t="str">
+      <c r="G105" s="217" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$F$19+'III. Finanzberichte'!$F$20,'III. Finanzberichte'!$M$19+'III. Finanzberichte'!$M$20,'III. Finanzberichte'!$T$19+'III. Finanzberichte'!$T$20,'III. Finanzberichte'!$AA$19+'III. Finanzberichte'!$AA$20,'III. Finanzberichte'!$AH$19+'III. Finanzberichte'!$AH$20,'III. Finanzberichte'!$AO$19+'III. Finanzberichte'!$AO$20,'III. Finanzberichte'!$AV$19+'III. Finanzberichte'!$AV$20,'III. Finanzberichte'!$BC$19+'III. Finanzberichte'!$BC$20,'III. Finanzberichte'!$BJ$19+'III. Finanzberichte'!$BJ$20,'III. Finanzberichte'!$BQ$19+'III. Finanzberichte'!$BQ$20,'III. Finanzberichte'!$BX$19+'III. Finanzberichte'!$BX$20,'III. Finanzberichte'!$CE$19+'III. Finanzberichte'!$CE$20,'III. Finanzberichte'!$CL$19+'III. Finanzberichte'!$CL$20,'III. Finanzberichte'!$CS$19+'III. Finanzberichte'!$CS$20,'III. Finanzberichte'!$CZ$19+'III. Finanzberichte'!$CZ$20,'III. Finanzberichte'!$DG$19+'III. Finanzberichte'!$DG$20,'III. Finanzberichte'!$DN$19+'III. Finanzberichte'!$DN$20,'III. Finanzberichte'!$DU$19+'III. Finanzberichte'!$DU$20),2),0)</f>
       </c>
-      <c r="H105" s="218" t="str">
+      <c r="H105" s="217" t="str">
         <f>=IFERROR(ROUND(Kosten_Bauausgaben_EUR,2),0)</f>
       </c>
       <c r="I105" s="182" t="str">
@@ -23504,22 +23522,22 @@
       <c r="B106" s="266" t="s">
         <v>210</v>
       </c>
-      <c r="C106" s="240" t="str">
+      <c r="C106" s="239" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$E$21,'III. Finanzberichte'!$L$21,'III. Finanzberichte'!$S$21,'III. Finanzberichte'!$Z$21,'III. Finanzberichte'!$AG$21,'III. Finanzberichte'!$AN$21,'III. Finanzberichte'!$AU$21,'III. Finanzberichte'!$BB$21,'III. Finanzberichte'!$BI$21,'III. Finanzberichte'!$BP$21,'III. Finanzberichte'!$BW$21,'III. Finanzberichte'!$CD$21,'III. Finanzberichte'!$CK$21,'III. Finanzberichte'!$CR$21,'III. Finanzberichte'!$CY$21,'III. Finanzberichte'!$DF$21,'III. Finanzberichte'!$DM$21,'III. Finanzberichte'!$DT$21),2),0)</f>
       </c>
-      <c r="D106" s="240" t="str">
+      <c r="D106" s="239" t="str">
         <f>=IFERROR(ROUND(Kosten_Investitionen_LW,2),0)</f>
       </c>
-      <c r="E106" s="202" t="str">
+      <c r="E106" s="201" t="str">
         <f>=ROUND(IFERROR($C$106-$D$106,0),2)</f>
       </c>
       <c r="F106" s="258" t="str">
         <f>=ROUND(IFERROR(($C$106/$D$106)-1,0),4)</f>
       </c>
-      <c r="G106" s="218" t="str">
+      <c r="G106" s="217" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$F$21,'III. Finanzberichte'!$M$21,'III. Finanzberichte'!$T$21,'III. Finanzberichte'!$AA$21,'III. Finanzberichte'!$AH$21,'III. Finanzberichte'!$AO$21,'III. Finanzberichte'!$AV$21,'III. Finanzberichte'!$BC$21,'III. Finanzberichte'!$BJ$21,'III. Finanzberichte'!$BQ$21,'III. Finanzberichte'!$BX$21,'III. Finanzberichte'!$CE$21,'III. Finanzberichte'!$CL$21,'III. Finanzberichte'!$CS$21,'III. Finanzberichte'!$CZ$21,'III. Finanzberichte'!$DG$21,'III. Finanzberichte'!$DN$21,'III. Finanzberichte'!$DU$21),2),0)</f>
       </c>
-      <c r="H106" s="218" t="str">
+      <c r="H106" s="217" t="str">
         <f>=IFERROR(ROUND(Kosten_Investitionen_EUR,2),0)</f>
       </c>
       <c r="I106" s="182" t="str">
@@ -23533,22 +23551,22 @@
       <c r="B107" s="266" t="s">
         <v>213</v>
       </c>
-      <c r="C107" s="240" t="str">
+      <c r="C107" s="239" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$E$22+'III. Finanzberichte'!$E$23,'III. Finanzberichte'!$L$22+'III. Finanzberichte'!$L$23,'III. Finanzberichte'!$S$22+'III. Finanzberichte'!$S$23,'III. Finanzberichte'!$Z$22+'III. Finanzberichte'!$Z$23,'III. Finanzberichte'!$AG$22+'III. Finanzberichte'!$AG$23,'III. Finanzberichte'!$AN$22+'III. Finanzberichte'!$AN$23,'III. Finanzberichte'!$AU$22+'III. Finanzberichte'!$AU$23,'III. Finanzberichte'!$BB$22+'III. Finanzberichte'!$BB$23,'III. Finanzberichte'!$BI$22+'III. Finanzberichte'!$BI$23,'III. Finanzberichte'!$BP$22+'III. Finanzberichte'!$BP$23,'III. Finanzberichte'!$BW$22+'III. Finanzberichte'!$BW$23,'III. Finanzberichte'!$CD$22+'III. Finanzberichte'!$CD$23,'III. Finanzberichte'!$CK$22+'III. Finanzberichte'!$CK$23,'III. Finanzberichte'!$CR$22+'III. Finanzberichte'!$CR$23,'III. Finanzberichte'!$CY$22+'III. Finanzberichte'!$CY$23,'III. Finanzberichte'!$DF$22+'III. Finanzberichte'!$DF$23,'III. Finanzberichte'!$DM$22+'III. Finanzberichte'!$DM$23,'III. Finanzberichte'!$DT$22+'III. Finanzberichte'!$DT$23),2),0)</f>
       </c>
-      <c r="D107" s="240" t="str">
+      <c r="D107" s="239" t="str">
         <f>=IFERROR(ROUND(Kosten_Personalkosten_LW,2),0)</f>
       </c>
-      <c r="E107" s="202" t="str">
+      <c r="E107" s="201" t="str">
         <f>=ROUND(IFERROR($C$107-$D$107,0),2)</f>
       </c>
       <c r="F107" s="258" t="str">
         <f>=ROUND(IFERROR(($C$107/$D$107)-1,0),4)</f>
       </c>
-      <c r="G107" s="218" t="str">
+      <c r="G107" s="217" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$F$22+'III. Finanzberichte'!$F$23,'III. Finanzberichte'!$M$22+'III. Finanzberichte'!$M$23,'III. Finanzberichte'!$T$22+'III. Finanzberichte'!$T$23,'III. Finanzberichte'!$AA$22+'III. Finanzberichte'!$AA$23,'III. Finanzberichte'!$AH$22+'III. Finanzberichte'!$AH$23,'III. Finanzberichte'!$AO$22+'III. Finanzberichte'!$AO$23,'III. Finanzberichte'!$AV$22+'III. Finanzberichte'!$AV$23,'III. Finanzberichte'!$BC$22+'III. Finanzberichte'!$BC$23,'III. Finanzberichte'!$BJ$22+'III. Finanzberichte'!$BJ$23,'III. Finanzberichte'!$BQ$22+'III. Finanzberichte'!$BQ$23,'III. Finanzberichte'!$BX$22+'III. Finanzberichte'!$BX$23,'III. Finanzberichte'!$CE$22+'III. Finanzberichte'!$CE$23,'III. Finanzberichte'!$CL$22+'III. Finanzberichte'!$CL$23,'III. Finanzberichte'!$CS$22+'III. Finanzberichte'!$CS$23,'III. Finanzberichte'!$CZ$22+'III. Finanzberichte'!$CZ$23,'III. Finanzberichte'!$DG$22+'III. Finanzberichte'!$DG$23,'III. Finanzberichte'!$DN$22+'III. Finanzberichte'!$DN$23,'III. Finanzberichte'!$DU$22+'III. Finanzberichte'!$DU$23),2),0)</f>
       </c>
-      <c r="H107" s="218" t="str">
+      <c r="H107" s="217" t="str">
         <f>=IFERROR(ROUND(Kosten_Personalkosten_EUR,2),0)</f>
       </c>
       <c r="I107" s="182" t="str">
@@ -23562,22 +23580,22 @@
       <c r="B108" s="266" t="s">
         <v>218</v>
       </c>
-      <c r="C108" s="240" t="str">
+      <c r="C108" s="239" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$E$24,'III. Finanzberichte'!$L$24,'III. Finanzberichte'!$S$24,'III. Finanzberichte'!$Z$24,'III. Finanzberichte'!$AG$24,'III. Finanzberichte'!$AN$24,'III. Finanzberichte'!$AU$24,'III. Finanzberichte'!$BB$24,'III. Finanzberichte'!$BI$24,'III. Finanzberichte'!$BP$24,'III. Finanzberichte'!$BW$24,'III. Finanzberichte'!$CD$24,'III. Finanzberichte'!$CK$24,'III. Finanzberichte'!$CR$24,'III. Finanzberichte'!$CY$24,'III. Finanzberichte'!$DF$24,'III. Finanzberichte'!$DM$24,'III. Finanzberichte'!$DT$24),2),0)</f>
       </c>
-      <c r="D108" s="240" t="str">
+      <c r="D108" s="239" t="str">
         <f>=IFERROR(ROUND(Kosten_Projektaktivitaeten_LW,2),0)</f>
       </c>
-      <c r="E108" s="202" t="str">
+      <c r="E108" s="201" t="str">
         <f>=ROUND(IFERROR($C$108-$D$108,0),2)</f>
       </c>
       <c r="F108" s="258" t="str">
         <f>=ROUND(IFERROR(($C$108/$D$108)-1,0),4)</f>
       </c>
-      <c r="G108" s="218" t="str">
+      <c r="G108" s="217" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$F$24,'III. Finanzberichte'!$M$24,'III. Finanzberichte'!$T$24,'III. Finanzberichte'!$AA$24,'III. Finanzberichte'!$AH$24,'III. Finanzberichte'!$AO$24,'III. Finanzberichte'!$AV$24,'III. Finanzberichte'!$BC$24,'III. Finanzberichte'!$BJ$24,'III. Finanzberichte'!$BQ$24,'III. Finanzberichte'!$BX$24,'III. Finanzberichte'!$CE$24,'III. Finanzberichte'!$CL$24,'III. Finanzberichte'!$CS$24,'III. Finanzberichte'!$CZ$24,'III. Finanzberichte'!$DG$24,'III. Finanzberichte'!$DN$24,'III. Finanzberichte'!$DU$24),2),0)</f>
       </c>
-      <c r="H108" s="218" t="str">
+      <c r="H108" s="217" t="str">
         <f>=IFERROR(ROUND(Kosten_Projektaktivitaeten_EUR,2),0)</f>
       </c>
       <c r="I108" s="182" t="str">
@@ -23591,22 +23609,22 @@
       <c r="B109" s="266" t="s">
         <v>221</v>
       </c>
-      <c r="C109" s="240" t="str">
+      <c r="C109" s="239" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$E$25,'III. Finanzberichte'!$L$25,'III. Finanzberichte'!$S$25,'III. Finanzberichte'!$Z$25,'III. Finanzberichte'!$AG$25,'III. Finanzberichte'!$AN$25,'III. Finanzberichte'!$AU$25,'III. Finanzberichte'!$BB$25,'III. Finanzberichte'!$BI$25,'III. Finanzberichte'!$BP$25,'III. Finanzberichte'!$BW$25,'III. Finanzberichte'!$CD$25,'III. Finanzberichte'!$CK$25,'III. Finanzberichte'!$CR$25,'III. Finanzberichte'!$CY$25,'III. Finanzberichte'!$DF$25,'III. Finanzberichte'!$DM$25,'III. Finanzberichte'!$DT$25),2),0)</f>
       </c>
-      <c r="D109" s="240" t="str">
+      <c r="D109" s="239" t="str">
         <f>=IFERROR(ROUND(Kosten_Projektverwaltung_LW,2),0)</f>
       </c>
-      <c r="E109" s="202" t="str">
+      <c r="E109" s="201" t="str">
         <f>=ROUND(IFERROR($C$109-$D$109,0),2)</f>
       </c>
       <c r="F109" s="258" t="str">
         <f>=ROUND(IFERROR(($C$109/$D$109)-1,0),4)</f>
       </c>
-      <c r="G109" s="218" t="str">
+      <c r="G109" s="217" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$F$25,'III. Finanzberichte'!$M$25,'III. Finanzberichte'!$T$25,'III. Finanzberichte'!$AA$25,'III. Finanzberichte'!$AH$25,'III. Finanzberichte'!$AO$25,'III. Finanzberichte'!$AV$25,'III. Finanzberichte'!$BC$25,'III. Finanzberichte'!$BJ$25,'III. Finanzberichte'!$BQ$25,'III. Finanzberichte'!$BX$25,'III. Finanzberichte'!$CE$25,'III. Finanzberichte'!$CL$25,'III. Finanzberichte'!$CS$25,'III. Finanzberichte'!$CZ$25,'III. Finanzberichte'!$DG$25,'III. Finanzberichte'!$DN$25,'III. Finanzberichte'!$DU$25),2),0)</f>
       </c>
-      <c r="H109" s="218" t="str">
+      <c r="H109" s="217" t="str">
         <f>=IFERROR(ROUND(Kosten_Projektverwaltung_EUR,2),0)</f>
       </c>
       <c r="I109" s="182" t="str">
@@ -23620,22 +23638,22 @@
       <c r="B110" s="266" t="s">
         <v>224</v>
       </c>
-      <c r="C110" s="240" t="str">
+      <c r="C110" s="239" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$E$26,'III. Finanzberichte'!$L$26,'III. Finanzberichte'!$S$26,'III. Finanzberichte'!$Z$26,'III. Finanzberichte'!$AG$26,'III. Finanzberichte'!$AN$26,'III. Finanzberichte'!$AU$26,'III. Finanzberichte'!$BB$26,'III. Finanzberichte'!$BI$26,'III. Finanzberichte'!$BP$26,'III. Finanzberichte'!$BW$26,'III. Finanzberichte'!$CD$26,'III. Finanzberichte'!$CK$26,'III. Finanzberichte'!$CR$26,'III. Finanzberichte'!$CY$26,'III. Finanzberichte'!$DF$26,'III. Finanzberichte'!$DM$26,'III. Finanzberichte'!$DT$26),2),0)</f>
       </c>
-      <c r="D110" s="240" t="str">
+      <c r="D110" s="239" t="str">
         <f>=IFERROR(ROUND(Kosten_Evaluierung_LW,2),0)</f>
       </c>
-      <c r="E110" s="202" t="str">
+      <c r="E110" s="201" t="str">
         <f>=ROUND(IFERROR($C$110-$D$110,0),2)</f>
       </c>
       <c r="F110" s="258" t="str">
         <f>=ROUND(IFERROR(($C$110/$D$110)-1,0),4)</f>
       </c>
-      <c r="G110" s="218" t="str">
+      <c r="G110" s="217" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$F$26,'III. Finanzberichte'!$M$26,'III. Finanzberichte'!$T$26,'III. Finanzberichte'!$AA$26,'III. Finanzberichte'!$AH$26,'III. Finanzberichte'!$AO$26,'III. Finanzberichte'!$AV$26,'III. Finanzberichte'!$BC$26,'III. Finanzberichte'!$BJ$26,'III. Finanzberichte'!$BQ$26,'III. Finanzberichte'!$BX$26,'III. Finanzberichte'!$CE$26,'III. Finanzberichte'!$CL$26,'III. Finanzberichte'!$CS$26,'III. Finanzberichte'!$CZ$26,'III. Finanzberichte'!$DG$26,'III. Finanzberichte'!$DN$26,'III. Finanzberichte'!$DU$26),2),0)</f>
       </c>
-      <c r="H110" s="218" t="str">
+      <c r="H110" s="217" t="str">
         <f>=IFERROR(ROUND(Kosten_Evaluierung_EUR,2),0)</f>
       </c>
       <c r="I110" s="182" t="str">
@@ -23649,22 +23667,22 @@
       <c r="B111" s="266" t="s">
         <v>227</v>
       </c>
-      <c r="C111" s="240" t="str">
+      <c r="C111" s="239" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$E$27,'III. Finanzberichte'!$L$27,'III. Finanzberichte'!$S$27,'III. Finanzberichte'!$Z$27,'III. Finanzberichte'!$AG$27,'III. Finanzberichte'!$AN$27,'III. Finanzberichte'!$AU$27,'III. Finanzberichte'!$BB$27,'III. Finanzberichte'!$BI$27,'III. Finanzberichte'!$BP$27,'III. Finanzberichte'!$BW$27,'III. Finanzberichte'!$CD$27,'III. Finanzberichte'!$CK$27,'III. Finanzberichte'!$CR$27,'III. Finanzberichte'!$CY$27,'III. Finanzberichte'!$DF$27,'III. Finanzberichte'!$DM$27,'III. Finanzberichte'!$DT$27),2),0)</f>
       </c>
-      <c r="D111" s="240" t="str">
+      <c r="D111" s="239" t="str">
         <f>=IFERROR(ROUND(Kosten_Audit_LW,2),0)</f>
       </c>
-      <c r="E111" s="202" t="str">
+      <c r="E111" s="201" t="str">
         <f>=ROUND(IFERROR($C$111-$D$111,0),2)</f>
       </c>
       <c r="F111" s="258" t="str">
         <f>=ROUND(IFERROR(($C$111/$D$111)-1,0),4)</f>
       </c>
-      <c r="G111" s="218" t="str">
+      <c r="G111" s="217" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$F$27,'III. Finanzberichte'!$M$27,'III. Finanzberichte'!$T$27,'III. Finanzberichte'!$AA$27,'III. Finanzberichte'!$AH$27,'III. Finanzberichte'!$AO$27,'III. Finanzberichte'!$AV$27,'III. Finanzberichte'!$BC$27,'III. Finanzberichte'!$BJ$27,'III. Finanzberichte'!$BQ$27,'III. Finanzberichte'!$BX$27,'III. Finanzberichte'!$CE$27,'III. Finanzberichte'!$CL$27,'III. Finanzberichte'!$CS$27,'III. Finanzberichte'!$CZ$27,'III. Finanzberichte'!$DG$27,'III. Finanzberichte'!$DN$27,'III. Finanzberichte'!$DU$27),2),0)</f>
       </c>
-      <c r="H111" s="218" t="str">
+      <c r="H111" s="217" t="str">
         <f>=IFERROR(ROUND(Kosten_Audit_EUR,2),0)</f>
       </c>
       <c r="I111" s="182" t="str">
@@ -23678,22 +23696,22 @@
       <c r="B112" s="266" t="s">
         <v>230</v>
       </c>
-      <c r="C112" s="240" t="str">
+      <c r="C112" s="239" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$E$28,'III. Finanzberichte'!$L$28,'III. Finanzberichte'!$S$28,'III. Finanzberichte'!$Z$28,'III. Finanzberichte'!$AG$28,'III. Finanzberichte'!$AN$28,'III. Finanzberichte'!$AU$28,'III. Finanzberichte'!$BB$28,'III. Finanzberichte'!$BI$28,'III. Finanzberichte'!$BP$28,'III. Finanzberichte'!$BW$28,'III. Finanzberichte'!$CD$28,'III. Finanzberichte'!$CK$28,'III. Finanzberichte'!$CR$28,'III. Finanzberichte'!$CY$28,'III. Finanzberichte'!$DF$28,'III. Finanzberichte'!$DM$28,'III. Finanzberichte'!$DT$28),2),0)</f>
       </c>
-      <c r="D112" s="240" t="str">
+      <c r="D112" s="239" t="str">
         <f>=IFERROR(ROUND(Kosten_Reserve_LW,2),0)</f>
       </c>
-      <c r="E112" s="202" t="str">
+      <c r="E112" s="201" t="str">
         <f>=ROUND(IFERROR($C$112-$D$112,0),2)</f>
       </c>
       <c r="F112" s="258" t="str">
         <f>=ROUND(IFERROR(($C$112/$D$112)-1,0),4)</f>
       </c>
-      <c r="G112" s="218" t="str">
+      <c r="G112" s="217" t="str">
         <f>=IFERROR(ROUND(CHOOSE(E81,'III. Finanzberichte'!$F$28,'III. Finanzberichte'!$M$28,'III. Finanzberichte'!$T$28,'III. Finanzberichte'!$AA$28,'III. Finanzberichte'!$AH$28,'III. Finanzberichte'!$AO$28,'III. Finanzberichte'!$AV$28,'III. Finanzberichte'!$BC$28,'III. Finanzberichte'!$BJ$28,'III. Finanzberichte'!$BQ$28,'III. Finanzberichte'!$BX$28,'III. Finanzberichte'!$CE$28,'III. Finanzberichte'!$CL$28,'III. Finanzberichte'!$CS$28,'III. Finanzberichte'!$CZ$28,'III. Finanzberichte'!$DG$28,'III. Finanzberichte'!$DN$28,'III. Finanzberichte'!$DU$28),2),0)</f>
       </c>
-      <c r="H112" s="218" t="str">
+      <c r="H112" s="217" t="str">
         <f>=IFERROR(ROUND(Kosten_Reserve_EUR,2),0)</f>
       </c>
       <c r="I112" s="182" t="str">

</xml_diff>

<commit_message>
refactor: adjust KMW calculation logic and layout settings
- Update KMW formulas to simplify remaining amount calculation
- Group and hide columns for periods 2–18 in reports
- Adjust column widths in dashboard and reporting tables for improved readability
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_befuellt.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_befuellt.xlsx
@@ -4969,7 +4969,7 @@
   <cols>
     <col customWidth="true" max="1" min="1" width="3"/>
     <col customWidth="true" max="2" min="2" width="32"/>
-    <col customWidth="true" max="3" min="3" width="25"/>
+    <col customWidth="true" max="3" min="3" width="43"/>
     <col customWidth="true" max="4" min="4" width="24"/>
     <col customWidth="true" max="5" min="5" width="35"/>
     <col customWidth="true" hidden="true" max="27" min="27" width="9.140625"/>
@@ -7170,42 +7170,42 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col customWidth="true" max="2" min="2" width="16"/>
-    <col customWidth="true" max="6" min="3" width="18"/>
-    <col customWidth="true" max="9" min="9" width="16"/>
-    <col customWidth="true" max="13" min="10" width="18"/>
-    <col customWidth="true" max="16" min="16" width="16"/>
-    <col customWidth="true" max="20" min="17" width="18"/>
-    <col customWidth="true" max="23" min="23" width="16"/>
-    <col customWidth="true" max="27" min="24" width="18"/>
-    <col customWidth="true" max="30" min="30" width="16"/>
-    <col customWidth="true" max="34" min="31" width="18"/>
-    <col customWidth="true" max="37" min="37" width="16"/>
-    <col customWidth="true" max="41" min="38" width="18"/>
-    <col customWidth="true" max="44" min="44" width="16"/>
-    <col customWidth="true" max="48" min="45" width="18"/>
-    <col customWidth="true" max="51" min="51" width="16"/>
-    <col customWidth="true" max="55" min="52" width="18"/>
-    <col customWidth="true" max="58" min="58" width="16"/>
-    <col customWidth="true" max="62" min="59" width="18"/>
-    <col customWidth="true" max="65" min="65" width="16"/>
-    <col customWidth="true" max="69" min="66" width="18"/>
-    <col customWidth="true" max="72" min="72" width="16"/>
-    <col customWidth="true" max="76" min="73" width="18"/>
-    <col customWidth="true" max="79" min="79" width="16"/>
-    <col customWidth="true" max="83" min="80" width="18"/>
-    <col customWidth="true" max="86" min="86" width="16"/>
-    <col customWidth="true" max="90" min="87" width="18"/>
-    <col customWidth="true" max="93" min="93" width="16"/>
-    <col customWidth="true" max="97" min="94" width="18"/>
-    <col customWidth="true" max="100" min="100" width="16"/>
-    <col customWidth="true" max="104" min="101" width="18"/>
-    <col customWidth="true" max="107" min="107" width="16"/>
-    <col customWidth="true" max="111" min="108" width="18"/>
-    <col customWidth="true" max="114" min="114" width="16"/>
-    <col customWidth="true" max="118" min="115" width="18"/>
-    <col customWidth="true" max="121" min="121" width="16"/>
-    <col customWidth="true" max="125" min="122" width="18"/>
+    <col customWidth="true" max="2" min="2" width="30.43"/>
+    <col customWidth="true" max="6" min="3" width="20.71"/>
+    <col customWidth="true" hidden="true" max="9" min="9" outlineLevel="1" width="30.43"/>
+    <col customWidth="true" hidden="true" max="13" min="10" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="16" min="16" outlineLevel="1" width="30.43"/>
+    <col customWidth="true" hidden="true" max="20" min="17" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="23" min="23" outlineLevel="1" width="30.43"/>
+    <col customWidth="true" hidden="true" max="27" min="24" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="30" min="30" outlineLevel="1" width="30.43"/>
+    <col customWidth="true" hidden="true" max="34" min="31" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="37" min="37" outlineLevel="1" width="30.43"/>
+    <col customWidth="true" hidden="true" max="41" min="38" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="44" min="44" outlineLevel="1" width="30.43"/>
+    <col customWidth="true" hidden="true" max="48" min="45" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="51" min="51" outlineLevel="1" width="30.43"/>
+    <col customWidth="true" hidden="true" max="55" min="52" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="58" min="58" outlineLevel="1" width="30.43"/>
+    <col customWidth="true" hidden="true" max="62" min="59" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="65" min="65" outlineLevel="1" width="30.43"/>
+    <col customWidth="true" hidden="true" max="69" min="66" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="72" min="72" outlineLevel="1" width="30.43"/>
+    <col customWidth="true" hidden="true" max="76" min="73" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="79" min="79" outlineLevel="1" width="30.43"/>
+    <col customWidth="true" hidden="true" max="83" min="80" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="86" min="86" outlineLevel="1" width="30.43"/>
+    <col customWidth="true" hidden="true" max="90" min="87" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="93" min="93" outlineLevel="1" width="30.43"/>
+    <col customWidth="true" hidden="true" max="97" min="94" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="100" min="100" outlineLevel="1" width="30.43"/>
+    <col customWidth="true" hidden="true" max="104" min="101" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="107" min="107" outlineLevel="1" width="30.43"/>
+    <col customWidth="true" hidden="true" max="111" min="108" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="114" min="114" outlineLevel="1" width="30.43"/>
+    <col customWidth="true" hidden="true" max="118" min="115" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="121" min="121" outlineLevel="1" width="30.43"/>
+    <col customWidth="true" hidden="true" max="125" min="122" outlineLevel="1" width="20.71"/>
   </cols>
   <sheetData>
     <row r="3">
@@ -18455,42 +18455,42 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col customWidth="true" max="2" min="2" width="25"/>
-    <col customWidth="true" max="4" min="3" width="18"/>
-    <col customWidth="true" max="6" min="6" width="25"/>
-    <col customWidth="true" max="8" min="7" width="18"/>
-    <col customWidth="true" max="10" min="10" width="25"/>
-    <col customWidth="true" max="12" min="11" width="18"/>
-    <col customWidth="true" max="14" min="14" width="25"/>
-    <col customWidth="true" max="16" min="15" width="18"/>
-    <col customWidth="true" max="18" min="18" width="25"/>
-    <col customWidth="true" max="20" min="19" width="18"/>
-    <col customWidth="true" max="22" min="22" width="25"/>
-    <col customWidth="true" max="24" min="23" width="18"/>
-    <col customWidth="true" max="26" min="26" width="25"/>
-    <col customWidth="true" max="28" min="27" width="18"/>
-    <col customWidth="true" max="30" min="30" width="25"/>
-    <col customWidth="true" max="32" min="31" width="18"/>
-    <col customWidth="true" max="34" min="34" width="25"/>
-    <col customWidth="true" max="36" min="35" width="18"/>
-    <col customWidth="true" max="38" min="38" width="25"/>
-    <col customWidth="true" max="40" min="39" width="18"/>
-    <col customWidth="true" max="42" min="42" width="25"/>
-    <col customWidth="true" max="44" min="43" width="18"/>
-    <col customWidth="true" max="46" min="46" width="25"/>
-    <col customWidth="true" max="48" min="47" width="18"/>
-    <col customWidth="true" max="50" min="50" width="25"/>
-    <col customWidth="true" max="52" min="51" width="18"/>
-    <col customWidth="true" max="54" min="54" width="25"/>
-    <col customWidth="true" max="56" min="55" width="18"/>
-    <col customWidth="true" max="58" min="58" width="25"/>
-    <col customWidth="true" max="60" min="59" width="18"/>
-    <col customWidth="true" max="62" min="62" width="25"/>
-    <col customWidth="true" max="64" min="63" width="18"/>
-    <col customWidth="true" max="66" min="66" width="25"/>
-    <col customWidth="true" max="68" min="67" width="18"/>
-    <col customWidth="true" max="70" min="70" width="25"/>
-    <col customWidth="true" max="72" min="71" width="18"/>
+    <col customWidth="true" max="2" min="2" width="25.14"/>
+    <col customWidth="true" max="4" min="3" width="20.71"/>
+    <col customWidth="true" hidden="true" max="6" min="6" outlineLevel="1" width="25.14"/>
+    <col customWidth="true" hidden="true" max="8" min="7" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="10" min="10" outlineLevel="1" width="25.14"/>
+    <col customWidth="true" hidden="true" max="12" min="11" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="14" min="14" outlineLevel="1" width="25.14"/>
+    <col customWidth="true" hidden="true" max="16" min="15" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="18" min="18" outlineLevel="1" width="25.14"/>
+    <col customWidth="true" hidden="true" max="20" min="19" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="22" min="22" outlineLevel="1" width="25.14"/>
+    <col customWidth="true" hidden="true" max="24" min="23" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="26" min="26" outlineLevel="1" width="25.14"/>
+    <col customWidth="true" hidden="true" max="28" min="27" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="30" min="30" outlineLevel="1" width="25.14"/>
+    <col customWidth="true" hidden="true" max="32" min="31" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="34" min="34" outlineLevel="1" width="25.14"/>
+    <col customWidth="true" hidden="true" max="36" min="35" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="38" min="38" outlineLevel="1" width="25.14"/>
+    <col customWidth="true" hidden="true" max="40" min="39" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="42" min="42" outlineLevel="1" width="25.14"/>
+    <col customWidth="true" hidden="true" max="44" min="43" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="46" min="46" outlineLevel="1" width="25.14"/>
+    <col customWidth="true" hidden="true" max="48" min="47" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="50" min="50" outlineLevel="1" width="25.14"/>
+    <col customWidth="true" hidden="true" max="52" min="51" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="54" min="54" outlineLevel="1" width="25.14"/>
+    <col customWidth="true" hidden="true" max="56" min="55" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="58" min="58" outlineLevel="1" width="25.14"/>
+    <col customWidth="true" hidden="true" max="60" min="59" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="62" min="62" outlineLevel="1" width="25.14"/>
+    <col customWidth="true" hidden="true" max="64" min="63" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="66" min="66" outlineLevel="1" width="25.14"/>
+    <col customWidth="true" hidden="true" max="68" min="67" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="70" min="70" outlineLevel="1" width="25.14"/>
+    <col customWidth="true" hidden="true" max="72" min="71" outlineLevel="1" width="20.71"/>
   </cols>
   <sheetData>
     <row r="3">
@@ -22064,7 +22064,7 @@
       </c>
       <c r="C33" s="228"/>
       <c r="D33" s="229" t="str">
-        <f>=ROUND($D$26-MAX(0,$D$29)-MAX(0,$D$32),2)</f>
+        <f>=ROUND(MAX(0,$D$26-MAX(0,$D$32)),2)</f>
       </c>
       <c r="F33" s="227" t="s">
         <v>361</v>
@@ -22072,7 +22072,7 @@
       <c r="G33" s="228"/>
       <c r="H33" s="228"/>
       <c r="I33" s="229" t="str">
-        <f>=ROUND($I$27-MAX(0,$I$29)-MAX(0,$I$32),2)</f>
+        <f>=ROUND(MAX(0,$I$27-MAX(0,$I$32)),2)</f>
       </c>
     </row>
     <row r="36" ht="22" customHeight="true">

</xml_diff>

<commit_message>
feat: add conditional formatting for disabled deduction fields
Implement visual feedback for value cells when 'Kein Abzug' is selected,
including custom background colors and border styles. Also adjust column
widths for improved layout.
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_befuellt.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_befuellt.xlsx
@@ -3320,7 +3320,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="17">
+  <dxfs count="19">
     <dxf>
       <font>
         <name val="Segoe UI"/>
@@ -3600,6 +3600,44 @@
       <font>
         <name val="Segoe UI"/>
         <family val="2"/>
+        <color rgb="FFA0A0A0"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="#,##0.00&quot; €&quot;"/>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="center"/>
+      <border>
+        <left style="thin">
+          <color rgb="FFD3D3D3"/>
+        </left>
+        <top style="thin">
+          <color rgb="FFD3D3D3"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFD3D3D3"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <color rgb="FF000000"/>
+      </font>
+      <alignment/>
+      <border>
+        <right style="medium">
+          <color rgb="FF808080"/>
+        </right>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Segoe UI"/>
+        <family val="2"/>
         <b val="1"/>
         <color rgb="FF006100"/>
       </font>
@@ -3631,7 +3669,7 @@
         <b val="1"/>
         <color rgb="FF9C0006"/>
       </font>
-      <numFmt numFmtId="165" formatCode="#,##0.00"/>
+      <numFmt numFmtId="166" formatCode="#,##0.00"/>
       <fill>
         <patternFill patternType="solid">
           <bgColor rgb="FFFFC7CE"/>
@@ -3646,7 +3684,7 @@
         <b val="1"/>
         <color rgb="FF9C0006"/>
       </font>
-      <numFmt numFmtId="166" formatCode="#,##0.00&quot; €&quot;"/>
+      <numFmt numFmtId="167" formatCode="#,##0.00&quot; €&quot;"/>
       <fill>
         <patternFill patternType="solid">
           <bgColor rgb="FFFFC7CE"/>
@@ -3661,7 +3699,7 @@
         <b val="1"/>
         <color rgb="FF9C0006"/>
       </font>
-      <numFmt numFmtId="167" formatCode="0.0%"/>
+      <numFmt numFmtId="168" formatCode="0.0%"/>
       <fill>
         <patternFill patternType="solid">
           <bgColor rgb="FFFFC7CE"/>
@@ -3676,7 +3714,7 @@
         <b val="1"/>
         <color rgb="FF9C640C"/>
       </font>
-      <numFmt numFmtId="168" formatCode="0.0%"/>
+      <numFmt numFmtId="169" formatCode="0.0%"/>
       <fill>
         <patternFill patternType="solid">
           <bgColor rgb="FFFCF3CF"/>
@@ -23932,113 +23970,163 @@
       <formula>$C$18&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="I23">
+    <cfRule type="expression" dxfId="11" priority="19">
+      <formula>$F$23="Kein Abzug"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I23">
+    <cfRule type="expression" dxfId="12" priority="20">
+      <formula>$F$23="Kein Abzug"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I24">
+    <cfRule type="expression" dxfId="11" priority="21">
+      <formula>$F$24="Kein Abzug"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I24">
+    <cfRule type="expression" dxfId="12" priority="22">
+      <formula>$F$24="Kein Abzug"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I25">
+    <cfRule type="expression" dxfId="11" priority="23">
+      <formula>$F$25="Kein Abzug"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I25">
+    <cfRule type="expression" dxfId="12" priority="24">
+      <formula>$F$25="Kein Abzug"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="C46">
-    <cfRule type="expression" dxfId="11" priority="19">
+    <cfRule type="expression" dxfId="13" priority="25">
       <formula>$C$46="OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C46">
-    <cfRule type="expression" dxfId="12" priority="20">
+    <cfRule type="expression" dxfId="14" priority="26">
       <formula>$C$46&lt;&gt;"OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E46">
-    <cfRule type="expression" dxfId="11" priority="21">
+    <cfRule type="expression" dxfId="13" priority="27">
       <formula>$E$46="OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E46">
-    <cfRule type="expression" dxfId="12" priority="22">
+    <cfRule type="expression" dxfId="14" priority="28">
       <formula>$E$46&lt;&gt;"OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C47">
-    <cfRule type="expression" dxfId="13" priority="23">
+    <cfRule type="expression" dxfId="15" priority="29">
       <formula>$C$47&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E47">
-    <cfRule type="expression" dxfId="14" priority="24">
+    <cfRule type="expression" dxfId="16" priority="30">
       <formula>$E$47&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F53:F56">
-    <cfRule type="expression" dxfId="15" priority="25">
+    <cfRule type="expression" dxfId="17" priority="31">
       <formula>F53&gt;=0.2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F53:F56">
-    <cfRule type="expression" dxfId="16" priority="26">
+    <cfRule type="expression" dxfId="18" priority="32">
       <formula>AND(F53&gt;=0.1,F53&lt;0.2)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J53:J56">
-    <cfRule type="expression" dxfId="15" priority="27">
+    <cfRule type="expression" dxfId="17" priority="33">
       <formula>J53&gt;=0.2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J53:J56">
-    <cfRule type="expression" dxfId="16" priority="28">
+    <cfRule type="expression" dxfId="18" priority="34">
       <formula>AND(J53&gt;=0.1,J53&lt;0.2)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F62:F69">
-    <cfRule type="expression" dxfId="15" priority="29">
+    <cfRule type="expression" dxfId="17" priority="35">
       <formula>F62&gt;=0.2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F62:F69">
-    <cfRule type="expression" dxfId="16" priority="30">
+    <cfRule type="expression" dxfId="18" priority="36">
       <formula>AND(F62&gt;=0.1,F62&lt;0.2)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J62:J69">
-    <cfRule type="expression" dxfId="15" priority="31">
+    <cfRule type="expression" dxfId="17" priority="37">
       <formula>J62&gt;=0.2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J62:J69">
-    <cfRule type="expression" dxfId="16" priority="32">
+    <cfRule type="expression" dxfId="18" priority="38">
       <formula>AND(J62&gt;=0.1,J62&lt;0.2)</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="I86">
+    <cfRule type="expression" dxfId="11" priority="39">
+      <formula>$F$86="Kein Abzug"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I86">
+    <cfRule type="expression" dxfId="12" priority="40">
+      <formula>$F$86="Kein Abzug"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I87">
+    <cfRule type="expression" dxfId="11" priority="41">
+      <formula>$F$87="Kein Abzug"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I87">
+    <cfRule type="expression" dxfId="12" priority="42">
+      <formula>$F$87="Kein Abzug"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="F96:F99">
-    <cfRule type="expression" dxfId="15" priority="33">
+    <cfRule type="expression" dxfId="17" priority="43">
       <formula>F96&gt;=0.2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F96:F99">
-    <cfRule type="expression" dxfId="16" priority="34">
+    <cfRule type="expression" dxfId="18" priority="44">
       <formula>AND(F96&gt;=0.1,F96&lt;0.2)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J96:J99">
-    <cfRule type="expression" dxfId="15" priority="35">
+    <cfRule type="expression" dxfId="17" priority="45">
       <formula>J96&gt;=0.2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J96:J99">
-    <cfRule type="expression" dxfId="16" priority="36">
+    <cfRule type="expression" dxfId="18" priority="46">
       <formula>AND(J96&gt;=0.1,J96&lt;0.2)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F105:F112">
-    <cfRule type="expression" dxfId="15" priority="37">
+    <cfRule type="expression" dxfId="17" priority="47">
       <formula>F105&gt;=0.2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F105:F112">
-    <cfRule type="expression" dxfId="16" priority="38">
+    <cfRule type="expression" dxfId="18" priority="48">
       <formula>AND(F105&gt;=0.1,F105&lt;0.2)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J105:J112">
-    <cfRule type="expression" dxfId="15" priority="39">
+    <cfRule type="expression" dxfId="17" priority="49">
       <formula>J105&gt;=0.2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J105:J112">
-    <cfRule type="expression" dxfId="16" priority="40">
+    <cfRule type="expression" dxfId="18" priority="50">
       <formula>AND(J105&gt;=0.1,J105&lt;0.2)</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
chore: update vorpruefung output files
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_befuellt.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_befuellt.xlsx
@@ -18493,41 +18493,41 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col customWidth="true" max="2" min="2" width="25.14"/>
+    <col customWidth="true" max="2" min="2" width="32"/>
     <col customWidth="true" max="4" min="3" width="20.71"/>
-    <col customWidth="true" hidden="true" max="6" min="6" outlineLevel="1" width="25.14"/>
+    <col customWidth="true" hidden="true" max="6" min="6" outlineLevel="1" width="32"/>
     <col customWidth="true" hidden="true" max="8" min="7" outlineLevel="1" width="20.71"/>
-    <col customWidth="true" hidden="true" max="10" min="10" outlineLevel="1" width="25.14"/>
+    <col customWidth="true" hidden="true" max="10" min="10" outlineLevel="1" width="32"/>
     <col customWidth="true" hidden="true" max="12" min="11" outlineLevel="1" width="20.71"/>
-    <col customWidth="true" hidden="true" max="14" min="14" outlineLevel="1" width="25.14"/>
+    <col customWidth="true" hidden="true" max="14" min="14" outlineLevel="1" width="32"/>
     <col customWidth="true" hidden="true" max="16" min="15" outlineLevel="1" width="20.71"/>
-    <col customWidth="true" hidden="true" max="18" min="18" outlineLevel="1" width="25.14"/>
+    <col customWidth="true" hidden="true" max="18" min="18" outlineLevel="1" width="32"/>
     <col customWidth="true" hidden="true" max="20" min="19" outlineLevel="1" width="20.71"/>
-    <col customWidth="true" hidden="true" max="22" min="22" outlineLevel="1" width="25.14"/>
+    <col customWidth="true" hidden="true" max="22" min="22" outlineLevel="1" width="32"/>
     <col customWidth="true" hidden="true" max="24" min="23" outlineLevel="1" width="20.71"/>
-    <col customWidth="true" hidden="true" max="26" min="26" outlineLevel="1" width="25.14"/>
+    <col customWidth="true" hidden="true" max="26" min="26" outlineLevel="1" width="32"/>
     <col customWidth="true" hidden="true" max="28" min="27" outlineLevel="1" width="20.71"/>
-    <col customWidth="true" hidden="true" max="30" min="30" outlineLevel="1" width="25.14"/>
+    <col customWidth="true" hidden="true" max="30" min="30" outlineLevel="1" width="32"/>
     <col customWidth="true" hidden="true" max="32" min="31" outlineLevel="1" width="20.71"/>
-    <col customWidth="true" hidden="true" max="34" min="34" outlineLevel="1" width="25.14"/>
+    <col customWidth="true" hidden="true" max="34" min="34" outlineLevel="1" width="32"/>
     <col customWidth="true" hidden="true" max="36" min="35" outlineLevel="1" width="20.71"/>
-    <col customWidth="true" hidden="true" max="38" min="38" outlineLevel="1" width="25.14"/>
+    <col customWidth="true" hidden="true" max="38" min="38" outlineLevel="1" width="32"/>
     <col customWidth="true" hidden="true" max="40" min="39" outlineLevel="1" width="20.71"/>
-    <col customWidth="true" hidden="true" max="42" min="42" outlineLevel="1" width="25.14"/>
+    <col customWidth="true" hidden="true" max="42" min="42" outlineLevel="1" width="32"/>
     <col customWidth="true" hidden="true" max="44" min="43" outlineLevel="1" width="20.71"/>
-    <col customWidth="true" hidden="true" max="46" min="46" outlineLevel="1" width="25.14"/>
+    <col customWidth="true" hidden="true" max="46" min="46" outlineLevel="1" width="32"/>
     <col customWidth="true" hidden="true" max="48" min="47" outlineLevel="1" width="20.71"/>
-    <col customWidth="true" hidden="true" max="50" min="50" outlineLevel="1" width="25.14"/>
+    <col customWidth="true" hidden="true" max="50" min="50" outlineLevel="1" width="32"/>
     <col customWidth="true" hidden="true" max="52" min="51" outlineLevel="1" width="20.71"/>
-    <col customWidth="true" hidden="true" max="54" min="54" outlineLevel="1" width="25.14"/>
+    <col customWidth="true" hidden="true" max="54" min="54" outlineLevel="1" width="32"/>
     <col customWidth="true" hidden="true" max="56" min="55" outlineLevel="1" width="20.71"/>
-    <col customWidth="true" hidden="true" max="58" min="58" outlineLevel="1" width="25.14"/>
+    <col customWidth="true" hidden="true" max="58" min="58" outlineLevel="1" width="32"/>
     <col customWidth="true" hidden="true" max="60" min="59" outlineLevel="1" width="20.71"/>
-    <col customWidth="true" hidden="true" max="62" min="62" outlineLevel="1" width="25.14"/>
+    <col customWidth="true" hidden="true" max="62" min="62" outlineLevel="1" width="32"/>
     <col customWidth="true" hidden="true" max="64" min="63" outlineLevel="1" width="20.71"/>
-    <col customWidth="true" hidden="true" max="66" min="66" outlineLevel="1" width="25.14"/>
+    <col customWidth="true" hidden="true" max="66" min="66" outlineLevel="1" width="32"/>
     <col customWidth="true" hidden="true" max="68" min="67" outlineLevel="1" width="20.71"/>
-    <col customWidth="true" hidden="true" max="70" min="70" outlineLevel="1" width="25.14"/>
+    <col customWidth="true" hidden="true" max="70" min="70" outlineLevel="1" width="32"/>
     <col customWidth="true" hidden="true" max="72" min="71" outlineLevel="1" width="20.71"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
style: adjust column widths for improved layout
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_befuellt.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_befuellt.xlsx
@@ -7209,41 +7209,41 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col customWidth="true" max="2" min="2" width="30.43"/>
-    <col customWidth="true" max="6" min="3" width="20.71"/>
+    <col customWidth="true" max="6" min="3" width="24.71"/>
     <col customWidth="true" hidden="true" max="9" min="9" outlineLevel="1" width="30.43"/>
-    <col customWidth="true" hidden="true" max="13" min="10" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="13" min="10" outlineLevel="1" width="24.71"/>
     <col customWidth="true" hidden="true" max="16" min="16" outlineLevel="1" width="30.43"/>
-    <col customWidth="true" hidden="true" max="20" min="17" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="20" min="17" outlineLevel="1" width="24.71"/>
     <col customWidth="true" hidden="true" max="23" min="23" outlineLevel="1" width="30.43"/>
-    <col customWidth="true" hidden="true" max="27" min="24" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="27" min="24" outlineLevel="1" width="24.71"/>
     <col customWidth="true" hidden="true" max="30" min="30" outlineLevel="1" width="30.43"/>
-    <col customWidth="true" hidden="true" max="34" min="31" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="34" min="31" outlineLevel="1" width="24.71"/>
     <col customWidth="true" hidden="true" max="37" min="37" outlineLevel="1" width="30.43"/>
-    <col customWidth="true" hidden="true" max="41" min="38" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="41" min="38" outlineLevel="1" width="24.71"/>
     <col customWidth="true" hidden="true" max="44" min="44" outlineLevel="1" width="30.43"/>
-    <col customWidth="true" hidden="true" max="48" min="45" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="48" min="45" outlineLevel="1" width="24.71"/>
     <col customWidth="true" hidden="true" max="51" min="51" outlineLevel="1" width="30.43"/>
-    <col customWidth="true" hidden="true" max="55" min="52" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="55" min="52" outlineLevel="1" width="24.71"/>
     <col customWidth="true" hidden="true" max="58" min="58" outlineLevel="1" width="30.43"/>
-    <col customWidth="true" hidden="true" max="62" min="59" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="62" min="59" outlineLevel="1" width="24.71"/>
     <col customWidth="true" hidden="true" max="65" min="65" outlineLevel="1" width="30.43"/>
-    <col customWidth="true" hidden="true" max="69" min="66" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="69" min="66" outlineLevel="1" width="24.71"/>
     <col customWidth="true" hidden="true" max="72" min="72" outlineLevel="1" width="30.43"/>
-    <col customWidth="true" hidden="true" max="76" min="73" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="76" min="73" outlineLevel="1" width="24.71"/>
     <col customWidth="true" hidden="true" max="79" min="79" outlineLevel="1" width="30.43"/>
-    <col customWidth="true" hidden="true" max="83" min="80" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="83" min="80" outlineLevel="1" width="24.71"/>
     <col customWidth="true" hidden="true" max="86" min="86" outlineLevel="1" width="30.43"/>
-    <col customWidth="true" hidden="true" max="90" min="87" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="90" min="87" outlineLevel="1" width="24.71"/>
     <col customWidth="true" hidden="true" max="93" min="93" outlineLevel="1" width="30.43"/>
-    <col customWidth="true" hidden="true" max="97" min="94" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="97" min="94" outlineLevel="1" width="24.71"/>
     <col customWidth="true" hidden="true" max="100" min="100" outlineLevel="1" width="30.43"/>
-    <col customWidth="true" hidden="true" max="104" min="101" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="104" min="101" outlineLevel="1" width="24.71"/>
     <col customWidth="true" hidden="true" max="107" min="107" outlineLevel="1" width="30.43"/>
-    <col customWidth="true" hidden="true" max="111" min="108" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="111" min="108" outlineLevel="1" width="24.71"/>
     <col customWidth="true" hidden="true" max="114" min="114" outlineLevel="1" width="30.43"/>
-    <col customWidth="true" hidden="true" max="118" min="115" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="118" min="115" outlineLevel="1" width="24.71"/>
     <col customWidth="true" hidden="true" max="121" min="121" outlineLevel="1" width="30.43"/>
-    <col customWidth="true" hidden="true" max="125" min="122" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="125" min="122" outlineLevel="1" width="24.71"/>
   </cols>
   <sheetData>
     <row r="3">
@@ -18494,41 +18494,41 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col customWidth="true" max="2" min="2" width="32"/>
-    <col customWidth="true" max="4" min="3" width="20.71"/>
+    <col customWidth="true" max="4" min="3" width="24.71"/>
     <col customWidth="true" hidden="true" max="6" min="6" outlineLevel="1" width="32"/>
-    <col customWidth="true" hidden="true" max="8" min="7" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="8" min="7" outlineLevel="1" width="24.71"/>
     <col customWidth="true" hidden="true" max="10" min="10" outlineLevel="1" width="32"/>
-    <col customWidth="true" hidden="true" max="12" min="11" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="12" min="11" outlineLevel="1" width="24.71"/>
     <col customWidth="true" hidden="true" max="14" min="14" outlineLevel="1" width="32"/>
-    <col customWidth="true" hidden="true" max="16" min="15" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="16" min="15" outlineLevel="1" width="24.71"/>
     <col customWidth="true" hidden="true" max="18" min="18" outlineLevel="1" width="32"/>
-    <col customWidth="true" hidden="true" max="20" min="19" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="20" min="19" outlineLevel="1" width="24.71"/>
     <col customWidth="true" hidden="true" max="22" min="22" outlineLevel="1" width="32"/>
-    <col customWidth="true" hidden="true" max="24" min="23" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="24" min="23" outlineLevel="1" width="24.71"/>
     <col customWidth="true" hidden="true" max="26" min="26" outlineLevel="1" width="32"/>
-    <col customWidth="true" hidden="true" max="28" min="27" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="28" min="27" outlineLevel="1" width="24.71"/>
     <col customWidth="true" hidden="true" max="30" min="30" outlineLevel="1" width="32"/>
-    <col customWidth="true" hidden="true" max="32" min="31" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="32" min="31" outlineLevel="1" width="24.71"/>
     <col customWidth="true" hidden="true" max="34" min="34" outlineLevel="1" width="32"/>
-    <col customWidth="true" hidden="true" max="36" min="35" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="36" min="35" outlineLevel="1" width="24.71"/>
     <col customWidth="true" hidden="true" max="38" min="38" outlineLevel="1" width="32"/>
-    <col customWidth="true" hidden="true" max="40" min="39" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="40" min="39" outlineLevel="1" width="24.71"/>
     <col customWidth="true" hidden="true" max="42" min="42" outlineLevel="1" width="32"/>
-    <col customWidth="true" hidden="true" max="44" min="43" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="44" min="43" outlineLevel="1" width="24.71"/>
     <col customWidth="true" hidden="true" max="46" min="46" outlineLevel="1" width="32"/>
-    <col customWidth="true" hidden="true" max="48" min="47" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="48" min="47" outlineLevel="1" width="24.71"/>
     <col customWidth="true" hidden="true" max="50" min="50" outlineLevel="1" width="32"/>
-    <col customWidth="true" hidden="true" max="52" min="51" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="52" min="51" outlineLevel="1" width="24.71"/>
     <col customWidth="true" hidden="true" max="54" min="54" outlineLevel="1" width="32"/>
-    <col customWidth="true" hidden="true" max="56" min="55" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="56" min="55" outlineLevel="1" width="24.71"/>
     <col customWidth="true" hidden="true" max="58" min="58" outlineLevel="1" width="32"/>
-    <col customWidth="true" hidden="true" max="60" min="59" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="60" min="59" outlineLevel="1" width="24.71"/>
     <col customWidth="true" hidden="true" max="62" min="62" outlineLevel="1" width="32"/>
-    <col customWidth="true" hidden="true" max="64" min="63" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="64" min="63" outlineLevel="1" width="24.71"/>
     <col customWidth="true" hidden="true" max="66" min="66" outlineLevel="1" width="32"/>
-    <col customWidth="true" hidden="true" max="68" min="67" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="68" min="67" outlineLevel="1" width="24.71"/>
     <col customWidth="true" hidden="true" max="70" min="70" outlineLevel="1" width="32"/>
-    <col customWidth="true" hidden="true" max="72" min="71" outlineLevel="1" width="20.71"/>
+    <col customWidth="true" hidden="true" max="72" min="71" outlineLevel="1" width="24.71"/>
   </cols>
   <sheetData>
     <row r="3">

</xml_diff>

<commit_message>
feat: add support for built-in Excel number formats
Introduce NumFmtID to StyleOptions to allow usage of predefined Excel 
number formats (e.g., ID 14 for locale-sensitive dates). Updated 
style generators to prioritize NumFmtID over custom format strings.
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_befuellt.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_befuellt.xlsx
@@ -1389,11 +1389,11 @@
     <numFmt numFmtId="166" formatCode="#,##0.00"/>
     <numFmt numFmtId="167" formatCode="#,##0.00&quot; €&quot;"/>
     <numFmt numFmtId="168" formatCode="@"/>
-    <numFmt numFmtId="169" formatCode="DD.MM.YYYY"/>
-    <numFmt numFmtId="170" formatCode="0&quot; Monate&quot;"/>
-    <numFmt numFmtId="171" formatCode="0.000000"/>
-    <numFmt numFmtId="172" formatCode="0"/>
-    <numFmt numFmtId="173" formatCode="0.0%"/>
+    <numFmt numFmtId="169" formatCode="0&quot; Monate&quot;"/>
+    <numFmt numFmtId="170" formatCode="0.000000"/>
+    <numFmt numFmtId="171" formatCode="0"/>
+    <numFmt numFmtId="172" formatCode="0.0%"/>
+    <numFmt numFmtId="173" formatCode="DD.MM.YYYY"/>
   </numFmts>
   <fonts count="26">
     <font>
@@ -2584,16 +2584,16 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="44" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="3" fillId="5" borderId="44" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="14" fontId="3" fillId="5" borderId="44" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="3" fillId="6" borderId="44" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="169" fontId="3" fillId="6" borderId="44" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="3" fillId="0" borderId="44" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="170" fontId="3" fillId="0" borderId="44" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="6" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
@@ -2752,7 +2752,7 @@
     <xf numFmtId="167" fontId="8" fillId="9" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="171" fontId="8" fillId="9" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="170" fontId="8" fillId="9" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
@@ -2767,7 +2767,7 @@
     <xf numFmtId="167" fontId="3" fillId="5" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="171" fontId="3" fillId="9" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="170" fontId="3" fillId="9" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="9" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
@@ -2782,7 +2782,7 @@
     <xf numFmtId="167" fontId="12" fillId="9" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="171" fontId="12" fillId="9" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="170" fontId="12" fillId="9" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="167" fontId="3" fillId="9" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
@@ -2794,7 +2794,7 @@
     <xf numFmtId="0" fontId="3" fillId="8" borderId="44" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="3" fillId="8" borderId="44" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="169" fontId="3" fillId="8" borderId="44" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="3" fillId="5" borderId="44" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
@@ -2854,7 +2854,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="12" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="171" fontId="12" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="7" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
@@ -2881,10 +2881,10 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="18" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="12" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="171" fontId="12" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="12" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="171" fontId="12" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="7" borderId="17" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
@@ -2983,10 +2983,10 @@
     <xf numFmtId="0" fontId="3" fillId="8" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment/>
     </xf>
-    <xf numFmtId="172" fontId="3" fillId="5" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="171" fontId="3" fillId="5" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="3" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="171" fontId="3" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="12" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
@@ -2995,7 +2995,7 @@
     <xf numFmtId="0" fontId="12" fillId="8" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="3" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="3" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="7" borderId="38" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
@@ -3007,10 +3007,10 @@
     <xf numFmtId="0" fontId="14" fillId="7" borderId="40" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="3" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="171" fontId="3" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="3" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="171" fontId="3" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
@@ -3022,19 +3022,19 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="3" fillId="8" borderId="20" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="3" fillId="8" borderId="20" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="20" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment/>
     </xf>
-    <xf numFmtId="173" fontId="3" fillId="8" borderId="21" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="3" fillId="8" borderId="21" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="11" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center" wrapText="true"/>
     </xf>
-    <xf numFmtId="173" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="11" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
@@ -3043,7 +3043,7 @@
     <xf numFmtId="166" fontId="25" fillId="11" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="25" fillId="11" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="25" fillId="11" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="25" fillId="11" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
@@ -3061,16 +3061,16 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="11" borderId="32" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
@@ -3079,103 +3079,103 @@
     <xf numFmtId="166" fontId="25" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="25" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="25" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="25" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="25" fillId="11" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="25" fillId="11" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="25" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="25" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="25" fillId="11" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="25" fillId="11" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="12" fillId="8" borderId="20" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="171" fontId="12" fillId="8" borderId="20" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="12" fillId="8" borderId="20" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="171" fontId="12" fillId="8" borderId="20" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="12" fillId="8" borderId="21" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="171" fontId="12" fillId="8" borderId="21" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="25" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="25" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="25" fillId="11" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="25" fillId="11" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="25" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="25" fillId="11" borderId="33" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="25" fillId="11" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="172" fontId="25" fillId="11" borderId="34" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
@@ -3184,12 +3184,12 @@
     <xf numFmtId="0" fontId="3" fillId="8" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="173" fontId="3" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="169" fontId="3" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="3" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="3" fillId="8" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3211,12 +3211,12 @@
     <xf numFmtId="0" fontId="3" fillId="8" borderId="18" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="173" fontId="3" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="169" fontId="3" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="3" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="3" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3241,15 +3241,15 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="10" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="173" fontId="3" fillId="6" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="169" fontId="3" fillId="6" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="170" fontId="3" fillId="6" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="3" fillId="6" borderId="10" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="7" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -3274,13 +3274,13 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="18" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="173" fontId="3" fillId="6" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="169" fontId="3" fillId="6" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="170" fontId="3" fillId="6" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="3" fillId="6" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="51" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">

</xml_diff>

<commit_message>
refactor: update Excel formulas to validate number types
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_befuellt.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_befuellt.xlsx
@@ -5129,13 +5129,13 @@
         <v>166</v>
       </c>
       <c r="C9" s="8" t="str">
-        <f>=IF(OR($C$8="",$E$8=""),"",TEXT($C$8,"dd.mm.yyyy")&amp;" - "&amp;TEXT($E$8,"dd.mm.yyyy"))</f>
+        <f>=IF(AND(ISNUMBER($C$8),ISNUMBER($E$8)),TEXT($C$8,"DD.MM.YYYY")&amp;" - "&amp;TEXT($E$8,"DD.MM.YYYY"),"")</f>
       </c>
       <c r="D9" s="4" t="s">
         <v>167</v>
       </c>
       <c r="E9" s="8" t="str">
-        <f>=IF(OR($C$8="",$E$8=""),"",DATEDIF($C$8,$E$8+1,"M"))</f>
+        <f>=IF(AND(ISNUMBER($C$8),ISNUMBER($E$8)),DATEDIF($C$8,$E$8+1,"M"),"")</f>
       </c>
       <c r="AA9" s="3" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
refactor: reorder financial report and monitoring lists
Adjust the `VSTACK` logic for FB and MA selection lists to place the
static options at the end of the arrays, ensuring chronological
consistency in the UI dropdowns.
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/vorpruefung_befuellt.xlsx
+++ b/sidecars/Vorpruefung/vorpruefung_befuellt.xlsx
@@ -24240,11 +24240,11 @@
         <f>=IF(BK1=1,"Periode "&amp;BJ1,"")</f>
       </c>
       <c r="BN1" cm="1" s="3">
-        <f t="array" ref="BN1">_xlfn.VSTACK("Neuste MA",_xlfn._xlws.FILTER($BE$1:$BE$18,($BB$1:$BB$18='V. AUSWERTUNG'!E81+1)*($BC$1:$BC$18=1),""))</f>
+        <f t="array" ref="BN1">_xlfn.VSTACK(_xlfn._xlws.FILTER($BE$1:$BE$18,($BB$1:$BB$18='V. AUSWERTUNG'!E81+1)*($BC$1:$BC$18=1),""),"Neuste MA")</f>
         <v>0</v>
       </c>
       <c r="BP1" cm="1" s="3">
-        <f t="array" ref="BP1">_xlfn.VSTACK("Neuester FB","Kein Finanzbericht (Projektbeginn)",_xlfn._xlws.FILTER($BL$1:$BL$18,$BK$1:$BK$18=1,""))</f>
+        <f t="array" ref="BP1">_xlfn.VSTACK("Kein Finanzbericht (Projektbeginn)",_xlfn._xlws.FILTER($BL$1:$BL$18,$BK$1:$BK$18=1,""),"Neuester FB")</f>
         <v>0</v>
       </c>
       <c r="BR1" t="str">

</xml_diff>